<commit_message>
Daily pulse data: 2026-04-20
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pulse Metrics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pulse Metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -63,10 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -518,6 +521,73 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Parse error</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Parse error</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Error: Locator.wait_for: Timeout 8000ms exceede</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Error: Locator.wait_for: Timeout 8000ms exceede</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Parse error</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Parse error</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Parse error</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Parse error</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Error: Locator.wait_for: Timeout 8000ms exceede</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Error: Locator.wait_for: Timeout 8000ms exceede</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Error: Locator.wait_for: Timeout 8000ms exceede</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Error: Locator.wait_for: Timeout 8000ms exceede</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-21
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -786,6 +786,163 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>24033643056.711117</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>648599094.697389</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>74650</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>642097352.468117</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>17717924874.871532</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>446839</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>10819</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>55364</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>274597</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>1244624</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>8717.298333516575</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>80215.6836678233</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>327518.33333787293</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>1073775.6989464809</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>93337958.64999992</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>300114863.86999995</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>1153654394.45</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>3292263028.7249994</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>954</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>3124</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>11968</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>33703</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>5981882.010000001</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>86314024.47516748</t>
+        </is>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>363708148.54860574</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>984227086.4317671</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>5156</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>47823</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr">
+        <is>
+          <t>189811</t>
+        </is>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>536966</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-22
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -943,6 +943,163 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>24076657199.418854</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>636857385.526881</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>74744</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>634924381.395854</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>17754937979.087486</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>447555</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>6682</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>58646</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>282253</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>1247447</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>5488.200666739153</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>85978.04466782589</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>344167.15967132</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>1071646.8332494558</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>49100411.06000002</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>294155449.15999985</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>1246995477.4299998</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>3315887248.464999</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>535</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>3011</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>12922</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>33942</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>2379395.6000000006</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>83670832.88516752</t>
+        </is>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>370820112.14860576</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>978818917.6517671</t>
+        </is>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>371</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>47578</t>
+        </is>
+      </c>
+      <c r="AD4" s="2" t="inlineStr">
+        <is>
+          <t>189806</t>
+        </is>
+      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>542865</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-23
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1100,6 +1100,163 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>24118263992.156555</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>614391336.6474568</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>74832</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>613156927.5535548</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>17805567986.457146</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>448330</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>4296</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>58815</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>282680</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>1246273</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>3416.59000004223</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>82813.33733445077</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>348005.350671354</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>1066419.0462160152</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>64734616.54000004</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>289054402.1099999</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>1296168322.35</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>3331162849.8249993</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>608</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>3024</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>13455</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>34145</t>
+        </is>
+      </c>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>748890.2700000003</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="inlineStr">
+        <is>
+          <t>85926503.04516752</t>
+        </is>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>375214046.6786058</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>976832888.6017672</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="AC5" s="2" t="inlineStr">
+        <is>
+          <t>46577</t>
+        </is>
+      </c>
+      <c r="AD5" s="2" t="inlineStr">
+        <is>
+          <t>189971</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>549533</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-24
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1257,6 +1257,163 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>24155326443.214474</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>604560105.2189887</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>74951</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>603247536.3114727</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>17830272971.948826</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>449054</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>4404</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>60860</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>285449</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>1241403</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>3292.67000004369</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>85330.88766776172</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>346322.0816712878</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>1052937.5233465564</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>49740210.230000004</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>305050622.11</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>1267899555.53</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>3355040688.7249994</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>546</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>3098</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>13088</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>34320</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>632428.5800000001</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>92182912.33000003</t>
+        </is>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>384510724.5986059</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>978963789.4917672</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="AC6" s="2" t="inlineStr">
+        <is>
+          <t>46797</t>
+        </is>
+      </c>
+      <c r="AD6" s="2" t="inlineStr">
+        <is>
+          <t>190815</t>
+        </is>
+      </c>
+      <c r="AE6" s="2" t="inlineStr">
+        <is>
+          <t>557098</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-25
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1414,6 +1414,163 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>24192180213.51774</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>595462796.2008193</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>75029</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>595380680.8547399</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>17876600537.386475</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>449724</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2867</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>67318</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>288338</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>1247241</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>2243.87000003326</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>88579.5543344148</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>335535.9723379041</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>1055788.7055224562</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>47743274.370000035</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>303652051.71999997</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>1262438482.36</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>3357856202.9149995</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>537</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>3118</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>13075</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>34392</t>
+        </is>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>616221.9200000002</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr">
+        <is>
+          <t>89744192.58999996</t>
+        </is>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>384800742.9986058</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>982791714.9317671</t>
+        </is>
+      </c>
+      <c r="AB7" s="2" t="inlineStr">
+        <is>
+          <t>168</t>
+        </is>
+      </c>
+      <c r="AC7" s="2" t="inlineStr">
+        <is>
+          <t>46310</t>
+        </is>
+      </c>
+      <c r="AD7" s="2" t="inlineStr">
+        <is>
+          <t>192474</t>
+        </is>
+      </c>
+      <c r="AE7" s="2" t="inlineStr">
+        <is>
+          <t>564889</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-26
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1571,6 +1571,163 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>24185460166.251564</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>595586902.615598</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>75119</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>595479576.328565</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>17869309106.595963</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>449725</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>1011</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>71452</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>286007</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>1238496</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>200.86666666983</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>89908.12066773704</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>328392.406337856</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>1056781.4620888657</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>305193931.75</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>1262120729.55</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>3405621840.5449996</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>3189</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>13122</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>34929</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>810467.0399999999</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>87529948.49999996</t>
+        </is>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
+          <t>380543899.2086058</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>984677704.251767</t>
+        </is>
+      </c>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="AC8" s="2" t="inlineStr">
+        <is>
+          <t>45707</t>
+        </is>
+      </c>
+      <c r="AD8" s="2" t="inlineStr">
+        <is>
+          <t>191796</t>
+        </is>
+      </c>
+      <c r="AE8" s="2" t="inlineStr">
+        <is>
+          <t>570841</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-27
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1728,6 +1728,163 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>24185033293.0534</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>598807131.1356605</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>75206</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>597905330.7703975</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>17867507006.779152</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>449725</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>1760</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>68919</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>283696</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>1217100</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>981.3700000154</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>91716.16766770786</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>319247.19967109326</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>1028382.8318113035</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>305193931.75</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>1217290017.57</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>3405565685.8249993</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>3189</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>12697</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>34927</t>
+        </is>
+      </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>325006.70000000007</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>89394350.50999996</t>
+        </is>
+      </c>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>376812465.0986059</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>981533834.0217671</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>46684</t>
+        </is>
+      </c>
+      <c r="AD9" s="2" t="inlineStr">
+        <is>
+          <t>191199</t>
+        </is>
+      </c>
+      <c r="AE9" s="2" t="inlineStr">
+        <is>
+          <t>571312</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-28
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1885,6 +1885,163 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>24284108027.49171</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>587161416.9588654</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>75295</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>585641716.0287116</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>17949914004.369225</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>451208</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>7272</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>63847</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>288856</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>1215971</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>5069.768000106276</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>97796.08633442395</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>329577.88000439596</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>1018063.2535654227</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>110659700.62999983</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>305169046.87</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>1178020731.8600001</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>3339849972.2149997</t>
+        </is>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>1141</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>3188</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>12296</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>34256</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>846365.2700000007</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>92240376.91999997</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>385824890.9486059</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>989605731.1717671</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr">
+        <is>
+          <t>192</t>
+        </is>
+      </c>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>46221</t>
+        </is>
+      </c>
+      <c r="AD10" s="2" t="inlineStr">
+        <is>
+          <t>190513</t>
+        </is>
+      </c>
+      <c r="AE10" s="2" t="inlineStr">
+        <is>
+          <t>572291</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-29
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2042,6 +2042,163 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>24339694651.58571</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>588706170.2477925</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>75372</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>587996205.8911095</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>17989352937.774403</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>451981</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>4545</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>67719</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>297171</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>1221655</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>3722.968000074432</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>100748.48666780238</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>349983.5146712406</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>1021040.8503892517</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>55581726.41999996</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>322705087.48999995</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>1288955342.2399998</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>3411954266.5399995</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>569</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>3375</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>13439</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>35037</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>525370.2400000002</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>101349506.41187827</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>403505879.1104842</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>1001374117.5436454</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>174</t>
+        </is>
+      </c>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>47731</t>
+        </is>
+      </c>
+      <c r="AD11" s="2" t="inlineStr">
+        <is>
+          <t>193470</t>
+        </is>
+      </c>
+      <c r="AE11" s="2" t="inlineStr">
+        <is>
+          <t>572876</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-04-30
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2199,6 +2199,163 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>24389091062.899487</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>588182634.6900712</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>75456</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>587409820.6464872</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>18021037461.603493</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>452728</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>4823</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>67533</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>299228</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>1221497</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>3834.14666672157</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>102412.6680011768</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>359616.4126713624</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>1021850.9375893673</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>55898751.13999997</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>328948500.39999986</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>1344360670.4299998</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>3427975684.959999</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>574</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>3409</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>14008</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>35236</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>957120.7500000002</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>104711997.12187818</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>404878326.5904841</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>1011508173.1736454</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>46441</t>
+        </is>
+      </c>
+      <c r="AD12" s="2" t="inlineStr">
+        <is>
+          <t>193063</t>
+        </is>
+      </c>
+      <c r="AE12" s="2" t="inlineStr">
+        <is>
+          <t>572452</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-01
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2356,6 +2356,163 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>24432956430.115635</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>587654527.2139236</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>75555</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>587297413.2418816</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>18056276967.386337</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>453403</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>4521</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>69688</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>306212</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>1228418</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>3935.94666672207</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>107516.53733452514</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>367896.90100473235</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>1021744.8783959332</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>46119929.130000025</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>320053551.0099998</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>1337572442.0099998</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>3448281450.709999</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>531</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>3374</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>13948</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>35416</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>990312.6100000001</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>95399721.09931473</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>392171714.5679207</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>1010951499.551082</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>292</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>45939</t>
+        </is>
+      </c>
+      <c r="AD13" s="2" t="inlineStr">
+        <is>
+          <t>197751</t>
+        </is>
+      </c>
+      <c r="AE13" s="2" t="inlineStr">
+        <is>
+          <t>572721</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-02
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2513,6 +2513,163 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>24426309252.322803</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>584485930.2498038</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>75613</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>584485930.2498038</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>18045584361.05624</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>453405</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>481</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>75006</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>304331</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>1236761</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>108175.54066786422</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>372609.12767149677</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>1028510.8995823022</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>316377802.40999985</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>1353814114.6799998</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>3467862542.1999993</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>3358</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>14172</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>35677</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>100279140.86931483</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>395488970.48792076</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>1010324412.121082</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>47600</t>
+        </is>
+      </c>
+      <c r="AD14" s="2" t="inlineStr">
+        <is>
+          <t>200008</t>
+        </is>
+      </c>
+      <c r="AE14" s="2" t="inlineStr">
+        <is>
+          <t>580130</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-03
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE14"/>
+  <dimension ref="A1:AE15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2670,6 +2670,163 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>24480078298.266872</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>588025555.0038742</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>75664</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>588025555.0038742</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>18093914596.97961</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>454216</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>10233</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>70441</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>294896</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>1228168</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>100686.9706677242</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>357061.36833788437</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>1020945.082309866</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>268599626.4799998</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>1234913405.09</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>3467738709.9099994</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>2820</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>12962</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>35674</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>93688505.38931485</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>374221055.18792075</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>1003571820.211082</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>41648</t>
+        </is>
+      </c>
+      <c r="AD15" s="2" t="inlineStr">
+        <is>
+          <t>191952</t>
+        </is>
+      </c>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
+          <t>573842</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-04
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2827,6 +2827,163 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>24476847891.082577</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>587911283.232907</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>75713</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>587911262.3495771</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>18092916769.331493</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>454216</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>5503</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>70692</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>298278</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>1224523</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>96154.08066764612</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>345039.6850043814</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>1007444.202248346</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>268599626.4799998</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>1182529995.1799998</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>3467611409.649999</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>2820</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>12424</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>35672</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>86556920.31931485</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>359775512.9979207</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>993602199.201082</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>35632</t>
+        </is>
+      </c>
+      <c r="AD16" s="2" t="inlineStr">
+        <is>
+          <t>184520</t>
+        </is>
+      </c>
+      <c r="AE16" s="2" t="inlineStr">
+        <is>
+          <t>567268</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-05
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2984,6 +2984,163 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>24475679737.161198</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>588399642.7181934</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>75788</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>588399637.7181983</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>18068644505.75492</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>454219</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>8934</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>59453</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>300111</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>1215424</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>78951.96866750676</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>340402.78167092265</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>990068.7842683855</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>268585647.0699998</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>1144042579.5099998</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>3390070351.0299993</t>
+        </is>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>2819</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>11989</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>34929</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>69532672.27931486</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>354006330.1879207</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>983969618.3310821</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>29302</t>
+        </is>
+      </c>
+      <c r="AD17" s="2" t="inlineStr">
+        <is>
+          <t>179189</t>
+        </is>
+      </c>
+      <c r="AE17" s="2" t="inlineStr">
+        <is>
+          <t>560883</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-06
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3141,6 +3141,163 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>24658553735.48785</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>607490331.5464963</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>75893</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>605365313.5448483</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>18214172472.93365</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>456567</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>5071</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>69902</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>316244</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>1221399</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>4144.015333399711</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>113300.51107498797</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>395826.6717452663</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>1029858.2006863927</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>58260094.15999995</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>319240831.8399999</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>1305568478.2299998</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>3515158587.669999</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>639</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>3472</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>13783</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>36334</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>1386573.8900000001</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>107389514.43618408</t>
+        </is>
+      </c>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
+          <t>408041954.09666824</t>
+        </is>
+      </c>
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
+          <t>1033891791.9698296</t>
+        </is>
+      </c>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
+      </c>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>49167</t>
+        </is>
+      </c>
+      <c r="AD18" s="2" t="inlineStr">
+        <is>
+          <t>200619</t>
+        </is>
+      </c>
+      <c r="AE18" s="2" t="inlineStr">
+        <is>
+          <t>582930</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-07
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE18"/>
+  <dimension ref="A1:AE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3298,6 +3298,163 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>24712338577.889763</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>601610926.0791327</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>75947</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>600697069.2167627</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>18254806880.86453</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>457483</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>5016</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>67629</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>317289</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>1221627</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>4008.312000062744</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>112197.8050749787</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>403775.6804120276</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>1029065.5567484258</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>64205063.019999966</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>321916069.07999986</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>1363577002.8299997</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>3537076281.459999</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>708</t>
+        </is>
+      </c>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>3541</t>
+        </is>
+      </c>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>14420</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="inlineStr">
+        <is>
+          <t>36607</t>
+        </is>
+      </c>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>1151237.9800000002</t>
+        </is>
+      </c>
+      <c r="Y19" s="2" t="inlineStr">
+        <is>
+          <t>105411249.88618414</t>
+        </is>
+      </c>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
+          <t>409583404.34666824</t>
+        </is>
+      </c>
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
+          <t>1035650072.6698296</t>
+        </is>
+      </c>
+      <c r="AB19" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="AC19" s="2" t="inlineStr">
+        <is>
+          <t>50786</t>
+        </is>
+      </c>
+      <c r="AD19" s="2" t="inlineStr">
+        <is>
+          <t>201484</t>
+        </is>
+      </c>
+      <c r="AE19" s="2" t="inlineStr">
+        <is>
+          <t>583466</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-08
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE19"/>
+  <dimension ref="A1:AE20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3455,6 +3455,163 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>24757935701.577908</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>594602518.1969038</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>76008</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>592921644.3949059</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>18293688515.375053</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>458250</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>3839</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>67120</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>317721</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>1225488</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>2070.19000006026</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>106494.20574164408</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>405650.3370786995</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>1031658.9033108396</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>56580620.09999999</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>330280609.5899999</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>1338618529.3199997</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>3563310478.019999</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>592</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>3676</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>14163</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>36922</t>
+        </is>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>949640.2199999997</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>108373987.46874748</t>
+        </is>
+      </c>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>412436583.3966682</t>
+        </is>
+      </c>
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>1040145199.1298295</t>
+        </is>
+      </c>
+      <c r="AB20" s="2" t="inlineStr">
+        <is>
+          <t>162</t>
+        </is>
+      </c>
+      <c r="AC20" s="2" t="inlineStr">
+        <is>
+          <t>50120</t>
+        </is>
+      </c>
+      <c r="AD20" s="2" t="inlineStr">
+        <is>
+          <t>202244</t>
+        </is>
+      </c>
+      <c r="AE20" s="2" t="inlineStr">
+        <is>
+          <t>583682</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-09
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE20"/>
+  <dimension ref="A1:AE21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3612,6 +3612,163 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>24800303033.526524</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>592189268.6867669</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>76060</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>591606629.3235248</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>18331649743.39641</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>458940</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>2853</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>79391</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>320359</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>1231070</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>1355.3933333777</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>97308.9843348166</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>403606.75707884284</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>1034999.7923049073</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>48492702.320000015</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>340781700.5599998</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>1343385734.2499995</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>3594503326.479999</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>526</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>3735</t>
+        </is>
+      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>14220</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>37229</t>
+        </is>
+      </c>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>613326.4099999999</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr">
+        <is>
+          <t>99655235.24874727</t>
+        </is>
+      </c>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>411543350.19322956</t>
+        </is>
+      </c>
+      <c r="AA21" s="2" t="inlineStr">
+        <is>
+          <t>1048212459.9698294</t>
+        </is>
+      </c>
+      <c r="AB21" s="2" t="inlineStr">
+        <is>
+          <t>193</t>
+        </is>
+      </c>
+      <c r="AC21" s="2" t="inlineStr">
+        <is>
+          <t>47354</t>
+        </is>
+      </c>
+      <c r="AD21" s="2" t="inlineStr">
+        <is>
+          <t>203102</t>
+        </is>
+      </c>
+      <c r="AE21" s="2" t="inlineStr">
+        <is>
+          <t>585264</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-10
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE21"/>
+  <dimension ref="A1:AE22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3769,6 +3769,163 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>24791205643.366314</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>590318749.3393633</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>76099</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>590265187.8733153</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>18330875521.097034</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>458941</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>1431</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>77174</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>317700</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>1230881</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>239.80000003429</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>91762.45407323516</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>396762.48707890924</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>1033425.123590252</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>335071471.0699999</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>1341459493.1699996</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>3642979234.169999</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>3681</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>14234</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>37755</t>
+        </is>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>430581.58999999997</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr">
+        <is>
+          <t>97946855.7587473</t>
+        </is>
+      </c>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>404368561.5132296</t>
+        </is>
+      </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
+          <t>1050337914.7898295</t>
+        </is>
+      </c>
+      <c r="AB22" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="AC22" s="2" t="inlineStr">
+        <is>
+          <t>46277</t>
+        </is>
+      </c>
+      <c r="AD22" s="2" t="inlineStr">
+        <is>
+          <t>202693</t>
+        </is>
+      </c>
+      <c r="AE22" s="2" t="inlineStr">
+        <is>
+          <t>586351</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-11
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE22"/>
+  <dimension ref="A1:AE23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3926,6 +3926,163 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>24789798029.3676</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>594605338.0646629</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>76141</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>592670488.0445989</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>18330314184.498703</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>458942</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>2362</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>76694</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>314601</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>1220754</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>416.10000005577</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>87990.9455152042</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>386962.3304122299</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>1025992.0947478197</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>335128096.73999983</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>1301749605.0999997</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>3642750659.819999</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>3682</t>
+        </is>
+      </c>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>13811</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>37751</t>
+        </is>
+      </c>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>696940.0099999998</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr">
+        <is>
+          <t>98513837.3987473</t>
+        </is>
+      </c>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>398272169.55322963</t>
+        </is>
+      </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>1049185285.0098294</t>
+        </is>
+      </c>
+      <c r="AB23" s="2" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="AC23" s="2" t="inlineStr">
+        <is>
+          <t>46001</t>
+        </is>
+      </c>
+      <c r="AD23" s="2" t="inlineStr">
+        <is>
+          <t>201570</t>
+        </is>
+      </c>
+      <c r="AE23" s="2" t="inlineStr">
+        <is>
+          <t>587123</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-12
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE23"/>
+  <dimension ref="A1:AE24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4083,6 +4083,163 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>24907716502.805717</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>599148368.660305</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>76197</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>597345278.2527161</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>18418926296.767567</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>460458</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>5879</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>62471</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>319870</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>1217450</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>2405.23000009075</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>81120.28566819157</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>390222.88474565034</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>1015720.6856143147</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>111356716.34000005</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>335067521.3699999</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>1263561665.4599996</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>3570109381.7799993</t>
+        </is>
+      </c>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>1226</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>3680</t>
+        </is>
+      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>13404</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>37056</t>
+        </is>
+      </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>973693.48</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="inlineStr">
+        <is>
+          <t>86287379.72999991</t>
+        </is>
+      </c>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>402861651.45322967</t>
+        </is>
+      </c>
+      <c r="AA24" s="2" t="inlineStr">
+        <is>
+          <t>1048954061.9298295</t>
+        </is>
+      </c>
+      <c r="AB24" s="2" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="AC24" s="2" t="inlineStr">
+        <is>
+          <t>45713</t>
+        </is>
+      </c>
+      <c r="AD24" s="2" t="inlineStr">
+        <is>
+          <t>201874</t>
+        </is>
+      </c>
+      <c r="AE24" s="2" t="inlineStr">
+        <is>
+          <t>586848</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-13
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE24"/>
+  <dimension ref="A1:AE25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4240,6 +4240,163 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>24949740240.818726</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>586300377.7016327</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>76233</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>585310564.6657237</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>18468853362.13907</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>461271</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>5159</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>64634</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>326795</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>1219701</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>2461.89000009225</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>74008.09200165486</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>401546.05307928275</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>1013739.4023020259</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>57141587.49999998</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>339223783.03</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>1374884353.7899997</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>3643564876.2799993</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>627</t>
+        </is>
+      </c>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>3701</t>
+        </is>
+      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>14630</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>37889</t>
+        </is>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>1427677.7799999996</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr">
+        <is>
+          <t>84081936.58999987</t>
+        </is>
+      </c>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>408844766.1532297</t>
+        </is>
+      </c>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>1050770003.5598295</t>
+        </is>
+      </c>
+      <c r="AB25" s="2" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
+      <c r="AC25" s="2" t="inlineStr">
+        <is>
+          <t>45768</t>
+        </is>
+      </c>
+      <c r="AD25" s="2" t="inlineStr">
+        <is>
+          <t>202326</t>
+        </is>
+      </c>
+      <c r="AE25" s="2" t="inlineStr">
+        <is>
+          <t>588106</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-14
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE25"/>
+  <dimension ref="A1:AE26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4397,6 +4397,163 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>25007446520.310986</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>582004143.2886906</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>76275</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>580866856.9579855</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>18512447692.268044</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>462180</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>6826</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>64670</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>326033</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>1221219</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>2452.66000010087</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>70309.17666846947</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>402094.37774616375</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>1011867.9684245292</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>66680223.86999996</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>338235250.40000004</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>1432002197.0199997</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>3659888268.0099993</t>
+        </is>
+      </c>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>714</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>3692</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>15259</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>38119</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>1010100.7999999999</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>79577068.7699999</t>
+        </is>
+      </c>
+      <c r="Z26" s="2" t="inlineStr">
+        <is>
+          <t>404400324.50322974</t>
+        </is>
+      </c>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>1053058610.2798295</t>
+        </is>
+      </c>
+      <c r="AB26" s="2" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="AC26" s="2" t="inlineStr">
+        <is>
+          <t>45465</t>
+        </is>
+      </c>
+      <c r="AD26" s="2" t="inlineStr">
+        <is>
+          <t>203082</t>
+        </is>
+      </c>
+      <c r="AE26" s="2" t="inlineStr">
+        <is>
+          <t>588329</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-16
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE26"/>
+  <dimension ref="A1:AE27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4554,6 +4554,163 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>25128471191.7208</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>600939666.6965741</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>76368</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>598982272.4978</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>18577366273.44068</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>463552</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>4349</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>74257</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>331915</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>1237562</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>1765.382666762539</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>81268.36333551748</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>405621.6804132786</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>1027168.3336173126</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>46678113.88999998</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>330912001.27000004</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>1391715284.6099997</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>3706843238.5599995</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>3634</t>
+        </is>
+      </c>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>14911</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>38661</t>
+        </is>
+      </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>847517.7700000004</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>80025736.43000007</t>
+        </is>
+      </c>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>405945874.0032298</t>
+        </is>
+      </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>1065992201.3898295</t>
+        </is>
+      </c>
+      <c r="AB27" s="2" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="AC27" s="2" t="inlineStr">
+        <is>
+          <t>47509</t>
+        </is>
+      </c>
+      <c r="AD27" s="2" t="inlineStr">
+        <is>
+          <t>204756</t>
+        </is>
+      </c>
+      <c r="AE27" s="2" t="inlineStr">
+        <is>
+          <t>591554</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-17
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE27"/>
+  <dimension ref="A1:AE28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4711,6 +4711,163 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>25121982741.72275</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>598904905.1260678</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>76401</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>598848790.5997498</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>18575373001.839596</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>463553</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>1782</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>77924</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>328744</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>1240490</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>312.06666671032</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>81327.0300021771</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>396142.8240799512</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>1025700.3162729698</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>329112300.84</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>1389631503.8199997</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>3753556938.299999</t>
+        </is>
+      </c>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>3626</t>
+        </is>
+      </c>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>14895</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>39180</t>
+        </is>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>385739.48999999993</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>80479734.42000009</t>
+        </is>
+      </c>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>399287423.9080623</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>1067964592.5498295</t>
+        </is>
+      </c>
+      <c r="AB28" s="2" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="AC28" s="2" t="inlineStr">
+        <is>
+          <t>47885</t>
+        </is>
+      </c>
+      <c r="AD28" s="2" t="inlineStr">
+        <is>
+          <t>204458</t>
+        </is>
+      </c>
+      <c r="AE28" s="2" t="inlineStr">
+        <is>
+          <t>591703</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-18
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE28"/>
+  <dimension ref="A1:AE29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4868,6 +4868,163 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>25118350871.093304</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>602402475.8296174</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>76436</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>599022484.2303023</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>18572832497.379574</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>463556</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>3370</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>74291</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>327912</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>1238312</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>458.18000006661</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>81729.22666889861</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>386756.5940799585</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>1019681.2701057581</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>164282.83</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>329134302.13</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>1338515882.6599996</t>
+        </is>
+      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>3753454020.6999993</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>3627</t>
+        </is>
+      </c>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>14370</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="inlineStr">
+        <is>
+          <t>39180</t>
+        </is>
+      </c>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>358256.42999999993</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr">
+        <is>
+          <t>80757277.57000008</t>
+        </is>
+      </c>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>391585681.86806226</t>
+        </is>
+      </c>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>1067235892.7398295</t>
+        </is>
+      </c>
+      <c r="AB29" s="2" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="AC29" s="2" t="inlineStr">
+        <is>
+          <t>48919</t>
+        </is>
+      </c>
+      <c r="AD29" s="2" t="inlineStr">
+        <is>
+          <t>203470</t>
+        </is>
+      </c>
+      <c r="AE29" s="2" t="inlineStr">
+        <is>
+          <t>592982</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-19
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE29"/>
+  <dimension ref="A1:AE30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5025,6 +5025,163 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>25239307102.661736</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>603224186.7875776</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>76497</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>601741161.6476362</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>18665203176.165836</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>465225</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>8577</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>69164</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>334127</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>1233132</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>4148.49666683478</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>82446.01666892643</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>390211.2770800741</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>1017749.4978186702</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>116704652.50000006</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>329216802.34999996</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>1292443869.5899997</t>
+        </is>
+      </c>
+      <c r="S30" s="2" t="inlineStr">
+        <is>
+          <t>3753613253.5299993</t>
+        </is>
+      </c>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>1306</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>3626</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>13904</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>39180</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>734547.5800000001</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>82122257.31000009</t>
+        </is>
+      </c>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>395070585.3480623</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>1071619826.6098295</t>
+        </is>
+      </c>
+      <c r="AB30" s="2" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="AC30" s="2" t="inlineStr">
+        <is>
+          <t>49993</t>
+        </is>
+      </c>
+      <c r="AD30" s="2" t="inlineStr">
+        <is>
+          <t>203811</t>
+        </is>
+      </c>
+      <c r="AE30" s="2" t="inlineStr">
+        <is>
+          <t>593376</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-20
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE30"/>
+  <dimension ref="A1:AE31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5182,6 +5182,163 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>25298864069.564796</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>602874373.6417382</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>76555</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>602359888.3217982</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>18709534520.01433</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>466079</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>5974</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>72662</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>343331</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>1237139</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>2829.09333344254</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>82631.39333562313</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>401966.24408037803</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>1013597.6374488198</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>60149034.85999997</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>334659445.14</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>1409266581.5499997</t>
+        </is>
+      </c>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>3784429396.1399994</t>
+        </is>
+      </c>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>659</t>
+        </is>
+      </c>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>3705</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>15211</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>39637</t>
+        </is>
+      </c>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
+          <t>1255521.7300000002</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>83886674.94000006</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>403855355.7080623</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>1073739777.7598295</t>
+        </is>
+      </c>
+      <c r="AB31" s="2" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="AC31" s="2" t="inlineStr">
+        <is>
+          <t>49002</t>
+        </is>
+      </c>
+      <c r="AD31" s="2" t="inlineStr">
+        <is>
+          <t>204360</t>
+        </is>
+      </c>
+      <c r="AE31" s="2" t="inlineStr">
+        <is>
+          <t>592519</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-21
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE31"/>
+  <dimension ref="A1:AE32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5339,6 +5339,163 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>25357790560.52197</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>599181816.7774217</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>76606</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>598976465.4789687</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>18754853922.588726</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>467005</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>5665</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>71220</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>342371</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>1243610</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>2406.37333346032</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>80540.09000227995</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>402418.78408062045</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>1011019.4965079906</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>64531762.22000005</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>337508812.96999997</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>1469396146.1199996</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>3807054088.9099994</t>
+        </is>
+      </c>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>721</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>3734</t>
+        </is>
+      </c>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>15869</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>39923</t>
+        </is>
+      </c>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>1687637.0500000003</t>
+        </is>
+      </c>
+      <c r="Y32" s="2" t="inlineStr">
+        <is>
+          <t>88064689.20486458</t>
+        </is>
+      </c>
+      <c r="Z32" s="2" t="inlineStr">
+        <is>
+          <t>406150989.23292685</t>
+        </is>
+      </c>
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>1079800643.234694</t>
+        </is>
+      </c>
+      <c r="AB32" s="2" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="AC32" s="2" t="inlineStr">
+        <is>
+          <t>50069</t>
+        </is>
+      </c>
+      <c r="AD32" s="2" t="inlineStr">
+        <is>
+          <t>205328</t>
+        </is>
+      </c>
+      <c r="AE32" s="2" t="inlineStr">
+        <is>
+          <t>594903</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-22
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE32"/>
+  <dimension ref="A1:AE33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5496,6 +5496,163 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>25432577096.45158</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>631487015.4254124</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>76717</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>630888962.3189205</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>18788782031.548374</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>467735</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>4960</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>70997</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>344097</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>1253194</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>2015.72666676237</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>80436.96133560591</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>396383.41408079216</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>1015512.3712700856</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>49106379.16999997</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>335245443.37000006</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>1440605282.2599998</t>
+        </is>
+      </c>
+      <c r="S33" s="2" t="inlineStr">
+        <is>
+          <t>3833138438.2499995</t>
+        </is>
+      </c>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>548</t>
+        </is>
+      </c>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>3742</t>
+        </is>
+      </c>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>15637</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="inlineStr">
+        <is>
+          <t>40259</t>
+        </is>
+      </c>
+      <c r="X33" s="2" t="inlineStr">
+        <is>
+          <t>908963.29</t>
+        </is>
+      </c>
+      <c r="Y33" s="2" t="inlineStr">
+        <is>
+          <t>88507414.56486459</t>
+        </is>
+      </c>
+      <c r="Z33" s="2" t="inlineStr">
+        <is>
+          <t>408215091.5929268</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
+        <is>
+          <t>1083551115.264694</t>
+        </is>
+      </c>
+      <c r="AB33" s="2" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="AC33" s="2" t="inlineStr">
+        <is>
+          <t>49870</t>
+        </is>
+      </c>
+      <c r="AD33" s="2" t="inlineStr">
+        <is>
+          <t>206026</t>
+        </is>
+      </c>
+      <c r="AE33" s="2" t="inlineStr">
+        <is>
+          <t>594954</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-23
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE33"/>
+  <dimension ref="A1:AE34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5653,6 +5653,163 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>25486958849.388367</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>638010975.9061819</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>76761</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>637407136.6353658</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>18827398758.17572</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>468471</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>4166</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>75067</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>342951</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>1262510</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>1893.75666673282</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>68963.41500209786</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>391771.7580809257</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>1023686.2409302808</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>49444145.40000003</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>337664372.92</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>1440325255.4199998</t>
+        </is>
+      </c>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>3827671479.5599995</t>
+        </is>
+      </c>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>526</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>3762</t>
+        </is>
+      </c>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>15649</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="inlineStr">
+        <is>
+          <t>40245</t>
+        </is>
+      </c>
+      <c r="X34" s="2" t="inlineStr">
+        <is>
+          <t>619950.1099999999</t>
+        </is>
+      </c>
+      <c r="Y34" s="2" t="inlineStr">
+        <is>
+          <t>88788766.27486451</t>
+        </is>
+      </c>
+      <c r="Z34" s="2" t="inlineStr">
+        <is>
+          <t>408808137.2329268</t>
+        </is>
+      </c>
+      <c r="AA34" s="2" t="inlineStr">
+        <is>
+          <t>1090837042.744694</t>
+        </is>
+      </c>
+      <c r="AB34" s="2" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
+      </c>
+      <c r="AC34" s="2" t="inlineStr">
+        <is>
+          <t>48848</t>
+        </is>
+      </c>
+      <c r="AD34" s="2" t="inlineStr">
+        <is>
+          <t>207027</t>
+        </is>
+      </c>
+      <c r="AE34" s="2" t="inlineStr">
+        <is>
+          <t>596848</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-24
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE34"/>
+  <dimension ref="A1:AE35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5810,6 +5810,163 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>25485407815.254112</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>644221364.7478875</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>76806</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>644158757.8011105</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>18821898220.92556</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>468475</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>1608</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>77308</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>337902</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>1266250</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>195.42000002224</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>69335.34166874416</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>380147.2780809336</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>1026078.769589557</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>340554173.56000006</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>1425135055.2699997</t>
+        </is>
+      </c>
+      <c r="S35" s="2" t="inlineStr">
+        <is>
+          <t>3877254144.0299993</t>
+        </is>
+      </c>
+      <c r="T35" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>3773</t>
+        </is>
+      </c>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>15570</t>
+        </is>
+      </c>
+      <c r="W35" s="2" t="inlineStr">
+        <is>
+          <t>40774</t>
+        </is>
+      </c>
+      <c r="X35" s="2" t="inlineStr">
+        <is>
+          <t>578313.38</t>
+        </is>
+      </c>
+      <c r="Y35" s="2" t="inlineStr">
+        <is>
+          <t>88906723.42486449</t>
+        </is>
+      </c>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>396011235.0029267</t>
+        </is>
+      </c>
+      <c r="AA35" s="2" t="inlineStr">
+        <is>
+          <t>1093750638.674694</t>
+        </is>
+      </c>
+      <c r="AB35" s="2" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="AC35" s="2" t="inlineStr">
+        <is>
+          <t>49032</t>
+        </is>
+      </c>
+      <c r="AD35" s="2" t="inlineStr">
+        <is>
+          <t>206693</t>
+        </is>
+      </c>
+      <c r="AE35" s="2" t="inlineStr">
+        <is>
+          <t>598001</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-25
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE35"/>
+  <dimension ref="A1:AE36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5967,6 +5967,163 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>25482761620.10392</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>647080061.9157171</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>76851</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>645472800.1109201</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>18819157911.363827</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>468476</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>2817</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>71438</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>334113</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>1263669</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>235.99000003227</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>68953.35500198182</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>367130.39474752557</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>1020084.4466162404</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>340480546.6000001</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>1375344377.5399997</t>
+        </is>
+      </c>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>3876460569.0099993</t>
+        </is>
+      </c>
+      <c r="T36" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>3772</t>
+        </is>
+      </c>
+      <c r="V36" s="2" t="inlineStr">
+        <is>
+          <t>15024</t>
+        </is>
+      </c>
+      <c r="W36" s="2" t="inlineStr">
+        <is>
+          <t>40770</t>
+        </is>
+      </c>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
+          <t>442933.16000000015</t>
+        </is>
+      </c>
+      <c r="Y36" s="2" t="inlineStr">
+        <is>
+          <t>89296676.9948645</t>
+        </is>
+      </c>
+      <c r="Z36" s="2" t="inlineStr">
+        <is>
+          <t>391138166.2729268</t>
+        </is>
+      </c>
+      <c r="AA36" s="2" t="inlineStr">
+        <is>
+          <t>1090315002.934694</t>
+        </is>
+      </c>
+      <c r="AB36" s="2" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="AC36" s="2" t="inlineStr">
+        <is>
+          <t>48556</t>
+        </is>
+      </c>
+      <c r="AD36" s="2" t="inlineStr">
+        <is>
+          <t>205716</t>
+        </is>
+      </c>
+      <c r="AE36" s="2" t="inlineStr">
+        <is>
+          <t>598997</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-26
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE36"/>
+  <dimension ref="A1:AE37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6124,6 +6124,163 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>25484066029.579697</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>649557592.7524322</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>76891</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>648701341.1866962</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>18816641251.57213</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>468476</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>1841</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>59608</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>334020</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>1261056</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>305.91666669363</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>60538.13500181103</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>360841.2914141481</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>1011782.7929076002</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>340316263.7700001</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>1327566201.6099997</t>
+        </is>
+      </c>
+      <c r="S37" s="2" t="inlineStr">
+        <is>
+          <t>3792516539.109999</t>
+        </is>
+      </c>
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>3771</t>
+        </is>
+      </c>
+      <c r="V37" s="2" t="inlineStr">
+        <is>
+          <t>14486</t>
+        </is>
+      </c>
+      <c r="W37" s="2" t="inlineStr">
+        <is>
+          <t>39932</t>
+        </is>
+      </c>
+      <c r="X37" s="2" t="inlineStr">
+        <is>
+          <t>590196.79</t>
+        </is>
+      </c>
+      <c r="Y37" s="2" t="inlineStr">
+        <is>
+          <t>82631036.39819784</t>
+        </is>
+      </c>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>390171673.24626017</t>
+        </is>
+      </c>
+      <c r="AA37" s="2" t="inlineStr">
+        <is>
+          <t>1083354443.9480274</t>
+        </is>
+      </c>
+      <c r="AB37" s="2" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="AC37" s="2" t="inlineStr">
+        <is>
+          <t>47318</t>
+        </is>
+      </c>
+      <c r="AD37" s="2" t="inlineStr">
+        <is>
+          <t>205422</t>
+        </is>
+      </c>
+      <c r="AE37" s="2" t="inlineStr">
+        <is>
+          <t>598083</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-27
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE37"/>
+  <dimension ref="A1:AE38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6281,6 +6281,163 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>25563345890.01489</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>636691953.2916331</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>76927</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>635255624.4318901</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>18890699464.425816</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>469607</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>5526</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>54829</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>333353</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>1241692</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>2549.55333342195</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>58632.65833494627</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>368882.73474761646</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>1013480.6695837781</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>94518903.25999989</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>223503731.25000006</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>1327576381.0499997</t>
+        </is>
+      </c>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>3750746090.689999</t>
+        </is>
+      </c>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>1059</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>2465</t>
+        </is>
+      </c>
+      <c r="V38" s="2" t="inlineStr">
+        <is>
+          <t>14487</t>
+        </is>
+      </c>
+      <c r="W38" s="2" t="inlineStr">
+        <is>
+          <t>39490</t>
+        </is>
+      </c>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>808599.04</t>
+        </is>
+      </c>
+      <c r="Y38" s="2" t="inlineStr">
+        <is>
+          <t>81767320.44819786</t>
+        </is>
+      </c>
+      <c r="Z38" s="2" t="inlineStr">
+        <is>
+          <t>396228325.6462602</t>
+        </is>
+      </c>
+      <c r="AA38" s="2" t="inlineStr">
+        <is>
+          <t>1086107459.8980274</t>
+        </is>
+      </c>
+      <c r="AB38" s="2" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="AC38" s="2" t="inlineStr">
+        <is>
+          <t>48397</t>
+        </is>
+      </c>
+      <c r="AD38" s="2" t="inlineStr">
+        <is>
+          <t>206073</t>
+        </is>
+      </c>
+      <c r="AE38" s="2" t="inlineStr">
+        <is>
+          <t>598772</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-28
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE38"/>
+  <dimension ref="A1:AE39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6438,6 +6438,163 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>25642156638.91362</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>637288348.9954208</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>76965</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>627173599.5106198</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>18964772037.11667</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>471039</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>8630</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>53699</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>330077</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>1248635</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>3049.2366668042</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>60540.14833491966</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>365162.8460811161</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>1018164.5810572585</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>86654052.23999995</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>257974245.4600001</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>1422201344.7099998</t>
+        </is>
+      </c>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>3803642940.9599996</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>931</t>
+        </is>
+      </c>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>2866</t>
+        </is>
+      </c>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>15547</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t>40117</t>
+        </is>
+      </c>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>1543104.81</t>
+        </is>
+      </c>
+      <c r="Y39" s="2" t="inlineStr">
+        <is>
+          <t>77285914.74333331</t>
+        </is>
+      </c>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>391196527.05626017</t>
+        </is>
+      </c>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>1088422549.5080273</t>
+        </is>
+      </c>
+      <c r="AB39" s="2" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="AC39" s="2" t="inlineStr">
+        <is>
+          <t>47912</t>
+        </is>
+      </c>
+      <c r="AD39" s="2" t="inlineStr">
+        <is>
+          <t>207019</t>
+        </is>
+      </c>
+      <c r="AE39" s="2" t="inlineStr">
+        <is>
+          <t>599487</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-29
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE39"/>
+  <dimension ref="A1:AE40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6595,6 +6595,163 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>25699049883.57583</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>625697630.5025531</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>77044</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>625320468.7428291</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>19001577713.424244</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>471928</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>7158</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>58362</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>333780</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>1261177</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>3101.49333344074</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>59986.1173349151</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>355621.04474790493</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>1022132.9065923458</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>61526530.61000003</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>280020591.8000001</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>1397920786.57</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>3846659827.2199993</t>
+        </is>
+      </c>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>643</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>3073</t>
+        </is>
+      </c>
+      <c r="V40" s="2" t="inlineStr">
+        <is>
+          <t>15335</t>
+        </is>
+      </c>
+      <c r="W40" s="2" t="inlineStr">
+        <is>
+          <t>40583</t>
+        </is>
+      </c>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>995820.3000000004</t>
+        </is>
+      </c>
+      <c r="Y40" s="2" t="inlineStr">
+        <is>
+          <t>80686627.95333327</t>
+        </is>
+      </c>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>387552213.13438183</t>
+        </is>
+      </c>
+      <c r="AA40" s="2" t="inlineStr">
+        <is>
+          <t>1094723859.2680273</t>
+        </is>
+      </c>
+      <c r="AB40" s="2" t="inlineStr">
+        <is>
+          <t>292</t>
+        </is>
+      </c>
+      <c r="AC40" s="2" t="inlineStr">
+        <is>
+          <t>49621</t>
+        </is>
+      </c>
+      <c r="AD40" s="2" t="inlineStr">
+        <is>
+          <t>207916</t>
+        </is>
+      </c>
+      <c r="AE40" s="2" t="inlineStr">
+        <is>
+          <t>600894</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-30
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE40"/>
+  <dimension ref="A1:AE41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6752,6 +6752,163 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>25765008690.321186</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>643109055.315113</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>77108</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>641504770.787162</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>19035162297.64739</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>472729</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>4464</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>64543</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>332757</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>1272630</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>1682.05666673335</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>61582.98666824786</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>350942.07674799673</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>1031095.85464737</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>52921746.80999999</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>292438205.7400001</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>1403814960.76</t>
+        </is>
+      </c>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>3875209886.6799994</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>583</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>3167</t>
+        </is>
+      </c>
+      <c r="V41" s="2" t="inlineStr">
+        <is>
+          <t>15407</t>
+        </is>
+      </c>
+      <c r="W41" s="2" t="inlineStr">
+        <is>
+          <t>40906</t>
+        </is>
+      </c>
+      <c r="X41" s="2" t="inlineStr">
+        <is>
+          <t>973955.5000000001</t>
+        </is>
+      </c>
+      <c r="Y41" s="2" t="inlineStr">
+        <is>
+          <t>83384662.68333322</t>
+        </is>
+      </c>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>387480802.79438186</t>
+        </is>
+      </c>
+      <c r="AA41" s="2" t="inlineStr">
+        <is>
+          <t>1103967300.4480274</t>
+        </is>
+      </c>
+      <c r="AB41" s="2" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="AC41" s="2" t="inlineStr">
+        <is>
+          <t>48609</t>
+        </is>
+      </c>
+      <c r="AD41" s="2" t="inlineStr">
+        <is>
+          <t>209195</t>
+        </is>
+      </c>
+      <c r="AE41" s="2" t="inlineStr">
+        <is>
+          <t>599984</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-05-31
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE41"/>
+  <dimension ref="A1:AE42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6909,6 +6909,163 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>25760477610.487717</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>644565058.3478509</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>77175</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>642775432.3847159</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>19030180260.29318</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>472730</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>1950</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>68454</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>327561</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>1274601</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>240.72333336336</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>61763.46333490298</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>334394.2040813115</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>1033531.0916327736</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>295761452.1700001</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>1400842956.43</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>3928085883.4899993</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>3221</t>
+        </is>
+      </c>
+      <c r="V42" s="2" t="inlineStr">
+        <is>
+          <t>15417</t>
+        </is>
+      </c>
+      <c r="W42" s="2" t="inlineStr">
+        <is>
+          <t>41489</t>
+        </is>
+      </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>340700.3300000001</t>
+        </is>
+      </c>
+      <c r="Y42" s="2" t="inlineStr">
+        <is>
+          <t>82280117.20333321</t>
+        </is>
+      </c>
+      <c r="Z42" s="2" t="inlineStr">
+        <is>
+          <t>382891631.1069452</t>
+        </is>
+      </c>
+      <c r="AA42" s="2" t="inlineStr">
+        <is>
+          <t>1096467936.2880273</t>
+        </is>
+      </c>
+      <c r="AB42" s="2" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="AC42" s="2" t="inlineStr">
+        <is>
+          <t>47840</t>
+        </is>
+      </c>
+      <c r="AD42" s="2" t="inlineStr">
+        <is>
+          <t>208594</t>
+        </is>
+      </c>
+      <c r="AE42" s="2" t="inlineStr">
+        <is>
+          <t>590494</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-01
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE42"/>
+  <dimension ref="A1:AE43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7066,6 +7066,163 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>25752626147.07494</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>639912352.0864731</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>77232</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>638442232.4719411</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>19028244642.396255</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>472731</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>2054</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>68543</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>332122</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>1271068</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>587.737333363433</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>62095.704668241975</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>316608.57400762476</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>1027569.3766223233</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>295767697.3600001</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>1354734272.49</t>
+        </is>
+      </c>
+      <c r="S43" s="2" t="inlineStr">
+        <is>
+          <t>3928017146.1999993</t>
+        </is>
+      </c>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
+          <t>3221</t>
+        </is>
+      </c>
+      <c r="V43" s="2" t="inlineStr">
+        <is>
+          <t>14883</t>
+        </is>
+      </c>
+      <c r="W43" s="2" t="inlineStr">
+        <is>
+          <t>41488</t>
+        </is>
+      </c>
+      <c r="X43" s="2" t="inlineStr">
+        <is>
+          <t>268131.86</t>
+        </is>
+      </c>
+      <c r="Y43" s="2" t="inlineStr">
+        <is>
+          <t>77681808.4533332</t>
+        </is>
+      </c>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
+          <t>361589499.52694505</t>
+        </is>
+      </c>
+      <c r="AA43" s="2" t="inlineStr">
+        <is>
+          <t>1088867095.9580274</t>
+        </is>
+      </c>
+      <c r="AB43" s="2" t="inlineStr">
+        <is>
+          <t>193</t>
+        </is>
+      </c>
+      <c r="AC43" s="2" t="inlineStr">
+        <is>
+          <t>42439</t>
+        </is>
+      </c>
+      <c r="AD43" s="2" t="inlineStr">
+        <is>
+          <t>200195</t>
+        </is>
+      </c>
+      <c r="AE43" s="2" t="inlineStr">
+        <is>
+          <t>584548</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-02
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE43"/>
+  <dimension ref="A1:AE44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7223,6 +7223,163 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>25895975268.648098</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>648864916.9064709</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>77287</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>646713071.9050978</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>19134419455.019394</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>474489</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>9562</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>67083</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>329744</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>1271325</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>2437.746000140925</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>69165.52200160755</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>315056.4844126264</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>1023480.5086478398</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>133844969.83999981</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>295794099.5400001</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>1300537045.01</t>
+        </is>
+      </c>
+      <c r="S44" s="2" t="inlineStr">
+        <is>
+          <t>3843573969.5399995</t>
+        </is>
+      </c>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>1400</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>3223</t>
+        </is>
+      </c>
+      <c r="V44" s="2" t="inlineStr">
+        <is>
+          <t>14304</t>
+        </is>
+      </c>
+      <c r="W44" s="2" t="inlineStr">
+        <is>
+          <t>40603</t>
+        </is>
+      </c>
+      <c r="X44" s="2" t="inlineStr">
+        <is>
+          <t>1353941.1599999995</t>
+        </is>
+      </c>
+      <c r="Y44" s="2" t="inlineStr">
+        <is>
+          <t>94865784.77999996</t>
+        </is>
+      </c>
+      <c r="Z44" s="2" t="inlineStr">
+        <is>
+          <t>374859071.6969452</t>
+        </is>
+      </c>
+      <c r="AA44" s="2" t="inlineStr">
+        <is>
+          <t>1100775981.9580274</t>
+        </is>
+      </c>
+      <c r="AB44" s="2" t="inlineStr">
+        <is>
+          <t>296</t>
+        </is>
+      </c>
+      <c r="AC44" s="2" t="inlineStr">
+        <is>
+          <t>45512</t>
+        </is>
+      </c>
+      <c r="AD44" s="2" t="inlineStr">
+        <is>
+          <t>201178</t>
+        </is>
+      </c>
+      <c r="AE44" s="2" t="inlineStr">
+        <is>
+          <t>586478</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-03
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE44"/>
+  <dimension ref="A1:AE45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7380,6 +7380,163 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>25941760138.455315</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>645265932.7340577</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>77367</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>643683581.5523157</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>19178721814.764454</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>475286</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>6928</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>70912</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>341536</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>1281549</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>2967.48000011167</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>69656.59066840798</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>322103.9178548016</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>1027871.2057564639</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>53027896.42999998</t>
+        </is>
+      </c>
+      <c r="Q45" s="2" t="inlineStr">
+        <is>
+          <t>429662982.7799999</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>1434416107.6899998</t>
+        </is>
+      </c>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>3933665665.6999993</t>
+        </is>
+      </c>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>4623</t>
+        </is>
+      </c>
+      <c r="V45" s="2" t="inlineStr">
+        <is>
+          <t>15705</t>
+        </is>
+      </c>
+      <c r="W45" s="2" t="inlineStr">
+        <is>
+          <t>41524</t>
+        </is>
+      </c>
+      <c r="X45" s="2" t="inlineStr">
+        <is>
+          <t>1534934.0699999994</t>
+        </is>
+      </c>
+      <c r="Y45" s="2" t="inlineStr">
+        <is>
+          <t>103591197.57999992</t>
+        </is>
+      </c>
+      <c r="Z45" s="2" t="inlineStr">
+        <is>
+          <t>390971369.4669452</t>
+        </is>
+      </c>
+      <c r="AA45" s="2" t="inlineStr">
+        <is>
+          <t>1112358826.9080274</t>
+        </is>
+      </c>
+      <c r="AB45" s="2" t="inlineStr">
+        <is>
+          <t>252</t>
+        </is>
+      </c>
+      <c r="AC45" s="2" t="inlineStr">
+        <is>
+          <t>46997</t>
+        </is>
+      </c>
+      <c r="AD45" s="2" t="inlineStr">
+        <is>
+          <t>202798</t>
+        </is>
+      </c>
+      <c r="AE45" s="2" t="inlineStr">
+        <is>
+          <t>588996</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-04
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE45"/>
+  <dimension ref="A1:AE46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7537,6 +7537,163 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>25992912519.26332</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>637583020.1716701</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>77415</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>634267468.54032</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>19231563442.644424</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>476269</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>7621</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>66246</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>330124</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>1287192</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>2214.822000133962</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>68039.95833501051</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>318200.95234112506</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>1030730.7634888557</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>67835658.24000004</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>388122305.26999986</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>1487372015.2699997</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="inlineStr">
+        <is>
+          <t>3931531924.809999</t>
+        </is>
+      </c>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>753</t>
+        </is>
+      </c>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>4165</t>
+        </is>
+      </c>
+      <c r="V46" s="2" t="inlineStr">
+        <is>
+          <t>16304</t>
+        </is>
+      </c>
+      <c r="W46" s="2" t="inlineStr">
+        <is>
+          <t>41587</t>
+        </is>
+      </c>
+      <c r="X46" s="2" t="inlineStr">
+        <is>
+          <t>944723.06</t>
+        </is>
+      </c>
+      <c r="Y46" s="2" t="inlineStr">
+        <is>
+          <t>107186591.40000002</t>
+        </is>
+      </c>
+      <c r="Z46" s="2" t="inlineStr">
+        <is>
+          <t>383407951.75819784</t>
+        </is>
+      </c>
+      <c r="AA46" s="2" t="inlineStr">
+        <is>
+          <t>1117142539.7380276</t>
+        </is>
+      </c>
+      <c r="AB46" s="2" t="inlineStr">
+        <is>
+          <t>321</t>
+        </is>
+      </c>
+      <c r="AC46" s="2" t="inlineStr">
+        <is>
+          <t>47003</t>
+        </is>
+      </c>
+      <c r="AD46" s="2" t="inlineStr">
+        <is>
+          <t>203970</t>
+        </is>
+      </c>
+      <c r="AE46" s="2" t="inlineStr">
+        <is>
+          <t>589781</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-05
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE46"/>
+  <dimension ref="A1:AE47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7694,6 +7694,163 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>26032914554.719116</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>634054333.6595922</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>77451</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>624074354.5461161</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>19265774422.214603</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>477055</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>6317</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>65989</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>331117</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>1297232</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>2492.78666678786</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>65357.34466821627</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>307677.8783411332</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>1033373.871083408</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>53882304.28999998</t>
+        </is>
+      </c>
+      <c r="Q47" s="2" t="inlineStr">
+        <is>
+          <t>369339122.6399998</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>1448019077.37</t>
+        </is>
+      </c>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>3949513053.129999</t>
+        </is>
+      </c>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>612</t>
+        </is>
+      </c>
+      <c r="U47" s="2" t="inlineStr">
+        <is>
+          <t>3989</t>
+        </is>
+      </c>
+      <c r="V47" s="2" t="inlineStr">
+        <is>
+          <t>15852</t>
+        </is>
+      </c>
+      <c r="W47" s="2" t="inlineStr">
+        <is>
+          <t>41828</t>
+        </is>
+      </c>
+      <c r="X47" s="2" t="inlineStr">
+        <is>
+          <t>1393437.3399999994</t>
+        </is>
+      </c>
+      <c r="Y47" s="2" t="inlineStr">
+        <is>
+          <t>110552043.13384324</t>
+        </is>
+      </c>
+      <c r="Z47" s="2" t="inlineStr">
+        <is>
+          <t>390714741.83204097</t>
+        </is>
+      </c>
+      <c r="AA47" s="2" t="inlineStr">
+        <is>
+          <t>1126762015.6618707</t>
+        </is>
+      </c>
+      <c r="AB47" s="2" t="inlineStr">
+        <is>
+          <t>253</t>
+        </is>
+      </c>
+      <c r="AC47" s="2" t="inlineStr">
+        <is>
+          <t>45896</t>
+        </is>
+      </c>
+      <c r="AD47" s="2" t="inlineStr">
+        <is>
+          <t>204645</t>
+        </is>
+      </c>
+      <c r="AE47" s="2" t="inlineStr">
+        <is>
+          <t>590573</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-06
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE47"/>
+  <dimension ref="A1:AE48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7851,6 +7851,163 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>26069604511.85625</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>613337554.6753067</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>77482</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>610587172.4232497</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>19305702665.11222</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>477813</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>5712</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>71921</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>332362</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>1308954</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>1873.149000096042</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>62951.52466818763</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>301695.79634120566</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>1041328.2375529293</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>54394425.27999998</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>362184768.7399997</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>1444083660.4199998</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="inlineStr">
+        <is>
+          <t>3968013219.689999</t>
+        </is>
+      </c>
+      <c r="T48" s="2" t="inlineStr">
+        <is>
+          <t>577</t>
+        </is>
+      </c>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>3963</t>
+        </is>
+      </c>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>15829</t>
+        </is>
+      </c>
+      <c r="W48" s="2" t="inlineStr">
+        <is>
+          <t>42068</t>
+        </is>
+      </c>
+      <c r="X48" s="2" t="inlineStr">
+        <is>
+          <t>927388.4799999995</t>
+        </is>
+      </c>
+      <c r="Y48" s="2" t="inlineStr">
+        <is>
+          <t>111515897.63384336</t>
+        </is>
+      </c>
+      <c r="Z48" s="2" t="inlineStr">
+        <is>
+          <t>393585450.54204106</t>
+        </is>
+      </c>
+      <c r="AA48" s="2" t="inlineStr">
+        <is>
+          <t>1138850893.1018708</t>
+        </is>
+      </c>
+      <c r="AB48" s="2" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+      <c r="AC48" s="2" t="inlineStr">
+        <is>
+          <t>47156</t>
+        </is>
+      </c>
+      <c r="AD48" s="2" t="inlineStr">
+        <is>
+          <t>205565</t>
+        </is>
+      </c>
+      <c r="AE48" s="2" t="inlineStr">
+        <is>
+          <t>593079</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-07
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE48"/>
+  <dimension ref="A1:AE49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8008,6 +8008,163 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>26064635530.28651</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>610813152.1439995</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>77508</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>610043761.6535105</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>19301009029.979206</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>477815</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>2363</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>75465</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>328196</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>1312578</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>354.909000052206</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>62457.3863348532</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>290357.3846745206</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>1043729.8789943197</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>363686247.7299997</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>1434248594.57</t>
+        </is>
+      </c>
+      <c r="S49" s="2" t="inlineStr">
+        <is>
+          <t>4022441445.4899993</t>
+        </is>
+      </c>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U49" s="2" t="inlineStr">
+        <is>
+          <t>3957</t>
+        </is>
+      </c>
+      <c r="V49" s="2" t="inlineStr">
+        <is>
+          <t>15698</t>
+        </is>
+      </c>
+      <c r="W49" s="2" t="inlineStr">
+        <is>
+          <t>42646</t>
+        </is>
+      </c>
+      <c r="X49" s="2" t="inlineStr">
+        <is>
+          <t>422781.2099999999</t>
+        </is>
+      </c>
+      <c r="Y49" s="2" t="inlineStr">
+        <is>
+          <t>112598982.9438434</t>
+        </is>
+      </c>
+      <c r="Z49" s="2" t="inlineStr">
+        <is>
+          <t>387116626.58204114</t>
+        </is>
+      </c>
+      <c r="AA49" s="2" t="inlineStr">
+        <is>
+          <t>1141431217.9518707</t>
+        </is>
+      </c>
+      <c r="AB49" s="2" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="AC49" s="2" t="inlineStr">
+        <is>
+          <t>47627</t>
+        </is>
+      </c>
+      <c r="AD49" s="2" t="inlineStr">
+        <is>
+          <t>206101</t>
+        </is>
+      </c>
+      <c r="AE49" s="2" t="inlineStr">
+        <is>
+          <t>594536</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-08
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE49"/>
+  <dimension ref="A1:AE50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8165,6 +8165,163 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>26065340876.50606</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>616283141.4225618</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>77543</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>613990903.6830597</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>19303121242.926334</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>477816</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>2831</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>72556</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>325126</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>1309751</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>320.157000055674</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>62219.337001511354</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>281518.92667431955</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>1038974.086594277</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>363687122.5399997</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>1377639694.4699998</t>
+        </is>
+      </c>
+      <c r="S50" s="2" t="inlineStr">
+        <is>
+          <t>4020655399.8899994</t>
+        </is>
+      </c>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
+          <t>3957</t>
+        </is>
+      </c>
+      <c r="V50" s="2" t="inlineStr">
+        <is>
+          <t>15105</t>
+        </is>
+      </c>
+      <c r="W50" s="2" t="inlineStr">
+        <is>
+          <t>42642</t>
+        </is>
+      </c>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>433803.28999999986</t>
+        </is>
+      </c>
+      <c r="Y50" s="2" t="inlineStr">
+        <is>
+          <t>116630222.16384341</t>
+        </is>
+      </c>
+      <c r="Z50" s="2" t="inlineStr">
+        <is>
+          <t>378564486.44204116</t>
+        </is>
+      </c>
+      <c r="AA50" s="2" t="inlineStr">
+        <is>
+          <t>1138395007.1483018</t>
+        </is>
+      </c>
+      <c r="AB50" s="2" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="AC50" s="2" t="inlineStr">
+        <is>
+          <t>52020</t>
+        </is>
+      </c>
+      <c r="AD50" s="2" t="inlineStr">
+        <is>
+          <t>204861</t>
+        </is>
+      </c>
+      <c r="AE50" s="2" t="inlineStr">
+        <is>
+          <t>594223</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-09
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE50"/>
+  <dimension ref="A1:AE51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8322,6 +8322,163 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>26182379241.1391</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>616634968.955074</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>77575</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>612949417.6260979</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>19393466748.802845</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>479454</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>8848</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>63390</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>328232</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>1310796</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>2867.44200015006</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>65002.616334888895</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>288296.6466742801</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>1041181.1184276728</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>120986688.41</t>
+        </is>
+      </c>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>363874500.76999974</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>1329340074.7099998</t>
+        </is>
+      </c>
+      <c r="S51" s="2" t="inlineStr">
+        <is>
+          <t>3926636236.1399994</t>
+        </is>
+      </c>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
+          <t>1287</t>
+        </is>
+      </c>
+      <c r="U51" s="2" t="inlineStr">
+        <is>
+          <t>3958</t>
+        </is>
+      </c>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>14581</t>
+        </is>
+      </c>
+      <c r="W51" s="2" t="inlineStr">
+        <is>
+          <t>41721</t>
+        </is>
+      </c>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>1429472.3899999997</t>
+        </is>
+      </c>
+      <c r="Y51" s="2" t="inlineStr">
+        <is>
+          <t>115730737.88384323</t>
+        </is>
+      </c>
+      <c r="Z51" s="2" t="inlineStr">
+        <is>
+          <t>392642953.8220411</t>
+        </is>
+      </c>
+      <c r="AA51" s="2" t="inlineStr">
+        <is>
+          <t>1147935030.298302</t>
+        </is>
+      </c>
+      <c r="AB51" s="2" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="AC51" s="2" t="inlineStr">
+        <is>
+          <t>50204</t>
+        </is>
+      </c>
+      <c r="AD51" s="2" t="inlineStr">
+        <is>
+          <t>205105</t>
+        </is>
+      </c>
+      <c r="AE51" s="2" t="inlineStr">
+        <is>
+          <t>594752</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-10
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE51"/>
+  <dimension ref="A1:AE52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8479,6 +8479,163 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>26263332444.04231</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>634559032.9080485</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>77630</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>628977357.1610465</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>19442641106.466984</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>480485</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>6359</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>65588</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>333241</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>1313755</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>2280.54333345886</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>63777.1763348201</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>297890.14867441746</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>1044031.6570945091</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>69447403.96999998</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>350982126.4999997</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>1450270137.4499998</t>
+        </is>
+      </c>
+      <c r="S52" s="2" t="inlineStr">
+        <is>
+          <t>4000171992.699999</t>
+        </is>
+      </c>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>781</t>
+        </is>
+      </c>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
+          <t>3844</t>
+        </is>
+      </c>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>15867</t>
+        </is>
+      </c>
+      <c r="W52" s="2" t="inlineStr">
+        <is>
+          <t>42524</t>
+        </is>
+      </c>
+      <c r="X52" s="2" t="inlineStr">
+        <is>
+          <t>2052628.8099999998</t>
+        </is>
+      </c>
+      <c r="Y52" s="2" t="inlineStr">
+        <is>
+          <t>121862364.24384336</t>
+        </is>
+      </c>
+      <c r="Z52" s="2" t="inlineStr">
+        <is>
+          <t>414319896.3120412</t>
+        </is>
+      </c>
+      <c r="AA52" s="2" t="inlineStr">
+        <is>
+          <t>1163549996.308302</t>
+        </is>
+      </c>
+      <c r="AB52" s="2" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="AC52" s="2" t="inlineStr">
+        <is>
+          <t>49093</t>
+        </is>
+      </c>
+      <c r="AD52" s="2" t="inlineStr">
+        <is>
+          <t>205890</t>
+        </is>
+      </c>
+      <c r="AE52" s="2" t="inlineStr">
+        <is>
+          <t>596116</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-11
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE52"/>
+  <dimension ref="A1:AE53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8636,6 +8636,163 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>26326558815.047752</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>632648269.013355</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>77675</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>629759803.684752</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>19490922694.959717</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>481437</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>7070</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>65981</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>332464</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>1322414</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>2433.32333348204</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>64998.861001704114</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>302079.52767463756</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>1045658.8174281403</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>65748278.00000003</t>
+        </is>
+      </c>
+      <c r="Q53" s="2" t="inlineStr">
+        <is>
+          <t>367358776.5399998</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>1519663270.4399998</t>
+        </is>
+      </c>
+      <c r="S53" s="2" t="inlineStr">
+        <is>
+          <t>4015729349.709999</t>
+        </is>
+      </c>
+      <c r="T53" s="2" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="U53" s="2" t="inlineStr">
+        <is>
+          <t>4024</t>
+        </is>
+      </c>
+      <c r="V53" s="2" t="inlineStr">
+        <is>
+          <t>16648</t>
+        </is>
+      </c>
+      <c r="W53" s="2" t="inlineStr">
+        <is>
+          <t>42789</t>
+        </is>
+      </c>
+      <c r="X53" s="2" t="inlineStr">
+        <is>
+          <t>1006881.0500000004</t>
+        </is>
+      </c>
+      <c r="Y53" s="2" t="inlineStr">
+        <is>
+          <t>127312059.81384325</t>
+        </is>
+      </c>
+      <c r="Z53" s="2" t="inlineStr">
+        <is>
+          <t>424432631.8420412</t>
+        </is>
+      </c>
+      <c r="AA53" s="2" t="inlineStr">
+        <is>
+          <t>1172956031.058302</t>
+        </is>
+      </c>
+      <c r="AB53" s="2" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="AC53" s="2" t="inlineStr">
+        <is>
+          <t>48874</t>
+        </is>
+      </c>
+      <c r="AD53" s="2" t="inlineStr">
+        <is>
+          <t>207131</t>
+        </is>
+      </c>
+      <c r="AE53" s="2" t="inlineStr">
+        <is>
+          <t>596340</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-12
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE53"/>
+  <dimension ref="A1:AE54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8793,6 +8793,163 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>26387033255.237473</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>642550098.7789639</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>77715</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>640623355.0144709</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>19539703820.76726</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>482260</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>6025</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>66324</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>334016</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>1333095</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>2019.570000104781</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>66619.53000183862</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>300289.31634131697</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>1044131.3420950404</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>55137725.08999998</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>365236184.9299999</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>1474031479.2699997</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>4034960494.399999</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>619</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>4017</t>
+        </is>
+      </c>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>16168</t>
+        </is>
+      </c>
+      <c r="W54" s="2" t="inlineStr">
+        <is>
+          <t>43047</t>
+        </is>
+      </c>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>1600712.6499999997</t>
+        </is>
+      </c>
+      <c r="Y54" s="2" t="inlineStr">
+        <is>
+          <t>126522570.58000012</t>
+        </is>
+      </c>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>433155375.8220412</t>
+        </is>
+      </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>1181210109.188302</t>
+        </is>
+      </c>
+      <c r="AB54" s="2" t="inlineStr">
+        <is>
+          <t>237</t>
+        </is>
+      </c>
+      <c r="AC54" s="2" t="inlineStr">
+        <is>
+          <t>48741</t>
+        </is>
+      </c>
+      <c r="AD54" s="2" t="inlineStr">
+        <is>
+          <t>207618</t>
+        </is>
+      </c>
+      <c r="AE54" s="2" t="inlineStr">
+        <is>
+          <t>596929</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-13
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE54"/>
+  <dimension ref="A1:AE55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8950,6 +8950,163 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>26407265390.84036</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>618039424.9104912</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>77737</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>615637144.3673592</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>19576235584.515213</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>483035</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>5478</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>71288</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>332030</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>1343934</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>1938.45666678141</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>68268.56000186948</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>299655.17967460566</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>1051877.9300952153</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>49491439.19000006</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>366376459.77999985</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>1472224869.7999997</t>
+        </is>
+      </c>
+      <c r="S55" s="2" t="inlineStr">
+        <is>
+          <t>4051692070.499999</t>
+        </is>
+      </c>
+      <c r="T55" s="2" t="inlineStr">
+        <is>
+          <t>583</t>
+        </is>
+      </c>
+      <c r="U55" s="2" t="inlineStr">
+        <is>
+          <t>4021</t>
+        </is>
+      </c>
+      <c r="V55" s="2" t="inlineStr">
+        <is>
+          <t>16158</t>
+        </is>
+      </c>
+      <c r="W55" s="2" t="inlineStr">
+        <is>
+          <t>43283</t>
+        </is>
+      </c>
+      <c r="X55" s="2" t="inlineStr">
+        <is>
+          <t>621566.1799999999</t>
+        </is>
+      </c>
+      <c r="Y55" s="2" t="inlineStr">
+        <is>
+          <t>129962259.94699924</t>
+        </is>
+      </c>
+      <c r="Z55" s="2" t="inlineStr">
+        <is>
+          <t>443970641.7190404</t>
+        </is>
+      </c>
+      <c r="AA55" s="2" t="inlineStr">
+        <is>
+          <t>1197285680.7157085</t>
+        </is>
+      </c>
+      <c r="AB55" s="2" t="inlineStr">
+        <is>
+          <t>174</t>
+        </is>
+      </c>
+      <c r="AC55" s="2" t="inlineStr">
+        <is>
+          <t>48801</t>
+        </is>
+      </c>
+      <c r="AD55" s="2" t="inlineStr">
+        <is>
+          <t>208901</t>
+        </is>
+      </c>
+      <c r="AE55" s="2" t="inlineStr">
+        <is>
+          <t>598961</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-14
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE55"/>
+  <dimension ref="A1:AE56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9107,6 +9107,163 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>26405807242.58274</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>618906245.9031675</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>77773</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>617039188.8097426</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>19573857880.473072</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>483036</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>2481</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>74405</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>325274</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>1214139</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>463.350000047391</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>68759.89833520721</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>290314.96667438286</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>1053790.9834286466</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>361450030.7199999</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>1454855591.0399997</t>
+        </is>
+      </c>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
+          <t>4101193867.2399993</t>
+        </is>
+      </c>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>4027</t>
+        </is>
+      </c>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>16026</t>
+        </is>
+      </c>
+      <c r="W56" s="2" t="inlineStr">
+        <is>
+          <t>43867</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>389534.36000000016</t>
+        </is>
+      </c>
+      <c r="Y56" s="2" t="inlineStr">
+        <is>
+          <t>129185812.60699925</t>
+        </is>
+      </c>
+      <c r="Z56" s="2" t="inlineStr">
+        <is>
+          <t>436983977.7690404</t>
+        </is>
+      </c>
+      <c r="AA56" s="2" t="inlineStr">
+        <is>
+          <t>1197214734.2357085</t>
+        </is>
+      </c>
+      <c r="AB56" s="2" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+      <c r="AC56" s="2" t="inlineStr">
+        <is>
+          <t>48606</t>
+        </is>
+      </c>
+      <c r="AD56" s="2" t="inlineStr">
+        <is>
+          <t>208843</t>
+        </is>
+      </c>
+      <c r="AE56" s="2" t="inlineStr">
+        <is>
+          <t>598868</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-15
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE56"/>
+  <dimension ref="A1:AE57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9264,6 +9264,163 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>26400671240.567257</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>617264166.9202025</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>77801</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>615735531.6742585</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>19568201232.63189</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>483039</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>3362</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>70884</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>321192</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>1061652</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>461.391000068286</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>69061.62033519946</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>269312.1836740015</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>1040023.8954277625</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>18026.9</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>361447912.7199999</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>1408175605.9199998</t>
+        </is>
+      </c>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>4101196038.709999</t>
+        </is>
+      </c>
+      <c r="T57" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U57" s="2" t="inlineStr">
+        <is>
+          <t>4027</t>
+        </is>
+      </c>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>15498</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="inlineStr">
+        <is>
+          <t>43867</t>
+        </is>
+      </c>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>7365768.749999982</t>
+        </is>
+      </c>
+      <c r="Y57" s="2" t="inlineStr">
+        <is>
+          <t>129412373.33699925</t>
+        </is>
+      </c>
+      <c r="Z57" s="2" t="inlineStr">
+        <is>
+          <t>427951123.3490404</t>
+        </is>
+      </c>
+      <c r="AA57" s="2" t="inlineStr">
+        <is>
+          <t>1193454314.8757083</t>
+        </is>
+      </c>
+      <c r="AB57" s="2" t="inlineStr">
+        <is>
+          <t>7194</t>
+        </is>
+      </c>
+      <c r="AC57" s="2" t="inlineStr">
+        <is>
+          <t>49038</t>
+        </is>
+      </c>
+      <c r="AD57" s="2" t="inlineStr">
+        <is>
+          <t>206390</t>
+        </is>
+      </c>
+      <c r="AE57" s="2" t="inlineStr">
+        <is>
+          <t>598862</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-16
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE57"/>
+  <dimension ref="A1:AE58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9421,6 +9421,163 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>26481322081.8692</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>601220294.0343875</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>77856</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>600325497.5962033</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>19642907146.447983</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>484531</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>9683</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>64759</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>323709</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>986980</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>3303.729000195048</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>67713.08800188405</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>274682.7046739871</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>1027621.2064264857</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>99184450.75999999</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>361349226.11999995</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>1361576999.9899998</t>
+        </is>
+      </c>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>4001450236.6399994</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>1117</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
+          <t>4029</t>
+        </is>
+      </c>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>14984</t>
+        </is>
+      </c>
+      <c r="W58" s="2" t="inlineStr">
+        <is>
+          <t>42866</t>
+        </is>
+      </c>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>1654404.0699999998</t>
+        </is>
+      </c>
+      <c r="Y58" s="2" t="inlineStr">
+        <is>
+          <t>120778604.66699933</t>
+        </is>
+      </c>
+      <c r="Z58" s="2" t="inlineStr">
+        <is>
+          <t>432941824.06904036</t>
+        </is>
+      </c>
+      <c r="AA58" s="2" t="inlineStr">
+        <is>
+          <t>1194659587.9457085</t>
+        </is>
+      </c>
+      <c r="AB58" s="2" t="inlineStr">
+        <is>
+          <t>248</t>
+        </is>
+      </c>
+      <c r="AC58" s="2" t="inlineStr">
+        <is>
+          <t>50502</t>
+        </is>
+      </c>
+      <c r="AD58" s="2" t="inlineStr">
+        <is>
+          <t>207722</t>
+        </is>
+      </c>
+      <c r="AE58" s="2" t="inlineStr">
+        <is>
+          <t>600050</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-17
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE58"/>
+  <dimension ref="A1:AE59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9578,6 +9578,163 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>26170104130.81579</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>224998489.6582316</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>77905</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>224528525.5827886</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>19688425207.271744</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>485540</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>7660</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>65812</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>329112</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>962810</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>2393.778666794896</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>68245.23533519296</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>284406.15734071186</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>1017962.0207591389</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>67538867.97</t>
+        </is>
+      </c>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>339569286.9499999</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>1460705122.2699997</t>
+        </is>
+      </c>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>4052196441.049999</t>
+        </is>
+      </c>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>783</t>
+        </is>
+      </c>
+      <c r="U59" s="2" t="inlineStr">
+        <is>
+          <t>3861</t>
+        </is>
+      </c>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
+          <t>16101</t>
+        </is>
+      </c>
+      <c r="W59" s="2" t="inlineStr">
+        <is>
+          <t>43464</t>
+        </is>
+      </c>
+      <c r="X59" s="2" t="inlineStr">
+        <is>
+          <t>823803.5299999999</t>
+        </is>
+      </c>
+      <c r="Y59" s="2" t="inlineStr">
+        <is>
+          <t>105417976.91699922</t>
+        </is>
+      </c>
+      <c r="Z59" s="2" t="inlineStr">
+        <is>
+          <t>438980595.65904033</t>
+        </is>
+      </c>
+      <c r="AA59" s="2" t="inlineStr">
+        <is>
+          <t>1195448422.3057084</t>
+        </is>
+      </c>
+      <c r="AB59" s="2" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="AC59" s="2" t="inlineStr">
+        <is>
+          <t>50784</t>
+        </is>
+      </c>
+      <c r="AD59" s="2" t="inlineStr">
+        <is>
+          <t>207755</t>
+        </is>
+      </c>
+      <c r="AE59" s="2" t="inlineStr">
+        <is>
+          <t>600714</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-18
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE59"/>
+  <dimension ref="A1:AE60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9735,6 +9735,163 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>26212660476.026962</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>197631356.6805187</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>77940</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>196238419.2739607</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>19756930355.508446</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>486587</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>7329</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>66478</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>327832</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>961644</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>2300.082000142815</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>66634.07700167809</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>286267.5880073893</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>1010701.3810922562</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>74735690.01000004</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>337662743.8699999</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>1528109211.9599996</t>
+        </is>
+      </c>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>4069257709.1599994</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>836</t>
+        </is>
+      </c>
+      <c r="U60" s="2" t="inlineStr">
+        <is>
+          <t>3864</t>
+        </is>
+      </c>
+      <c r="V60" s="2" t="inlineStr">
+        <is>
+          <t>16886</t>
+        </is>
+      </c>
+      <c r="W60" s="2" t="inlineStr">
+        <is>
+          <t>43723</t>
+        </is>
+      </c>
+      <c r="X60" s="2" t="inlineStr">
+        <is>
+          <t>793871.7100000002</t>
+        </is>
+      </c>
+      <c r="Y60" s="2" t="inlineStr">
+        <is>
+          <t>97818199.62699924</t>
+        </is>
+      </c>
+      <c r="Z60" s="2" t="inlineStr">
+        <is>
+          <t>440128574.15904033</t>
+        </is>
+      </c>
+      <c r="AA60" s="2" t="inlineStr">
+        <is>
+          <t>1198118167.3357084</t>
+        </is>
+      </c>
+      <c r="AB60" s="2" t="inlineStr">
+        <is>
+          <t>245</t>
+        </is>
+      </c>
+      <c r="AC60" s="2" t="inlineStr">
+        <is>
+          <t>51859</t>
+        </is>
+      </c>
+      <c r="AD60" s="2" t="inlineStr">
+        <is>
+          <t>208997</t>
+        </is>
+      </c>
+      <c r="AE60" s="2" t="inlineStr">
+        <is>
+          <t>603334</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-19
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE60"/>
+  <dimension ref="A1:AE61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9892,6 +9892,163 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>26247855567.460777</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>183687616.26659897</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>77984</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>182243715.26777884</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>19783626663.693264</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>487426</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>6790</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>67092</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>327902</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>966106</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>2116.038000144636</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>66127.46833494105</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>283785.3913406349</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>1008475.2134256584</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>53193776.049999975</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>347267924.6799998</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>1486639958.8099997</t>
+        </is>
+      </c>
+      <c r="S61" s="2" t="inlineStr">
+        <is>
+          <t>4098377508.9899993</t>
+        </is>
+      </c>
+      <c r="T61" s="2" t="inlineStr">
+        <is>
+          <t>642</t>
+        </is>
+      </c>
+      <c r="U61" s="2" t="inlineStr">
+        <is>
+          <t>3956</t>
+        </is>
+      </c>
+      <c r="V61" s="2" t="inlineStr">
+        <is>
+          <t>16419</t>
+        </is>
+      </c>
+      <c r="W61" s="2" t="inlineStr">
+        <is>
+          <t>44089</t>
+        </is>
+      </c>
+      <c r="X61" s="2" t="inlineStr">
+        <is>
+          <t>1794706.01</t>
+        </is>
+      </c>
+      <c r="Y61" s="2" t="inlineStr">
+        <is>
+          <t>89605874.1120733</t>
+        </is>
+      </c>
+      <c r="Z61" s="2" t="inlineStr">
+        <is>
+          <t>438874574.99411446</t>
+        </is>
+      </c>
+      <c r="AA61" s="2" t="inlineStr">
+        <is>
+          <t>1198937556.4807825</t>
+        </is>
+      </c>
+      <c r="AB61" s="2" t="inlineStr">
+        <is>
+          <t>274</t>
+        </is>
+      </c>
+      <c r="AC61" s="2" t="inlineStr">
+        <is>
+          <t>53296</t>
+        </is>
+      </c>
+      <c r="AD61" s="2" t="inlineStr">
+        <is>
+          <t>211912</t>
+        </is>
+      </c>
+      <c r="AE61" s="2" t="inlineStr">
+        <is>
+          <t>604855</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-20
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE61"/>
+  <dimension ref="A1:AE62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10049,6 +10049,163 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>26250267173.208817</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>187357351.01405162</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>78026</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>187205859.3758166</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>19777727106.090515</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>487427</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>68956</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>323233</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>969851</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>331.986000054249</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>59917.36833491273</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>279032.45800723846</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>1008969.5754257318</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>344965499.4799999</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>1479681556.3099997</t>
+        </is>
+      </c>
+      <c r="S62" s="2" t="inlineStr">
+        <is>
+          <t>4102732096.879999</t>
+        </is>
+      </c>
+      <c r="T62" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U62" s="2" t="inlineStr">
+        <is>
+          <t>3978</t>
+        </is>
+      </c>
+      <c r="V62" s="2" t="inlineStr">
+        <is>
+          <t>16402</t>
+        </is>
+      </c>
+      <c r="W62" s="2" t="inlineStr">
+        <is>
+          <t>44239</t>
+        </is>
+      </c>
+      <c r="X62" s="2" t="inlineStr">
+        <is>
+          <t>345208.69000000006</t>
+        </is>
+      </c>
+      <c r="Y62" s="2" t="inlineStr">
+        <is>
+          <t>76310090.20507416</t>
+        </is>
+      </c>
+      <c r="Z62" s="2" t="inlineStr">
+        <is>
+          <t>432216042.71924996</t>
+        </is>
+      </c>
+      <c r="AA62" s="2" t="inlineStr">
+        <is>
+          <t>1202075180.5007825</t>
+        </is>
+      </c>
+      <c r="AB62" s="2" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="AC62" s="2" t="inlineStr">
+        <is>
+          <t>51598</t>
+        </is>
+      </c>
+      <c r="AD62" s="2" t="inlineStr">
+        <is>
+          <t>210430</t>
+        </is>
+      </c>
+      <c r="AE62" s="2" t="inlineStr">
+        <is>
+          <t>605569</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-21
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE62"/>
+  <dimension ref="A1:AE63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10206,6 +10206,163 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>26247256646.262264</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>187223069.623766</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>78058</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>186938016.179263</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>19772413290.183075</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>487427</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>2506</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>68724</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>314849</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>966829</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>379.97000005596</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>58900.547001501116</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>268778.55234027805</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>1009329.1260923903</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>295463702.73999983</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>1415073850.4099996</t>
+        </is>
+      </c>
+      <c r="S63" s="2" t="inlineStr">
+        <is>
+          <t>4102674610.0999994</t>
+        </is>
+      </c>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U63" s="2" t="inlineStr">
+        <is>
+          <t>3394</t>
+        </is>
+      </c>
+      <c r="V63" s="2" t="inlineStr">
+        <is>
+          <t>15678</t>
+        </is>
+      </c>
+      <c r="W63" s="2" t="inlineStr">
+        <is>
+          <t>44237</t>
+        </is>
+      </c>
+      <c r="X63" s="2" t="inlineStr">
+        <is>
+          <t>183588.14999999994</t>
+        </is>
+      </c>
+      <c r="Y63" s="2" t="inlineStr">
+        <is>
+          <t>76153291.96507414</t>
+        </is>
+      </c>
+      <c r="Z63" s="2" t="inlineStr">
+        <is>
+          <t>424629855.16924995</t>
+        </is>
+      </c>
+      <c r="AA63" s="2" t="inlineStr">
+        <is>
+          <t>1203665058.9107826</t>
+        </is>
+      </c>
+      <c r="AB63" s="2" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="AC63" s="2" t="inlineStr">
+        <is>
+          <t>52277</t>
+        </is>
+      </c>
+      <c r="AD63" s="2" t="inlineStr">
+        <is>
+          <t>211250</t>
+        </is>
+      </c>
+      <c r="AE63" s="2" t="inlineStr">
+        <is>
+          <t>607082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-22
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE63"/>
+  <dimension ref="A1:AE64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10363,6 +10363,163 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>26243638708.55432</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>185119254.21191168</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>78098</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>184912712.18131968</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>19774038869.450954</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>487428</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>3042</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>63823</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>310224</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>958315</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>307.018666720112</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>58863.878001499426</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>259212.64667340307</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>998989.7554256828</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>295469872.85999984</t>
+        </is>
+      </c>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>1365981105.8599997</t>
+        </is>
+      </c>
+      <c r="S64" s="2" t="inlineStr">
+        <is>
+          <t>4102474683.629999</t>
+        </is>
+      </c>
+      <c r="T64" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U64" s="2" t="inlineStr">
+        <is>
+          <t>3394</t>
+        </is>
+      </c>
+      <c r="V64" s="2" t="inlineStr">
+        <is>
+          <t>15130</t>
+        </is>
+      </c>
+      <c r="W64" s="2" t="inlineStr">
+        <is>
+          <t>44234</t>
+        </is>
+      </c>
+      <c r="X64" s="2" t="inlineStr">
+        <is>
+          <t>5088314.130000015</t>
+        </is>
+      </c>
+      <c r="Y64" s="2" t="inlineStr">
+        <is>
+          <t>74690826.40507413</t>
+        </is>
+      </c>
+      <c r="Z64" s="2" t="inlineStr">
+        <is>
+          <t>413853183.47925</t>
+        </is>
+      </c>
+      <c r="AA64" s="2" t="inlineStr">
+        <is>
+          <t>1197875367.3907826</t>
+        </is>
+      </c>
+      <c r="AB64" s="2" t="inlineStr">
+        <is>
+          <t>6297</t>
+        </is>
+      </c>
+      <c r="AC64" s="2" t="inlineStr">
+        <is>
+          <t>51948</t>
+        </is>
+      </c>
+      <c r="AD64" s="2" t="inlineStr">
+        <is>
+          <t>209490</t>
+        </is>
+      </c>
+      <c r="AE64" s="2" t="inlineStr">
+        <is>
+          <t>606488</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-23
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE64"/>
+  <dimension ref="A1:AE65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10520,6 +10520,163 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>26350898934.172123</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>183739182.72249323</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>78125</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>182013340.12912393</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>19861852031.839252</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>489144</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>9682</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>55671</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>313345</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>954950</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>5109.42666686116</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>58294.1370014656</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>263641.50000670855</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>990110.8597589299</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>110760007.47000006</t>
+        </is>
+      </c>
+      <c r="Q65" s="2" t="inlineStr">
+        <is>
+          <t>295476105.54999983</t>
+        </is>
+      </c>
+      <c r="R65" s="2" t="inlineStr">
+        <is>
+          <t>1316498931.9799995</t>
+        </is>
+      </c>
+      <c r="S65" s="2" t="inlineStr">
+        <is>
+          <t>4009533542.7799993</t>
+        </is>
+      </c>
+      <c r="T65" s="2" t="inlineStr">
+        <is>
+          <t>1236</t>
+        </is>
+      </c>
+      <c r="U65" s="2" t="inlineStr">
+        <is>
+          <t>3393</t>
+        </is>
+      </c>
+      <c r="V65" s="2" t="inlineStr">
+        <is>
+          <t>14604</t>
+        </is>
+      </c>
+      <c r="W65" s="2" t="inlineStr">
+        <is>
+          <t>43262</t>
+        </is>
+      </c>
+      <c r="X65" s="2" t="inlineStr">
+        <is>
+          <t>1191711.9000000004</t>
+        </is>
+      </c>
+      <c r="Y65" s="2" t="inlineStr">
+        <is>
+          <t>71555285.62507416</t>
+        </is>
+      </c>
+      <c r="Z65" s="2" t="inlineStr">
+        <is>
+          <t>415590386.26925004</t>
+        </is>
+      </c>
+      <c r="AA65" s="2" t="inlineStr">
+        <is>
+          <t>1196112345.8707826</t>
+        </is>
+      </c>
+      <c r="AB65" s="2" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="AC65" s="2" t="inlineStr">
+        <is>
+          <t>50931</t>
+        </is>
+      </c>
+      <c r="AD65" s="2" t="inlineStr">
+        <is>
+          <t>209621</t>
+        </is>
+      </c>
+      <c r="AE65" s="2" t="inlineStr">
+        <is>
+          <t>607129</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-24
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE65"/>
+  <dimension ref="A1:AE66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10677,6 +10677,163 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>26416641738.55839</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>181836374.05732498</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>78157</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>180900786.07539156</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>19909249115.524628</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>490156</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>6649</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>56720</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>324944</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>960788</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>2994.546000133125</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>62734.669668234164</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>278187.47200696415</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>980853.8390923938</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>71044331.81000002</t>
+        </is>
+      </c>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>307128222.76</t>
+        </is>
+      </c>
+      <c r="R66" s="2" t="inlineStr">
+        <is>
+          <t>1427352798.4299996</t>
+        </is>
+      </c>
+      <c r="S66" s="2" t="inlineStr">
+        <is>
+          <t>4065135658.3299994</t>
+        </is>
+      </c>
+      <c r="T66" s="2" t="inlineStr">
+        <is>
+          <t>793</t>
+        </is>
+      </c>
+      <c r="U66" s="2" t="inlineStr">
+        <is>
+          <t>3513</t>
+        </is>
+      </c>
+      <c r="V66" s="2" t="inlineStr">
+        <is>
+          <t>15842</t>
+        </is>
+      </c>
+      <c r="W66" s="2" t="inlineStr">
+        <is>
+          <t>43941</t>
+        </is>
+      </c>
+      <c r="X66" s="2" t="inlineStr">
+        <is>
+          <t>2310644.7199999997</t>
+        </is>
+      </c>
+      <c r="Y66" s="2" t="inlineStr">
+        <is>
+          <t>79590356.05562574</t>
+        </is>
+      </c>
+      <c r="Z66" s="2" t="inlineStr">
+        <is>
+          <t>429274274.7198016</t>
+        </is>
+      </c>
+      <c r="AA66" s="2" t="inlineStr">
+        <is>
+          <t>1205213183.9913342</t>
+        </is>
+      </c>
+      <c r="AB66" s="2" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="AC66" s="2" t="inlineStr">
+        <is>
+          <t>51245</t>
+        </is>
+      </c>
+      <c r="AD66" s="2" t="inlineStr">
+        <is>
+          <t>210444</t>
+        </is>
+      </c>
+      <c r="AE66" s="2" t="inlineStr">
+        <is>
+          <t>608634</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-25
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE66"/>
+  <dimension ref="A1:AE67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10834,6 +10834,163 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>26500180246.326992</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>177700017.4921303</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>78195</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>177374511.12399048</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>19981384931.3004</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>491434</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>7514</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>58844</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>331917</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>966305</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>2179.545000102513</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>66413.82933501064</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>292143.28234058886</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>981376.980092593</t>
+        </is>
+      </c>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>88173177.24999994</t>
+        </is>
+      </c>
+      <c r="Q67" s="2" t="inlineStr">
+        <is>
+          <t>310831848.16999996</t>
+        </is>
+      </c>
+      <c r="R67" s="2" t="inlineStr">
+        <is>
+          <t>1498624796.3599994</t>
+        </is>
+      </c>
+      <c r="S67" s="2" t="inlineStr">
+        <is>
+          <t>4088311727.519999</t>
+        </is>
+      </c>
+      <c r="T67" s="2" t="inlineStr">
+        <is>
+          <t>1037</t>
+        </is>
+      </c>
+      <c r="U67" s="2" t="inlineStr">
+        <is>
+          <t>3521</t>
+        </is>
+      </c>
+      <c r="V67" s="2" t="inlineStr">
+        <is>
+          <t>16636</t>
+        </is>
+      </c>
+      <c r="W67" s="2" t="inlineStr">
+        <is>
+          <t>44244</t>
+        </is>
+      </c>
+      <c r="X67" s="2" t="inlineStr">
+        <is>
+          <t>934337.2900000002</t>
+        </is>
+      </c>
+      <c r="Y67" s="2" t="inlineStr">
+        <is>
+          <t>83416012.22562574</t>
+        </is>
+      </c>
+      <c r="Z67" s="2" t="inlineStr">
+        <is>
+          <t>440913549.98646826</t>
+        </is>
+      </c>
+      <c r="AA67" s="2" t="inlineStr">
+        <is>
+          <t>1211629122.4413342</t>
+        </is>
+      </c>
+      <c r="AB67" s="2" t="inlineStr">
+        <is>
+          <t>265</t>
+        </is>
+      </c>
+      <c r="AC67" s="2" t="inlineStr">
+        <is>
+          <t>50662</t>
+        </is>
+      </c>
+      <c r="AD67" s="2" t="inlineStr">
+        <is>
+          <t>212341</t>
+        </is>
+      </c>
+      <c r="AE67" s="2" t="inlineStr">
+        <is>
+          <t>609559</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-26
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE67"/>
+  <dimension ref="A1:AE68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10991,6 +10991,163 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>26547356173.847557</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>167939537.53669629</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>78228</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>167607193.7945583</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>20023292972.056667</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>492431</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>7821</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>68691</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>338225</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>978722</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>2900.94600014901</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>67949.16200179582</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>293101.8950074844</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>981231.8294261942</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>64542816.029999994</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>323721367.59</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="inlineStr">
+        <is>
+          <t>1586857595.1499996</t>
+        </is>
+      </c>
+      <c r="S68" s="2" t="inlineStr">
+        <is>
+          <t>4131723993.769999</t>
+        </is>
+      </c>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>787</t>
+        </is>
+      </c>
+      <c r="U68" s="2" t="inlineStr">
+        <is>
+          <t>3720</t>
+        </is>
+      </c>
+      <c r="V68" s="2" t="inlineStr">
+        <is>
+          <t>17674</t>
+        </is>
+      </c>
+      <c r="W68" s="2" t="inlineStr">
+        <is>
+          <t>44858</t>
+        </is>
+      </c>
+      <c r="X68" s="2" t="inlineStr">
+        <is>
+          <t>15360650.670000002</t>
+        </is>
+      </c>
+      <c r="Y68" s="2" t="inlineStr">
+        <is>
+          <t>84078825.50055161</t>
+        </is>
+      </c>
+      <c r="Z68" s="2" t="inlineStr">
+        <is>
+          <t>441186080.0464682</t>
+        </is>
+      </c>
+      <c r="AA68" s="2" t="inlineStr">
+        <is>
+          <t>1214226870.7913342</t>
+        </is>
+      </c>
+      <c r="AB68" s="2" t="inlineStr">
+        <is>
+          <t>428</t>
+        </is>
+      </c>
+      <c r="AC68" s="2" t="inlineStr">
+        <is>
+          <t>48800</t>
+        </is>
+      </c>
+      <c r="AD68" s="2" t="inlineStr">
+        <is>
+          <t>212315</t>
+        </is>
+      </c>
+      <c r="AE68" s="2" t="inlineStr">
+        <is>
+          <t>609587</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-27
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE68"/>
+  <dimension ref="A1:AE69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11148,6 +11148,163 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>26605550610.132324</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>170650153.42399296</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>78260</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>170363431.63932398</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>20073513496.66118</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>493317</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>5712</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>78457</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>334944</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>988042</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>1592.178000094557</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>73136.3650018199</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>291628.6746741387</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>986369.4007596507</t>
+        </is>
+      </c>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>60314329.859999985</t>
+        </is>
+      </c>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>335054157.2599999</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="inlineStr">
+        <is>
+          <t>1556761468.1099994</t>
+        </is>
+      </c>
+      <c r="S69" s="2" t="inlineStr">
+        <is>
+          <t>4156983544.6799994</t>
+        </is>
+      </c>
+      <c r="T69" s="2" t="inlineStr">
+        <is>
+          <t>702</t>
+        </is>
+      </c>
+      <c r="U69" s="2" t="inlineStr">
+        <is>
+          <t>3864</t>
+        </is>
+      </c>
+      <c r="V69" s="2" t="inlineStr">
+        <is>
+          <t>17400</t>
+        </is>
+      </c>
+      <c r="W69" s="2" t="inlineStr">
+        <is>
+          <t>45243</t>
+        </is>
+      </c>
+      <c r="X69" s="2" t="inlineStr">
+        <is>
+          <t>1091504.6199999996</t>
+        </is>
+      </c>
+      <c r="Y69" s="2" t="inlineStr">
+        <is>
+          <t>112960568.78055155</t>
+        </is>
+      </c>
+      <c r="Z69" s="2" t="inlineStr">
+        <is>
+          <t>467890696.7564682</t>
+        </is>
+      </c>
+      <c r="AA69" s="2" t="inlineStr">
+        <is>
+          <t>1244912114.7613342</t>
+        </is>
+      </c>
+      <c r="AB69" s="2" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="AC69" s="2" t="inlineStr">
+        <is>
+          <t>50988</t>
+        </is>
+      </c>
+      <c r="AD69" s="2" t="inlineStr">
+        <is>
+          <t>213506</t>
+        </is>
+      </c>
+      <c r="AE69" s="2" t="inlineStr">
+        <is>
+          <t>611038</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-28
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE69"/>
+  <dimension ref="A1:AE70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11305,6 +11305,163 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>26600982754.531536</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>169598087.94411966</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>78303</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>169514137.75853568</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>20070199799.677902</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>493318</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>2453</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>83073</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>328754</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>988160</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>275.187000051765</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>73990.66300188839</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>282783.09800725133</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>988387.6574263969</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>106259.33</t>
+        </is>
+      </c>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>395368487.1199998</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr">
+        <is>
+          <t>1530421745.7299993</t>
+        </is>
+      </c>
+      <c r="S70" s="2" t="inlineStr">
+        <is>
+          <t>4217297874.539999</t>
+        </is>
+      </c>
+      <c r="T70" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U70" s="2" t="inlineStr">
+        <is>
+          <t>4566</t>
+        </is>
+      </c>
+      <c r="V70" s="2" t="inlineStr">
+        <is>
+          <t>17171</t>
+        </is>
+      </c>
+      <c r="W70" s="2" t="inlineStr">
+        <is>
+          <t>45945</t>
+        </is>
+      </c>
+      <c r="X70" s="2" t="inlineStr">
+        <is>
+          <t>587939.4700000001</t>
+        </is>
+      </c>
+      <c r="Y70" s="2" t="inlineStr">
+        <is>
+          <t>114411040.72055152</t>
+        </is>
+      </c>
+      <c r="Z70" s="2" t="inlineStr">
+        <is>
+          <t>458354267.93646824</t>
+        </is>
+      </c>
+      <c r="AA70" s="2" t="inlineStr">
+        <is>
+          <t>1249412360.1813343</t>
+        </is>
+      </c>
+      <c r="AB70" s="2" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="AC70" s="2" t="inlineStr">
+        <is>
+          <t>50992</t>
+        </is>
+      </c>
+      <c r="AD70" s="2" t="inlineStr">
+        <is>
+          <t>212621</t>
+        </is>
+      </c>
+      <c r="AE70" s="2" t="inlineStr">
+        <is>
+          <t>614007</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-29
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE70"/>
+  <dimension ref="A1:AE71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11462,6 +11462,163 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>26597981495.497906</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>171836806.71515846</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>78329</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>170705818.94490546</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>20068948565.266804</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>493318</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>3443</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>79648</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>324539</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>980844</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>404.680000064552</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>73918.23100189038</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>271547.8910070456</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>982106.3804264048</t>
+        </is>
+      </c>
+      <c r="P71" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>395458574.3299998</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t>1469001474.4499993</t>
+        </is>
+      </c>
+      <c r="S71" s="2" t="inlineStr">
+        <is>
+          <t>4217177105.639999</t>
+        </is>
+      </c>
+      <c r="T71" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U71" s="2" t="inlineStr">
+        <is>
+          <t>4566</t>
+        </is>
+      </c>
+      <c r="V71" s="2" t="inlineStr">
+        <is>
+          <t>16529</t>
+        </is>
+      </c>
+      <c r="W71" s="2" t="inlineStr">
+        <is>
+          <t>45944</t>
+        </is>
+      </c>
+      <c r="X71" s="2" t="inlineStr">
+        <is>
+          <t>667183.9099999998</t>
+        </is>
+      </c>
+      <c r="Y71" s="2" t="inlineStr">
+        <is>
+          <t>117697512.29055153</t>
+        </is>
+      </c>
+      <c r="Z71" s="2" t="inlineStr">
+        <is>
+          <t>448166033.0864683</t>
+        </is>
+      </c>
+      <c r="AA71" s="2" t="inlineStr">
+        <is>
+          <t>1240525162.4713342</t>
+        </is>
+      </c>
+      <c r="AB71" s="2" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="AC71" s="2" t="inlineStr">
+        <is>
+          <t>52543</t>
+        </is>
+      </c>
+      <c r="AD71" s="2" t="inlineStr">
+        <is>
+          <t>213424</t>
+        </is>
+      </c>
+      <c r="AE71" s="2" t="inlineStr">
+        <is>
+          <t>615682</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-06-30
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE71"/>
+  <dimension ref="A1:AE72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11619,6 +11619,163 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>26692234789.45333</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>167516840.45814496</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>78368</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>166304232.40032998</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>20153758260.73484</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>494556</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>6063</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>72144</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>328545</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>981118</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>2740.023000106353</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>75156.41100193092</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>277034.4476737365</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>979325.5527597803</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>101927598.09</t>
+        </is>
+      </c>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>396787574.8399998</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t>1417525054.6499994</t>
+        </is>
+      </c>
+      <c r="S72" s="2" t="inlineStr">
+        <is>
+          <t>4155940453.089999</t>
+        </is>
+      </c>
+      <c r="T72" s="2" t="inlineStr">
+        <is>
+          <t>1221</t>
+        </is>
+      </c>
+      <c r="U72" s="2" t="inlineStr">
+        <is>
+          <t>4566</t>
+        </is>
+      </c>
+      <c r="V72" s="2" t="inlineStr">
+        <is>
+          <t>15949</t>
+        </is>
+      </c>
+      <c r="W72" s="2" t="inlineStr">
+        <is>
+          <t>45314</t>
+        </is>
+      </c>
+      <c r="X72" s="2" t="inlineStr">
+        <is>
+          <t>745322.5100000004</t>
+        </is>
+      </c>
+      <c r="Y72" s="2" t="inlineStr">
+        <is>
+          <t>120295479.70055147</t>
+        </is>
+      </c>
+      <c r="Z72" s="2" t="inlineStr">
+        <is>
+          <t>453605748.7664683</t>
+        </is>
+      </c>
+      <c r="AA72" s="2" t="inlineStr">
+        <is>
+          <t>1228669094.4413342</t>
+        </is>
+      </c>
+      <c r="AB72" s="2" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="AC72" s="2" t="inlineStr">
+        <is>
+          <t>51366</t>
+        </is>
+      </c>
+      <c r="AD72" s="2" t="inlineStr">
+        <is>
+          <t>213147</t>
+        </is>
+      </c>
+      <c r="AE72" s="2" t="inlineStr">
+        <is>
+          <t>619492</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-01
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE72"/>
+  <dimension ref="A1:AE73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11776,6 +11776,163 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>26930941558.357304</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>354698826.61145604</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>78400</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>351305355.64430404</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>20161038385.40544</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>495273</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>5545</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>69284</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>334118</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>978907</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>1852.432000062928</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>71824.20600179968</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>287915.97334052186</t>
+        </is>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>981575.659759922</t>
+        </is>
+      </c>
+      <c r="P73" s="2" t="inlineStr">
+        <is>
+          <t>59282457.14</t>
+        </is>
+      </c>
+      <c r="Q73" s="2" t="inlineStr">
+        <is>
+          <t>387934442.79</t>
+        </is>
+      </c>
+      <c r="R73" s="2" t="inlineStr">
+        <is>
+          <t>1519519543.8599994</t>
+        </is>
+      </c>
+      <c r="S73" s="2" t="inlineStr">
+        <is>
+          <t>4228067931.0299993</t>
+        </is>
+      </c>
+      <c r="T73" s="2" t="inlineStr">
+        <is>
+          <t>696</t>
+        </is>
+      </c>
+      <c r="U73" s="2" t="inlineStr">
+        <is>
+          <t>4550</t>
+        </is>
+      </c>
+      <c r="V73" s="2" t="inlineStr">
+        <is>
+          <t>17171</t>
+        </is>
+      </c>
+      <c r="W73" s="2" t="inlineStr">
+        <is>
+          <t>46230</t>
+        </is>
+      </c>
+      <c r="X73" s="2" t="inlineStr">
+        <is>
+          <t>9065359.559999997</t>
+        </is>
+      </c>
+      <c r="Y73" s="2" t="inlineStr">
+        <is>
+          <t>125391915.17999996</t>
+        </is>
+      </c>
+      <c r="Z73" s="2" t="inlineStr">
+        <is>
+          <t>476984381.44646835</t>
+        </is>
+      </c>
+      <c r="AA73" s="2" t="inlineStr">
+        <is>
+          <t>1241014185.7913344</t>
+        </is>
+      </c>
+      <c r="AB73" s="2" t="inlineStr">
+        <is>
+          <t>430</t>
+        </is>
+      </c>
+      <c r="AC73" s="2" t="inlineStr">
+        <is>
+          <t>51238</t>
+        </is>
+      </c>
+      <c r="AD73" s="2" t="inlineStr">
+        <is>
+          <t>219243</t>
+        </is>
+      </c>
+      <c r="AE73" s="2" t="inlineStr">
+        <is>
+          <t>619806</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-02
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE73"/>
+  <dimension ref="A1:AE74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11933,6 +11933,163 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>27050380384.45192</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>373153462.187456</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>78427</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>373066769.73892</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>20250945682.7417</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>497171</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>9786</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>62639</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>329952</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>982120</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>3007.978666810864</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>67801.73433500713</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>290779.49467398843</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>977160.7057599042</t>
+        </is>
+      </c>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>94664821.25000003</t>
+        </is>
+      </c>
+      <c r="Q74" s="2" t="inlineStr">
+        <is>
+          <t>376151301.76000005</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="inlineStr">
+        <is>
+          <t>1578981998.5799994</t>
+        </is>
+      </c>
+      <c r="S74" s="2" t="inlineStr">
+        <is>
+          <t>4168656078.339999</t>
+        </is>
+      </c>
+      <c r="T74" s="2" t="inlineStr">
+        <is>
+          <t>1036</t>
+        </is>
+      </c>
+      <c r="U74" s="2" t="inlineStr">
+        <is>
+          <t>4456</t>
+        </is>
+      </c>
+      <c r="V74" s="2" t="inlineStr">
+        <is>
+          <t>17869</t>
+        </is>
+      </c>
+      <c r="W74" s="2" t="inlineStr">
+        <is>
+          <t>45720</t>
+        </is>
+      </c>
+      <c r="X74" s="2" t="inlineStr">
+        <is>
+          <t>2329004.06</t>
+        </is>
+      </c>
+      <c r="Y74" s="2" t="inlineStr">
+        <is>
+          <t>132029754.53999995</t>
+        </is>
+      </c>
+      <c r="Z74" s="2" t="inlineStr">
+        <is>
+          <t>478077519.74646825</t>
+        </is>
+      </c>
+      <c r="AA74" s="2" t="inlineStr">
+        <is>
+          <t>1243647527.5713344</t>
+        </is>
+      </c>
+      <c r="AB74" s="2" t="inlineStr">
+        <is>
+          <t>324</t>
+        </is>
+      </c>
+      <c r="AC74" s="2" t="inlineStr">
+        <is>
+          <t>54593</t>
+        </is>
+      </c>
+      <c r="AD74" s="2" t="inlineStr">
+        <is>
+          <t>221422</t>
+        </is>
+      </c>
+      <c r="AE74" s="2" t="inlineStr">
+        <is>
+          <t>622660</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-03
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE74"/>
+  <dimension ref="A1:AE75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12090,6 +12090,163 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>27102371899.32616</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>377910740.0253136</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>78458</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>375895790.2531616</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>20285640955.676094</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>497993</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>5193</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>68284</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>336982</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>995056</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>1795.872000083166</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>68481.97233492533</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>291927.2766740018</t>
+        </is>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>979352.2064267615</t>
+        </is>
+      </c>
+      <c r="P75" s="2" t="inlineStr">
+        <is>
+          <t>52232286.62000002</t>
+        </is>
+      </c>
+      <c r="Q75" s="2" t="inlineStr">
+        <is>
+          <t>382629929.3500001</t>
+        </is>
+      </c>
+      <c r="R75" s="2" t="inlineStr">
+        <is>
+          <t>1539824541.7199996</t>
+        </is>
+      </c>
+      <c r="S75" s="2" t="inlineStr">
+        <is>
+          <t>4210994274.2499995</t>
+        </is>
+      </c>
+      <c r="T75" s="2" t="inlineStr">
+        <is>
+          <t>622</t>
+        </is>
+      </c>
+      <c r="U75" s="2" t="inlineStr">
+        <is>
+          <t>4455</t>
+        </is>
+      </c>
+      <c r="V75" s="2" t="inlineStr">
+        <is>
+          <t>17506</t>
+        </is>
+      </c>
+      <c r="W75" s="2" t="inlineStr">
+        <is>
+          <t>46220</t>
+        </is>
+      </c>
+      <c r="X75" s="2" t="inlineStr">
+        <is>
+          <t>1170932.32</t>
+        </is>
+      </c>
+      <c r="Y75" s="2" t="inlineStr">
+        <is>
+          <t>139833583.07000005</t>
+        </is>
+      </c>
+      <c r="Z75" s="2" t="inlineStr">
+        <is>
+          <t>477428465.5364684</t>
+        </is>
+      </c>
+      <c r="AA75" s="2" t="inlineStr">
+        <is>
+          <t>1250466581.4413342</t>
+        </is>
+      </c>
+      <c r="AB75" s="2" t="inlineStr">
+        <is>
+          <t>266</t>
+        </is>
+      </c>
+      <c r="AC75" s="2" t="inlineStr">
+        <is>
+          <t>57172</t>
+        </is>
+      </c>
+      <c r="AD75" s="2" t="inlineStr">
+        <is>
+          <t>222490</t>
+        </is>
+      </c>
+      <c r="AE75" s="2" t="inlineStr">
+        <is>
+          <t>624448</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-04
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE75"/>
+  <dimension ref="A1:AE76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12247,6 +12247,163 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>27103750284.53926</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>381391980.63071656</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>78478</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>381230825.1762616</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>20280893240.571213</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>497994</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>1829</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>70181</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>332946</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>1001828</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>775.71000003699</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>63616.752334878</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>287205.4686740062</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>981859.0860935487</t>
+        </is>
+      </c>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q76" s="2" t="inlineStr">
+        <is>
+          <t>370349671.66000015</t>
+        </is>
+      </c>
+      <c r="R76" s="2" t="inlineStr">
+        <is>
+          <t>1538988834.4999998</t>
+        </is>
+      </c>
+      <c r="S76" s="2" t="inlineStr">
+        <is>
+          <t>4224769416.919999</t>
+        </is>
+      </c>
+      <c r="T76" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U76" s="2" t="inlineStr">
+        <is>
+          <t>4291</t>
+        </is>
+      </c>
+      <c r="V76" s="2" t="inlineStr">
+        <is>
+          <t>17526</t>
+        </is>
+      </c>
+      <c r="W76" s="2" t="inlineStr">
+        <is>
+          <t>46408</t>
+        </is>
+      </c>
+      <c r="X76" s="2" t="inlineStr">
+        <is>
+          <t>202550.82</t>
+        </is>
+      </c>
+      <c r="Y76" s="2" t="inlineStr">
+        <is>
+          <t>111964568.5900001</t>
+        </is>
+      </c>
+      <c r="Z76" s="2" t="inlineStr">
+        <is>
+          <t>472668673.9464683</t>
+        </is>
+      </c>
+      <c r="AA76" s="2" t="inlineStr">
+        <is>
+          <t>1255525450.3113344</t>
+        </is>
+      </c>
+      <c r="AB76" s="2" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="AC76" s="2" t="inlineStr">
+        <is>
+          <t>56670</t>
+        </is>
+      </c>
+      <c r="AD76" s="2" t="inlineStr">
+        <is>
+          <t>223173</t>
+        </is>
+      </c>
+      <c r="AE76" s="2" t="inlineStr">
+        <is>
+          <t>627082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-05
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE76"/>
+  <dimension ref="A1:AE77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12404,6 +12404,163 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>27100479903.050747</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>380728641.4604612</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>78495</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>380350571.3577482</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>20272544625.456734</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>497995</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>70567</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>323185</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>998525</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>121.077333353568</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>60269.85833480577</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>277695.61167384085</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>981200.1617602403</t>
+        </is>
+      </c>
+      <c r="P77" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q77" s="2" t="inlineStr">
+        <is>
+          <t>310040416.8000002</t>
+        </is>
+      </c>
+      <c r="R77" s="2" t="inlineStr">
+        <is>
+          <t>1471123039.8899996</t>
+        </is>
+      </c>
+      <c r="S77" s="2" t="inlineStr">
+        <is>
+          <t>4224710595.4899993</t>
+        </is>
+      </c>
+      <c r="T77" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U77" s="2" t="inlineStr">
+        <is>
+          <t>3590</t>
+        </is>
+      </c>
+      <c r="V77" s="2" t="inlineStr">
+        <is>
+          <t>16772</t>
+        </is>
+      </c>
+      <c r="W77" s="2" t="inlineStr">
+        <is>
+          <t>46407</t>
+        </is>
+      </c>
+      <c r="X77" s="2" t="inlineStr">
+        <is>
+          <t>1791198.48</t>
+        </is>
+      </c>
+      <c r="Y77" s="2" t="inlineStr">
+        <is>
+          <t>109233901.01000012</t>
+        </is>
+      </c>
+      <c r="Z77" s="2" t="inlineStr">
+        <is>
+          <t>457036125.8126251</t>
+        </is>
+      </c>
+      <c r="AA77" s="2" t="inlineStr">
+        <is>
+          <t>1255792821.7413344</t>
+        </is>
+      </c>
+      <c r="AB77" s="2" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="AC77" s="2" t="inlineStr">
+        <is>
+          <t>55779</t>
+        </is>
+      </c>
+      <c r="AD77" s="2" t="inlineStr">
+        <is>
+          <t>222504</t>
+        </is>
+      </c>
+      <c r="AE77" s="2" t="inlineStr">
+        <is>
+          <t>627768</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-06
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE77"/>
+  <dimension ref="A1:AE78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12561,6 +12561,163 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>27099086199.29406</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>381089677.1580897</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>78523</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>380971760.13106066</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>20272488833.282146</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>497998</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>2526</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>65243</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>318323</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>989809</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>267.128000039112</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>59687.77800145587</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>268284.1443403138</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>973755.621093547</t>
+        </is>
+      </c>
+      <c r="P78" s="2" t="inlineStr">
+        <is>
+          <t>19237.3</t>
+        </is>
+      </c>
+      <c r="Q78" s="2" t="inlineStr">
+        <is>
+          <t>309977802.47000015</t>
+        </is>
+      </c>
+      <c r="R78" s="2" t="inlineStr">
+        <is>
+          <t>1416794508.1799998</t>
+        </is>
+      </c>
+      <c r="S78" s="2" t="inlineStr">
+        <is>
+          <t>4224455171.4299994</t>
+        </is>
+      </c>
+      <c r="T78" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U78" s="2" t="inlineStr">
+        <is>
+          <t>3591</t>
+        </is>
+      </c>
+      <c r="V78" s="2" t="inlineStr">
+        <is>
+          <t>16157</t>
+        </is>
+      </c>
+      <c r="W78" s="2" t="inlineStr">
+        <is>
+          <t>46406</t>
+        </is>
+      </c>
+      <c r="X78" s="2" t="inlineStr">
+        <is>
+          <t>242083.53000000003</t>
+        </is>
+      </c>
+      <c r="Y78" s="2" t="inlineStr">
+        <is>
+          <t>108223743.22000012</t>
+        </is>
+      </c>
+      <c r="Z78" s="2" t="inlineStr">
+        <is>
+          <t>444873878.67262506</t>
+        </is>
+      </c>
+      <c r="AA78" s="2" t="inlineStr">
+        <is>
+          <t>1248042733.5613344</t>
+        </is>
+      </c>
+      <c r="AB78" s="2" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="AC78" s="2" t="inlineStr">
+        <is>
+          <t>54983</t>
+        </is>
+      </c>
+      <c r="AD78" s="2" t="inlineStr">
+        <is>
+          <t>221251</t>
+        </is>
+      </c>
+      <c r="AE78" s="2" t="inlineStr">
+        <is>
+          <t>628300</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-07
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE78"/>
+  <dimension ref="A1:AE79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12718,6 +12718,163 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>27224975046.96354</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>383221360.96577114</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>78547</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>383194129.30053914</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>20376950816.39623</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>499852</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>9971</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>59212</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>320774</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>984389</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>3180.840000149432</t>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>58524.4360013885</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>273101.4973402718</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>969109.2190934919</t>
+        </is>
+      </c>
+      <c r="P79" s="2" t="inlineStr">
+        <is>
+          <t>121706871.07999991</t>
+        </is>
+      </c>
+      <c r="Q79" s="2" t="inlineStr">
+        <is>
+          <t>310313039.39000016</t>
+        </is>
+      </c>
+      <c r="R79" s="2" t="inlineStr">
+        <is>
+          <t>1364151846.3099997</t>
+        </is>
+      </c>
+      <c r="S79" s="2" t="inlineStr">
+        <is>
+          <t>4137018970.1999993</t>
+        </is>
+      </c>
+      <c r="T79" s="2" t="inlineStr">
+        <is>
+          <t>1377</t>
+        </is>
+      </c>
+      <c r="U79" s="2" t="inlineStr">
+        <is>
+          <t>3592</t>
+        </is>
+      </c>
+      <c r="V79" s="2" t="inlineStr">
+        <is>
+          <t>15584</t>
+        </is>
+      </c>
+      <c r="W79" s="2" t="inlineStr">
+        <is>
+          <t>45445</t>
+        </is>
+      </c>
+      <c r="X79" s="2" t="inlineStr">
+        <is>
+          <t>12878837.220000003</t>
+        </is>
+      </c>
+      <c r="Y79" s="2" t="inlineStr">
+        <is>
+          <t>107857976.23000014</t>
+        </is>
+      </c>
+      <c r="Z79" s="2" t="inlineStr">
+        <is>
+          <t>448864742.052625</t>
+        </is>
+      </c>
+      <c r="AA79" s="2" t="inlineStr">
+        <is>
+          <t>1248417952.0313344</t>
+        </is>
+      </c>
+      <c r="AB79" s="2" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
+      <c r="AC79" s="2" t="inlineStr">
+        <is>
+          <t>56346</t>
+        </is>
+      </c>
+      <c r="AD79" s="2" t="inlineStr">
+        <is>
+          <t>221866</t>
+        </is>
+      </c>
+      <c r="AE79" s="2" t="inlineStr">
+        <is>
+          <t>630211</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-08
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE79"/>
+  <dimension ref="A1:AE80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12875,6 +12875,163 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>25329280844.327854</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>1739487613.3590474</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>78569</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>1739167527.0151184</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 500</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 500</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>6278</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>60358</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>326920</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>988550</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>57255.013001443556</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>282951.6493404541</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>968077.3330936164</t>
+        </is>
+      </c>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q80" s="2" t="inlineStr">
+        <is>
+          <t>330159435.2799999</t>
+        </is>
+      </c>
+      <c r="R80" s="2" t="inlineStr">
+        <is>
+          <t>1485991856.5999997</t>
+        </is>
+      </c>
+      <c r="S80" s="2" t="inlineStr">
+        <is>
+          <t>4207017285.319999</t>
+        </is>
+      </c>
+      <c r="T80" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U80" s="2" t="inlineStr">
+        <is>
+          <t>3749</t>
+        </is>
+      </c>
+      <c r="V80" s="2" t="inlineStr">
+        <is>
+          <t>16963</t>
+        </is>
+      </c>
+      <c r="W80" s="2" t="inlineStr">
+        <is>
+          <t>46288</t>
+        </is>
+      </c>
+      <c r="X80" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Y80" s="2" t="inlineStr">
+        <is>
+          <t>106508895.91000003</t>
+        </is>
+      </c>
+      <c r="Z80" s="2" t="inlineStr">
+        <is>
+          <t>466863055.192625</t>
+        </is>
+      </c>
+      <c r="AA80" s="2" t="inlineStr">
+        <is>
+          <t>1256970891.8278956</t>
+        </is>
+      </c>
+      <c r="AB80" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="AC80" s="2" t="inlineStr">
+        <is>
+          <t>55306</t>
+        </is>
+      </c>
+      <c r="AD80" s="2" t="inlineStr">
+        <is>
+          <t>222529</t>
+        </is>
+      </c>
+      <c r="AE80" s="2" t="inlineStr">
+        <is>
+          <t>630492</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-09
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE80"/>
+  <dimension ref="A1:AE81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13032,6 +13032,163 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>25421101718.376057</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>1760677850.7923367</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>78624</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>1752775925.6313236</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>20253621525.360012</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>333776</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>6805</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>53691</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>325085</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>990995</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>2384.125333441496</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>58836.25266807266</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>284613.1310071722</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>969672.2647603616</t>
+        </is>
+      </c>
+      <c r="P81" s="2" t="inlineStr">
+        <is>
+          <t>81199253.24999997</t>
+        </is>
+      </c>
+      <c r="Q81" s="2" t="inlineStr">
+        <is>
+          <t>338232734.23999995</t>
+        </is>
+      </c>
+      <c r="R81" s="2" t="inlineStr">
+        <is>
+          <t>1553340232.0499997</t>
+        </is>
+      </c>
+      <c r="S81" s="2" t="inlineStr">
+        <is>
+          <t>4224139799.9299994</t>
+        </is>
+      </c>
+      <c r="T81" s="2" t="inlineStr">
+        <is>
+          <t>867</t>
+        </is>
+      </c>
+      <c r="U81" s="2" t="inlineStr">
+        <is>
+          <t>3803</t>
+        </is>
+      </c>
+      <c r="V81" s="2" t="inlineStr">
+        <is>
+          <t>17714</t>
+        </is>
+      </c>
+      <c r="W81" s="2" t="inlineStr">
+        <is>
+          <t>46529</t>
+        </is>
+      </c>
+      <c r="X81" s="2" t="inlineStr">
+        <is>
+          <t>965188.9800000007</t>
+        </is>
+      </c>
+      <c r="Y81" s="2" t="inlineStr">
+        <is>
+          <t>95669998.56000005</t>
+        </is>
+      </c>
+      <c r="Z81" s="2" t="inlineStr">
+        <is>
+          <t>458016780.42262506</t>
+        </is>
+      </c>
+      <c r="AA81" s="2" t="inlineStr">
+        <is>
+          <t>1255028295.7578957</t>
+        </is>
+      </c>
+      <c r="AB81" s="2" t="inlineStr">
+        <is>
+          <t>283</t>
+        </is>
+      </c>
+      <c r="AC81" s="2" t="inlineStr">
+        <is>
+          <t>52302</t>
+        </is>
+      </c>
+      <c r="AD81" s="2" t="inlineStr">
+        <is>
+          <t>223520</t>
+        </is>
+      </c>
+      <c r="AE81" s="2" t="inlineStr">
+        <is>
+          <t>631318</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-10
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE81"/>
+  <dimension ref="A1:AE82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13189,6 +13189,163 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>25521631751.48163</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>1751773709.8546863</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>78655</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>1751658335.1422892</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>20329183588.990005</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>334909</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>6872</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>57352</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>324317</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>996976</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>2509.611000123744</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>55602.76466802952</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>283752.8650072112</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>968605.3440938586</t>
+        </is>
+      </c>
+      <c r="P82" s="2" t="inlineStr">
+        <is>
+          <t>81588162.26000008</t>
+        </is>
+      </c>
+      <c r="Q82" s="2" t="inlineStr">
+        <is>
+          <t>324710381.6699999</t>
+        </is>
+      </c>
+      <c r="R82" s="2" t="inlineStr">
+        <is>
+          <t>1513552796.8899999</t>
+        </is>
+      </c>
+      <c r="S82" s="2" t="inlineStr">
+        <is>
+          <t>4265572539.439999</t>
+        </is>
+      </c>
+      <c r="T82" s="2" t="inlineStr">
+        <is>
+          <t>971</t>
+        </is>
+      </c>
+      <c r="U82" s="2" t="inlineStr">
+        <is>
+          <t>3632</t>
+        </is>
+      </c>
+      <c r="V82" s="2" t="inlineStr">
+        <is>
+          <t>17294</t>
+        </is>
+      </c>
+      <c r="W82" s="2" t="inlineStr">
+        <is>
+          <t>46972</t>
+        </is>
+      </c>
+      <c r="X82" s="2" t="inlineStr">
+        <is>
+          <t>985877.9499999998</t>
+        </is>
+      </c>
+      <c r="Y82" s="2" t="inlineStr">
+        <is>
+          <t>86933756.19999994</t>
+        </is>
+      </c>
+      <c r="Z82" s="2" t="inlineStr">
+        <is>
+          <t>442499857.49262494</t>
+        </is>
+      </c>
+      <c r="AA82" s="2" t="inlineStr">
+        <is>
+          <t>1255091923.3578959</t>
+        </is>
+      </c>
+      <c r="AB82" s="2" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="AC82" s="2" t="inlineStr">
+        <is>
+          <t>50931</t>
+        </is>
+      </c>
+      <c r="AD82" s="2" t="inlineStr">
+        <is>
+          <t>224328</t>
+        </is>
+      </c>
+      <c r="AE82" s="2" t="inlineStr">
+        <is>
+          <t>631788</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-11
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE82"/>
+  <dimension ref="A1:AE83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13346,6 +13346,163 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>25555374407.167973</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>1754406308.1598217</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>78688</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>1753005120.1486158</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>20379004907.83004</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>335747</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>5265</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>65638</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>322499</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>1005318</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>1628.008000079864</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>57443.95766798996</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>279650.56534029206</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>971952.9777605799</t>
+        </is>
+      </c>
+      <c r="P83" s="2" t="inlineStr">
+        <is>
+          <t>54167393.02000001</t>
+        </is>
+      </c>
+      <c r="Q83" s="2" t="inlineStr">
+        <is>
+          <t>354385984.75</t>
+        </is>
+      </c>
+      <c r="R83" s="2" t="inlineStr">
+        <is>
+          <t>1526016042.7099998</t>
+        </is>
+      </c>
+      <c r="S83" s="2" t="inlineStr">
+        <is>
+          <t>4309240978.61</t>
+        </is>
+      </c>
+      <c r="T83" s="2" t="inlineStr">
+        <is>
+          <t>633</t>
+        </is>
+      </c>
+      <c r="U83" s="2" t="inlineStr">
+        <is>
+          <t>3981</t>
+        </is>
+      </c>
+      <c r="V83" s="2" t="inlineStr">
+        <is>
+          <t>17483</t>
+        </is>
+      </c>
+      <c r="W83" s="2" t="inlineStr">
+        <is>
+          <t>47535</t>
+        </is>
+      </c>
+      <c r="X83" s="2" t="inlineStr">
+        <is>
+          <t>808048.2099999997</t>
+        </is>
+      </c>
+      <c r="Y83" s="2" t="inlineStr">
+        <is>
+          <t>90021325.5899999</t>
+        </is>
+      </c>
+      <c r="Z83" s="2" t="inlineStr">
+        <is>
+          <t>435377939.7226249</t>
+        </is>
+      </c>
+      <c r="AA83" s="2" t="inlineStr">
+        <is>
+          <t>1262672223.0178957</t>
+        </is>
+      </c>
+      <c r="AB83" s="2" t="inlineStr">
+        <is>
+          <t>172</t>
+        </is>
+      </c>
+      <c r="AC83" s="2" t="inlineStr">
+        <is>
+          <t>51147</t>
+        </is>
+      </c>
+      <c r="AD83" s="2" t="inlineStr">
+        <is>
+          <t>225446</t>
+        </is>
+      </c>
+      <c r="AE83" s="2" t="inlineStr">
+        <is>
+          <t>634451</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-12
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE83"/>
+  <dimension ref="A1:AE84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13503,6 +13503,163 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>25556360282.214172</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>1760884180.4982843</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>78719</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>1760868509.6605492</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>20375636033.609993</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>335711</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>1369</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>70294</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>317329</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>1004975</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>204.522666685928</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>60447.69366804455</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>271523.7753400468</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>973359.1447606465</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q84" s="2" t="inlineStr">
+        <is>
+          <t>408637325.88</t>
+        </is>
+      </c>
+      <c r="R84" s="2" t="inlineStr">
+        <is>
+          <t>1514524180.84</t>
+        </is>
+      </c>
+      <c r="S84" s="2" t="inlineStr">
+        <is>
+          <t>4363440013.9</t>
+        </is>
+      </c>
+      <c r="T84" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U84" s="2" t="inlineStr">
+        <is>
+          <t>4614</t>
+        </is>
+      </c>
+      <c r="V84" s="2" t="inlineStr">
+        <is>
+          <t>17369</t>
+        </is>
+      </c>
+      <c r="W84" s="2" t="inlineStr">
+        <is>
+          <t>48167</t>
+        </is>
+      </c>
+      <c r="X84" s="2" t="inlineStr">
+        <is>
+          <t>592521.5399999999</t>
+        </is>
+      </c>
+      <c r="Y84" s="2" t="inlineStr">
+        <is>
+          <t>91204359.6899999</t>
+        </is>
+      </c>
+      <c r="Z84" s="2" t="inlineStr">
+        <is>
+          <t>421717914.9226249</t>
+        </is>
+      </c>
+      <c r="AA84" s="2" t="inlineStr">
+        <is>
+          <t>1263718056.8978958</t>
+        </is>
+      </c>
+      <c r="AB84" s="2" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="AC84" s="2" t="inlineStr">
+        <is>
+          <t>51422</t>
+        </is>
+      </c>
+      <c r="AD84" s="2" t="inlineStr">
+        <is>
+          <t>225185</t>
+        </is>
+      </c>
+      <c r="AE84" s="2" t="inlineStr">
+        <is>
+          <t>635129</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-13
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE84"/>
+  <dimension ref="A1:AE85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13660,6 +13660,163 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>25531293362.665104</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>1761575137.260809</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>78746</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>1761561884.8794649</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>20348374192.059963</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>335316</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>1974</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>66787</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>313156</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>994818</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>267.558666702754</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>60739.12833471211</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>260754.71267315643</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>962504.2700939259</t>
+        </is>
+      </c>
+      <c r="P85" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q85" s="2" t="inlineStr">
+        <is>
+          <t>408689094.25</t>
+        </is>
+      </c>
+      <c r="R85" s="2" t="inlineStr">
+        <is>
+          <t>1459107142.6499999</t>
+        </is>
+      </c>
+      <c r="S85" s="2" t="inlineStr">
+        <is>
+          <t>4363334209.469999</t>
+        </is>
+      </c>
+      <c r="T85" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U85" s="2" t="inlineStr">
+        <is>
+          <t>4614</t>
+        </is>
+      </c>
+      <c r="V85" s="2" t="inlineStr">
+        <is>
+          <t>16750</t>
+        </is>
+      </c>
+      <c r="W85" s="2" t="inlineStr">
+        <is>
+          <t>48167</t>
+        </is>
+      </c>
+      <c r="X85" s="2" t="inlineStr">
+        <is>
+          <t>617405.23</t>
+        </is>
+      </c>
+      <c r="Y85" s="2" t="inlineStr">
+        <is>
+          <t>90632390.56999987</t>
+        </is>
+      </c>
+      <c r="Z85" s="2" t="inlineStr">
+        <is>
+          <t>405544009.2956257</t>
+        </is>
+      </c>
+      <c r="AA85" s="2" t="inlineStr">
+        <is>
+          <t>1253914975.5178957</t>
+        </is>
+      </c>
+      <c r="AB85" s="2" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="AC85" s="2" t="inlineStr">
+        <is>
+          <t>51570</t>
+        </is>
+      </c>
+      <c r="AD85" s="2" t="inlineStr">
+        <is>
+          <t>224020</t>
+        </is>
+      </c>
+      <c r="AE85" s="2" t="inlineStr">
+        <is>
+          <t>636003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-14
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE85"/>
+  <dimension ref="A1:AE86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13817,6 +13817,163 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>25729007146.07762</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>1805198875.3392935</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>78784</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>1796753784.8044493</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>20436181701.810013</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>336510</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>8149</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>60030</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>316066</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>990564</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>2702.721000097683</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>59715.752334750105</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>264057.35133981466</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>956296.8154272097</t>
+        </is>
+      </c>
+      <c r="P86" s="2" t="inlineStr">
+        <is>
+          <t>118010906.42000002</t>
+        </is>
+      </c>
+      <c r="Q86" s="2" t="inlineStr">
+        <is>
+          <t>407028483.48</t>
+        </is>
+      </c>
+      <c r="R86" s="2" t="inlineStr">
+        <is>
+          <t>1409730299.07</t>
+        </is>
+      </c>
+      <c r="S86" s="2" t="inlineStr">
+        <is>
+          <t>4264101178.1599994</t>
+        </is>
+      </c>
+      <c r="T86" s="2" t="inlineStr">
+        <is>
+          <t>1373</t>
+        </is>
+      </c>
+      <c r="U86" s="2" t="inlineStr">
+        <is>
+          <t>4610</t>
+        </is>
+      </c>
+      <c r="V86" s="2" t="inlineStr">
+        <is>
+          <t>16167</t>
+        </is>
+      </c>
+      <c r="W86" s="2" t="inlineStr">
+        <is>
+          <t>47099</t>
+        </is>
+      </c>
+      <c r="X86" s="2" t="inlineStr">
+        <is>
+          <t>3801444.7000000016</t>
+        </is>
+      </c>
+      <c r="Y86" s="2" t="inlineStr">
+        <is>
+          <t>90977432.08999985</t>
+        </is>
+      </c>
+      <c r="Z86" s="2" t="inlineStr">
+        <is>
+          <t>410656361.53562564</t>
+        </is>
+      </c>
+      <c r="AA86" s="2" t="inlineStr">
+        <is>
+          <t>1251018849.2178957</t>
+        </is>
+      </c>
+      <c r="AB86" s="2" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="AC86" s="2" t="inlineStr">
+        <is>
+          <t>51143</t>
+        </is>
+      </c>
+      <c r="AD86" s="2" t="inlineStr">
+        <is>
+          <t>224403</t>
+        </is>
+      </c>
+      <c r="AE86" s="2" t="inlineStr">
+        <is>
+          <t>636980</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-15
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE86"/>
+  <dimension ref="A1:AE87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13974,6 +13974,163 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>25773518758.97997</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>1782225765.554186</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>78825</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>1782181310.695702</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>20481670222.290016</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>337217</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>5379</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>62837</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>323163</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>993790</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>2378.05500008583</t>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>64006.44833480512</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>277896.47734005976</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>952830.3414273398</t>
+        </is>
+      </c>
+      <c r="P87" s="2" t="inlineStr">
+        <is>
+          <t>62452804.32000003</t>
+        </is>
+      </c>
+      <c r="Q87" s="2" t="inlineStr">
+        <is>
+          <t>403251498.37</t>
+        </is>
+      </c>
+      <c r="R87" s="2" t="inlineStr">
+        <is>
+          <t>1527795442.2499998</t>
+        </is>
+      </c>
+      <c r="S87" s="2" t="inlineStr">
+        <is>
+          <t>4327686332.779999</t>
+        </is>
+      </c>
+      <c r="T87" s="2" t="inlineStr">
+        <is>
+          <t>707</t>
+        </is>
+      </c>
+      <c r="U87" s="2" t="inlineStr">
+        <is>
+          <t>4605</t>
+        </is>
+      </c>
+      <c r="V87" s="2" t="inlineStr">
+        <is>
+          <t>17541</t>
+        </is>
+      </c>
+      <c r="W87" s="2" t="inlineStr">
+        <is>
+          <t>47950</t>
+        </is>
+      </c>
+      <c r="X87" s="2" t="inlineStr">
+        <is>
+          <t>1493681.5900000003</t>
+        </is>
+      </c>
+      <c r="Y87" s="2" t="inlineStr">
+        <is>
+          <t>80798811.89999992</t>
+        </is>
+      </c>
+      <c r="Z87" s="2" t="inlineStr">
+        <is>
+          <t>418249493.75562567</t>
+        </is>
+      </c>
+      <c r="AA87" s="2" t="inlineStr">
+        <is>
+          <t>1252146491.1078959</t>
+        </is>
+      </c>
+      <c r="AB87" s="2" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="AC87" s="2" t="inlineStr">
+        <is>
+          <t>51502</t>
+        </is>
+      </c>
+      <c r="AD87" s="2" t="inlineStr">
+        <is>
+          <t>224993</t>
+        </is>
+      </c>
+      <c r="AE87" s="2" t="inlineStr">
+        <is>
+          <t>636139</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-16
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE87"/>
+  <dimension ref="A1:AE88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14131,6 +14131,163 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>25842653026.448963</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>1803326564.079765</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>78861</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>1803049548.883315</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>20552143491.930023</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>338293</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>6333</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>61925</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>320430</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>995120</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>2167.592000098776</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>60863.65933482108</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>277763.7023401092</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>948589.2310940475</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>74916552.18000008</t>
+        </is>
+      </c>
+      <c r="Q88" s="2" t="inlineStr">
+        <is>
+          <t>398190022.89000005</t>
+        </is>
+      </c>
+      <c r="R88" s="2" t="inlineStr">
+        <is>
+          <t>1590181028.82</t>
+        </is>
+      </c>
+      <c r="S88" s="2" t="inlineStr">
+        <is>
+          <t>4341389532.629999</t>
+        </is>
+      </c>
+      <c r="T88" s="2" t="inlineStr">
+        <is>
+          <t>883</t>
+        </is>
+      </c>
+      <c r="U88" s="2" t="inlineStr">
+        <is>
+          <t>4560</t>
+        </is>
+      </c>
+      <c r="V88" s="2" t="inlineStr">
+        <is>
+          <t>18245</t>
+        </is>
+      </c>
+      <c r="W88" s="2" t="inlineStr">
+        <is>
+          <t>48124</t>
+        </is>
+      </c>
+      <c r="X88" s="2" t="inlineStr">
+        <is>
+          <t>1154079.9099999997</t>
+        </is>
+      </c>
+      <c r="Y88" s="2" t="inlineStr">
+        <is>
+          <t>84581293.17999992</t>
+        </is>
+      </c>
+      <c r="Z88" s="2" t="inlineStr">
+        <is>
+          <t>421819468.9356257</t>
+        </is>
+      </c>
+      <c r="AA88" s="2" t="inlineStr">
+        <is>
+          <t>1254048716.9127283</t>
+        </is>
+      </c>
+      <c r="AB88" s="2" t="inlineStr">
+        <is>
+          <t>302</t>
+        </is>
+      </c>
+      <c r="AC88" s="2" t="inlineStr">
+        <is>
+          <t>53207</t>
+        </is>
+      </c>
+      <c r="AD88" s="2" t="inlineStr">
+        <is>
+          <t>226225</t>
+        </is>
+      </c>
+      <c r="AE88" s="2" t="inlineStr">
+        <is>
+          <t>638405</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-17
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE88"/>
+  <dimension ref="A1:AE89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14288,6 +14288,163 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>25883522489.071564</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>1793504440.3002703</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>78903</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>1793492952.2689662</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>20579835723.149994</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>338673</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>4576</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>62491</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>318512</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>1001560</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>2008.792000075072</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>62479.64600144928</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>277987.27567346755</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>949150.0270941379</t>
+        </is>
+      </c>
+      <c r="P89" s="2" t="inlineStr">
+        <is>
+          <t>51018553.47999998</t>
+        </is>
+      </c>
+      <c r="Q89" s="2" t="inlineStr">
+        <is>
+          <t>392061327.45</t>
+        </is>
+      </c>
+      <c r="R89" s="2" t="inlineStr">
+        <is>
+          <t>1566044837.3899999</t>
+        </is>
+      </c>
+      <c r="S89" s="2" t="inlineStr">
+        <is>
+          <t>4365265842.319999</t>
+        </is>
+      </c>
+      <c r="T89" s="2" t="inlineStr">
+        <is>
+          <t>592</t>
+        </is>
+      </c>
+      <c r="U89" s="2" t="inlineStr">
+        <is>
+          <t>4579</t>
+        </is>
+      </c>
+      <c r="V89" s="2" t="inlineStr">
+        <is>
+          <t>18012</t>
+        </is>
+      </c>
+      <c r="W89" s="2" t="inlineStr">
+        <is>
+          <t>48483</t>
+        </is>
+      </c>
+      <c r="X89" s="2" t="inlineStr">
+        <is>
+          <t>687435.9100000001</t>
+        </is>
+      </c>
+      <c r="Y89" s="2" t="inlineStr">
+        <is>
+          <t>85245054.85999995</t>
+        </is>
+      </c>
+      <c r="Z89" s="2" t="inlineStr">
+        <is>
+          <t>422326935.4356257</t>
+        </is>
+      </c>
+      <c r="AA89" s="2" t="inlineStr">
+        <is>
+          <t>1252893212.9627283</t>
+        </is>
+      </c>
+      <c r="AB89" s="2" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="AC89" s="2" t="inlineStr">
+        <is>
+          <t>53702</t>
+        </is>
+      </c>
+      <c r="AD89" s="2" t="inlineStr">
+        <is>
+          <t>227246</t>
+        </is>
+      </c>
+      <c r="AE89" s="2" t="inlineStr">
+        <is>
+          <t>638471</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-18
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE89"/>
+  <dimension ref="A1:AE90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14445,6 +14445,163 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>25962138702.605747</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>1807026370.9424837</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>78929</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>1807001401.3775177</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>20622230290.510033</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>339482</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>5192</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>67057</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>317294</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>1010200</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>1683.706666718928</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>66780.7846681698</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>279797.27300678374</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>956276.1380942471</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>63425619.99000006</t>
+        </is>
+      </c>
+      <c r="Q90" s="2" t="inlineStr">
+        <is>
+          <t>361276312.1899999</t>
+        </is>
+      </c>
+      <c r="R90" s="2" t="inlineStr">
+        <is>
+          <t>1549629611.03</t>
+        </is>
+      </c>
+      <c r="S90" s="2" t="inlineStr">
+        <is>
+          <t>4370182692.579999</t>
+        </is>
+      </c>
+      <c r="T90" s="2" t="inlineStr">
+        <is>
+          <t>781</t>
+        </is>
+      </c>
+      <c r="U90" s="2" t="inlineStr">
+        <is>
+          <t>4201</t>
+        </is>
+      </c>
+      <c r="V90" s="2" t="inlineStr">
+        <is>
+          <t>17820</t>
+        </is>
+      </c>
+      <c r="W90" s="2" t="inlineStr">
+        <is>
+          <t>48610</t>
+        </is>
+      </c>
+      <c r="X90" s="2" t="inlineStr">
+        <is>
+          <t>595431.1799999999</t>
+        </is>
+      </c>
+      <c r="Y90" s="2" t="inlineStr">
+        <is>
+          <t>85738514.16000003</t>
+        </is>
+      </c>
+      <c r="Z90" s="2" t="inlineStr">
+        <is>
+          <t>423298254.2556257</t>
+        </is>
+      </c>
+      <c r="AA90" s="2" t="inlineStr">
+        <is>
+          <t>1258497413.7627282</t>
+        </is>
+      </c>
+      <c r="AB90" s="2" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="AC90" s="2" t="inlineStr">
+        <is>
+          <t>54877</t>
+        </is>
+      </c>
+      <c r="AD90" s="2" t="inlineStr">
+        <is>
+          <t>228464</t>
+        </is>
+      </c>
+      <c r="AE90" s="2" t="inlineStr">
+        <is>
+          <t>641272</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-19
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE90"/>
+  <dimension ref="A1:AE91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14602,6 +14602,163 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>25948631606.128986</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>1800644080.128978</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>78946</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>1800234537.853929</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>20617861460.39999</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>339452</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>1379</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>71592</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>315792</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>1011046</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>166.757333361816</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>66922.88333484739</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>272319.1903399531</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>958070.825760966</t>
+        </is>
+      </c>
+      <c r="P91" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q91" s="2" t="inlineStr">
+        <is>
+          <t>370445516.04999995</t>
+        </is>
+      </c>
+      <c r="R91" s="2" t="inlineStr">
+        <is>
+          <t>1537701772.21</t>
+        </is>
+      </c>
+      <c r="S91" s="2" t="inlineStr">
+        <is>
+          <t>4433608312.569999</t>
+        </is>
+      </c>
+      <c r="T91" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U91" s="2" t="inlineStr">
+        <is>
+          <t>4348</t>
+        </is>
+      </c>
+      <c r="V91" s="2" t="inlineStr">
+        <is>
+          <t>17761</t>
+        </is>
+      </c>
+      <c r="W91" s="2" t="inlineStr">
+        <is>
+          <t>49391</t>
+        </is>
+      </c>
+      <c r="X91" s="2" t="inlineStr">
+        <is>
+          <t>163979.52000000005</t>
+        </is>
+      </c>
+      <c r="Y91" s="2" t="inlineStr">
+        <is>
+          <t>87498845.87000003</t>
+        </is>
+      </c>
+      <c r="Z91" s="2" t="inlineStr">
+        <is>
+          <t>419610886.6805516</t>
+        </is>
+      </c>
+      <c r="AA91" s="2" t="inlineStr">
+        <is>
+          <t>1262340817.3827283</t>
+        </is>
+      </c>
+      <c r="AB91" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="AC91" s="2" t="inlineStr">
+        <is>
+          <t>55986</t>
+        </is>
+      </c>
+      <c r="AD91" s="2" t="inlineStr">
+        <is>
+          <t>227875</t>
+        </is>
+      </c>
+      <c r="AE91" s="2" t="inlineStr">
+        <is>
+          <t>644147</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-20
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE91"/>
+  <dimension ref="A1:AE92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14759,6 +14759,163 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>25962549549.084007</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>1819668580.3321004</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>78975</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>1816681785.6883953</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>20615233531.420002</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>339423</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>1491</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>68234</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>315576</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>1000152</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>201.704000021816</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>67101.79800152384</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>267939.14233976754</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>949390.3844276265</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q92" s="2" t="inlineStr">
+        <is>
+          <t>370350102.67999995</t>
+        </is>
+      </c>
+      <c r="R92" s="2" t="inlineStr">
+        <is>
+          <t>1484491745.85</t>
+        </is>
+      </c>
+      <c r="S92" s="2" t="inlineStr">
+        <is>
+          <t>4433569448.279999</t>
+        </is>
+      </c>
+      <c r="T92" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U92" s="2" t="inlineStr">
+        <is>
+          <t>4346</t>
+        </is>
+      </c>
+      <c r="V92" s="2" t="inlineStr">
+        <is>
+          <t>17118</t>
+        </is>
+      </c>
+      <c r="W92" s="2" t="inlineStr">
+        <is>
+          <t>49389</t>
+        </is>
+      </c>
+      <c r="X92" s="2" t="inlineStr">
+        <is>
+          <t>326697.33999999997</t>
+        </is>
+      </c>
+      <c r="Y92" s="2" t="inlineStr">
+        <is>
+          <t>85723267.03000005</t>
+        </is>
+      </c>
+      <c r="Z92" s="2" t="inlineStr">
+        <is>
+          <t>414957186.1205516</t>
+        </is>
+      </c>
+      <c r="AA92" s="2" t="inlineStr">
+        <is>
+          <t>1253324218.0727284</t>
+        </is>
+      </c>
+      <c r="AB92" s="2" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="AC92" s="2" t="inlineStr">
+        <is>
+          <t>54488</t>
+        </is>
+      </c>
+      <c r="AD92" s="2" t="inlineStr">
+        <is>
+          <t>226910</t>
+        </is>
+      </c>
+      <c r="AE92" s="2" t="inlineStr">
+        <is>
+          <t>642668</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-21
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE92"/>
+  <dimension ref="A1:AE93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14916,6 +14916,163 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>26110998695.776688</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>1825578282.2560942</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>79015</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>1824689220.3103082</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>20772359323.03998</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>344015</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>8199</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>60331</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>319671</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>995306</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>3378.300000140106</t>
+        </is>
+      </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>67860.41666818704</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>273017.2210065006</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>938179.1874275708</t>
+        </is>
+      </c>
+      <c r="P93" s="2" t="inlineStr">
+        <is>
+          <t>121256582.59999986</t>
+        </is>
+      </c>
+      <c r="Q93" s="2" t="inlineStr">
+        <is>
+          <t>370458607.3899999</t>
+        </is>
+      </c>
+      <c r="R93" s="2" t="inlineStr">
+        <is>
+          <t>1484725203.7199998</t>
+        </is>
+      </c>
+      <c r="S93" s="2" t="inlineStr">
+        <is>
+          <t>4340404336.389999</t>
+        </is>
+      </c>
+      <c r="T93" s="2" t="inlineStr">
+        <is>
+          <t>1441</t>
+        </is>
+      </c>
+      <c r="U93" s="2" t="inlineStr">
+        <is>
+          <t>4352</t>
+        </is>
+      </c>
+      <c r="V93" s="2" t="inlineStr">
+        <is>
+          <t>17125</t>
+        </is>
+      </c>
+      <c r="W93" s="2" t="inlineStr">
+        <is>
+          <t>48440</t>
+        </is>
+      </c>
+      <c r="X93" s="2" t="inlineStr">
+        <is>
+          <t>1054288.0799999996</t>
+        </is>
+      </c>
+      <c r="Y93" s="2" t="inlineStr">
+        <is>
+          <t>90202259.72000003</t>
+        </is>
+      </c>
+      <c r="Z93" s="2" t="inlineStr">
+        <is>
+          <t>424705329.2905515</t>
+        </is>
+      </c>
+      <c r="AA93" s="2" t="inlineStr">
+        <is>
+          <t>1257550276.0527284</t>
+        </is>
+      </c>
+      <c r="AB93" s="2" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="AC93" s="2" t="inlineStr">
+        <is>
+          <t>55403</t>
+        </is>
+      </c>
+      <c r="AD93" s="2" t="inlineStr">
+        <is>
+          <t>227529</t>
+        </is>
+      </c>
+      <c r="AE93" s="2" t="inlineStr">
+        <is>
+          <t>644805</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-22
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE93"/>
+  <dimension ref="A1:AE94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15073,6 +15073,163 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>26308648215.15519</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>1819519848.7853594</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>79054</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>1819198533.6427743</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>20940792515.890007</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>350657</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>9630</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>66620</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>331379</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>1000880</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>38092.44666699404</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>86322.27733496607</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>305354.8766735264</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>956339.2814278551</t>
+        </is>
+      </c>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>64120526.69000003</t>
+        </is>
+      </c>
+      <c r="Q94" s="2" t="inlineStr">
+        <is>
+          <t>373766329.9499999</t>
+        </is>
+      </c>
+      <c r="R94" s="2" t="inlineStr">
+        <is>
+          <t>1606091899.34</t>
+        </is>
+      </c>
+      <c r="S94" s="2" t="inlineStr">
+        <is>
+          <t>4412398260.619999</t>
+        </is>
+      </c>
+      <c r="T94" s="2" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="U94" s="2" t="inlineStr">
+        <is>
+          <t>4421</t>
+        </is>
+      </c>
+      <c r="V94" s="2" t="inlineStr">
+        <is>
+          <t>18568</t>
+        </is>
+      </c>
+      <c r="W94" s="2" t="inlineStr">
+        <is>
+          <t>49347</t>
+        </is>
+      </c>
+      <c r="X94" s="2" t="inlineStr">
+        <is>
+          <t>932884.0700000001</t>
+        </is>
+      </c>
+      <c r="Y94" s="2" t="inlineStr">
+        <is>
+          <t>98337395.92000009</t>
+        </is>
+      </c>
+      <c r="Z94" s="2" t="inlineStr">
+        <is>
+          <t>441896063.2705516</t>
+        </is>
+      </c>
+      <c r="AA94" s="2" t="inlineStr">
+        <is>
+          <t>1264557383.9827285</t>
+        </is>
+      </c>
+      <c r="AB94" s="2" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="AC94" s="2" t="inlineStr">
+        <is>
+          <t>55275</t>
+        </is>
+      </c>
+      <c r="AD94" s="2" t="inlineStr">
+        <is>
+          <t>228320</t>
+        </is>
+      </c>
+      <c r="AE94" s="2" t="inlineStr">
+        <is>
+          <t>644837</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-23
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE94"/>
+  <dimension ref="A1:AE95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15230,6 +15230,163 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>26369869294.871487</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>1861870072.3390176</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>79099</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>1859600013.2070706</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>21021054795.419994</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>352491</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>5726</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>69997</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>331789</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>1004239</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>2098.86400008684</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>121117.35833516094</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>340586.92367380456</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>984375.7017614468</t>
+        </is>
+      </c>
+      <c r="P95" s="2" t="inlineStr">
+        <is>
+          <t>66351271.970000006</t>
+        </is>
+      </c>
+      <c r="Q95" s="2" t="inlineStr">
+        <is>
+          <t>375386176.25999993</t>
+        </is>
+      </c>
+      <c r="R95" s="2" t="inlineStr">
+        <is>
+          <t>1670091099.53</t>
+        </is>
+      </c>
+      <c r="S95" s="2" t="inlineStr">
+        <is>
+          <t>4411725086.779999</t>
+        </is>
+      </c>
+      <c r="T95" s="2" t="inlineStr">
+        <is>
+          <t>735</t>
+        </is>
+      </c>
+      <c r="U95" s="2" t="inlineStr">
+        <is>
+          <t>4454</t>
+        </is>
+      </c>
+      <c r="V95" s="2" t="inlineStr">
+        <is>
+          <t>19306</t>
+        </is>
+      </c>
+      <c r="W95" s="2" t="inlineStr">
+        <is>
+          <t>49480</t>
+        </is>
+      </c>
+      <c r="X95" s="2" t="inlineStr">
+        <is>
+          <t>1653056.2300000002</t>
+        </is>
+      </c>
+      <c r="Y95" s="2" t="inlineStr">
+        <is>
+          <t>94951333.5100001</t>
+        </is>
+      </c>
+      <c r="Z95" s="2" t="inlineStr">
+        <is>
+          <t>445215516.8205516</t>
+        </is>
+      </c>
+      <c r="AA95" s="2" t="inlineStr">
+        <is>
+          <t>1256817138.0927284</t>
+        </is>
+      </c>
+      <c r="AB95" s="2" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="AC95" s="2" t="inlineStr">
+        <is>
+          <t>54025</t>
+        </is>
+      </c>
+      <c r="AD95" s="2" t="inlineStr">
+        <is>
+          <t>229319</t>
+        </is>
+      </c>
+      <c r="AE95" s="2" t="inlineStr">
+        <is>
+          <t>645633</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-24
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE95"/>
+  <dimension ref="A1:AE96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15387,6 +15387,163 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>26418186167.016285</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>1849831291.6771133</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>79134</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>1848175388.2214854</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>21045970134.249958</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>352801</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>4872</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>70974</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>329424</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>1009722</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>1911.378666740552</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>119179.88900180317</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>334432.49500703654</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>979750.3617615263</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>56160724.99000004</t>
+        </is>
+      </c>
+      <c r="Q96" s="2" t="inlineStr">
+        <is>
+          <t>366808240.9200001</t>
+        </is>
+      </c>
+      <c r="R96" s="2" t="inlineStr">
+        <is>
+          <t>1625724855.55</t>
+        </is>
+      </c>
+      <c r="S96" s="2" t="inlineStr">
+        <is>
+          <t>4428422031.5199995</t>
+        </is>
+      </c>
+      <c r="T96" s="2" t="inlineStr">
+        <is>
+          <t>623</t>
+        </is>
+      </c>
+      <c r="U96" s="2" t="inlineStr">
+        <is>
+          <t>4307</t>
+        </is>
+      </c>
+      <c r="V96" s="2" t="inlineStr">
+        <is>
+          <t>18806</t>
+        </is>
+      </c>
+      <c r="W96" s="2" t="inlineStr">
+        <is>
+          <t>49672</t>
+        </is>
+      </c>
+      <c r="X96" s="2" t="inlineStr">
+        <is>
+          <t>858648.4100000001</t>
+        </is>
+      </c>
+      <c r="Y96" s="2" t="inlineStr">
+        <is>
+          <t>107513664.53000021</t>
+        </is>
+      </c>
+      <c r="Z96" s="2" t="inlineStr">
+        <is>
+          <t>450250243.91000015</t>
+        </is>
+      </c>
+      <c r="AA96" s="2" t="inlineStr">
+        <is>
+          <t>1270662684.9027286</t>
+        </is>
+      </c>
+      <c r="AB96" s="2" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="AC96" s="2" t="inlineStr">
+        <is>
+          <t>54222</t>
+        </is>
+      </c>
+      <c r="AD96" s="2" t="inlineStr">
+        <is>
+          <t>230223</t>
+        </is>
+      </c>
+      <c r="AE96" s="2" t="inlineStr">
+        <is>
+          <t>646383</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-25
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE96"/>
+  <dimension ref="A1:AE97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15544,6 +15544,163 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>26401894836.871403</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>1755949256.8800576</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>79181</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>1755682838.2551556</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>21091804587.620007</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>353408</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>4961</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>74498</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>321599</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>1016625</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>2662.78800008412</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>117714.7073351331</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>331098.15100690624</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>984082.7247616432</t>
+        </is>
+      </c>
+      <c r="P97" s="2" t="inlineStr">
+        <is>
+          <t>52036967.930000044</t>
+        </is>
+      </c>
+      <c r="Q97" s="2" t="inlineStr">
+        <is>
+          <t>371947286.00000006</t>
+        </is>
+      </c>
+      <c r="R97" s="2" t="inlineStr">
+        <is>
+          <t>1610745048.86</t>
+        </is>
+      </c>
+      <c r="S97" s="2" t="inlineStr">
+        <is>
+          <t>4436936046.829999</t>
+        </is>
+      </c>
+      <c r="T97" s="2" t="inlineStr">
+        <is>
+          <t>587</t>
+        </is>
+      </c>
+      <c r="U97" s="2" t="inlineStr">
+        <is>
+          <t>4339</t>
+        </is>
+      </c>
+      <c r="V97" s="2" t="inlineStr">
+        <is>
+          <t>18638</t>
+        </is>
+      </c>
+      <c r="W97" s="2" t="inlineStr">
+        <is>
+          <t>49760</t>
+        </is>
+      </c>
+      <c r="X97" s="2" t="inlineStr">
+        <is>
+          <t>1466183.4200000006</t>
+        </is>
+      </c>
+      <c r="Y97" s="2" t="inlineStr">
+        <is>
+          <t>111363719.90271434</t>
+        </is>
+      </c>
+      <c r="Z97" s="2" t="inlineStr">
+        <is>
+          <t>451245961.9327143</t>
+        </is>
+      </c>
+      <c r="AA97" s="2" t="inlineStr">
+        <is>
+          <t>1282331185.1654427</t>
+        </is>
+      </c>
+      <c r="AB97" s="2" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="AC97" s="2" t="inlineStr">
+        <is>
+          <t>53972</t>
+        </is>
+      </c>
+      <c r="AD97" s="2" t="inlineStr">
+        <is>
+          <t>231774</t>
+        </is>
+      </c>
+      <c r="AE97" s="2" t="inlineStr">
+        <is>
+          <t>649537</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-26
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE97"/>
+  <dimension ref="A1:AE98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15701,6 +15701,163 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>26369905457.333923</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>1750422917.6571834</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>79207</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>1749901498.2549794</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>21087692760.37996</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>353372</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>1396</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>78707</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>315826</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>1015012</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>224.101333353576</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>118461.7980017948</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>322831.82633995207</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>984816.456095053</t>
+        </is>
+      </c>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q98" s="2" t="inlineStr">
+        <is>
+          <t>360563978.99</t>
+        </is>
+      </c>
+      <c r="R98" s="2" t="inlineStr">
+        <is>
+          <t>1574544383.61</t>
+        </is>
+      </c>
+      <c r="S98" s="2" t="inlineStr">
+        <is>
+          <t>4488978359.809999</t>
+        </is>
+      </c>
+      <c r="T98" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U98" s="2" t="inlineStr">
+        <is>
+          <t>4146</t>
+        </is>
+      </c>
+      <c r="V98" s="2" t="inlineStr">
+        <is>
+          <t>18187</t>
+        </is>
+      </c>
+      <c r="W98" s="2" t="inlineStr">
+        <is>
+          <t>50348</t>
+        </is>
+      </c>
+      <c r="X98" s="2" t="inlineStr">
+        <is>
+          <t>754551.3400000003</t>
+        </is>
+      </c>
+      <c r="Y98" s="2" t="inlineStr">
+        <is>
+          <t>110477008.07271433</t>
+        </is>
+      </c>
+      <c r="Z98" s="2" t="inlineStr">
+        <is>
+          <t>446009069.25271434</t>
+        </is>
+      </c>
+      <c r="AA98" s="2" t="inlineStr">
+        <is>
+          <t>1283423474.9454427</t>
+        </is>
+      </c>
+      <c r="AB98" s="2" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="AC98" s="2" t="inlineStr">
+        <is>
+          <t>52399</t>
+        </is>
+      </c>
+      <c r="AD98" s="2" t="inlineStr">
+        <is>
+          <t>231474</t>
+        </is>
+      </c>
+      <c r="AE98" s="2" t="inlineStr">
+        <is>
+          <t>649862</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-27
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE98"/>
+  <dimension ref="A1:AE99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15858,6 +15858,163 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>26389668426.72856</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>1752195454.2576227</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>79242</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>1751314452.5687478</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>21082635232.29997</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>353333</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>2198</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>74715</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>311313</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>1002302</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>465.975000048339</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>118704.82700179561</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>313507.60433974327</t>
+        </is>
+      </c>
+      <c r="O99" s="2" t="inlineStr">
+        <is>
+          <t>970299.1250949982</t>
+        </is>
+      </c>
+      <c r="P99" s="2" t="inlineStr">
+        <is>
+          <t>7000.0</t>
+        </is>
+      </c>
+      <c r="Q99" s="2" t="inlineStr">
+        <is>
+          <t>360563978.99</t>
+        </is>
+      </c>
+      <c r="R99" s="2" t="inlineStr">
+        <is>
+          <t>1510001567.5800002</t>
+        </is>
+      </c>
+      <c r="S99" s="2" t="inlineStr">
+        <is>
+          <t>4488964380.4</t>
+        </is>
+      </c>
+      <c r="T99" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U99" s="2" t="inlineStr">
+        <is>
+          <t>4146</t>
+        </is>
+      </c>
+      <c r="V99" s="2" t="inlineStr">
+        <is>
+          <t>17400</t>
+        </is>
+      </c>
+      <c r="W99" s="2" t="inlineStr">
+        <is>
+          <t>50347</t>
+        </is>
+      </c>
+      <c r="X99" s="2" t="inlineStr">
+        <is>
+          <t>484599.0300000001</t>
+        </is>
+      </c>
+      <c r="Y99" s="2" t="inlineStr">
+        <is>
+          <t>114050512.42271434</t>
+        </is>
+      </c>
+      <c r="Z99" s="2" t="inlineStr">
+        <is>
+          <t>416047129.7627144</t>
+        </is>
+      </c>
+      <c r="AA99" s="2" t="inlineStr">
+        <is>
+          <t>1275134353.5754428</t>
+        </is>
+      </c>
+      <c r="AB99" s="2" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="AC99" s="2" t="inlineStr">
+        <is>
+          <t>54323</t>
+        </is>
+      </c>
+      <c r="AD99" s="2" t="inlineStr">
+        <is>
+          <t>230245</t>
+        </is>
+      </c>
+      <c r="AE99" s="2" t="inlineStr">
+        <is>
+          <t>650770</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-28
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE99"/>
+  <dimension ref="A1:AE100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16015,6 +16015,163 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>26535192720.40093</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>1765966407.4965937</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>79280</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>1765801907.7197077</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>21201738447.939983</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>355165</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>9226</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>64281</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>316012</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>997628</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>2881.092000134097</t>
+        </is>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>123049.7723351682</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>322076.3303397804</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>960480.4730949367</t>
+        </is>
+      </c>
+      <c r="P100" s="2" t="inlineStr">
+        <is>
+          <t>131511422.94</t>
+        </is>
+      </c>
+      <c r="Q100" s="2" t="inlineStr">
+        <is>
+          <t>360844452.99</t>
+        </is>
+      </c>
+      <c r="R100" s="2" t="inlineStr">
+        <is>
+          <t>1450201169.5900002</t>
+        </is>
+      </c>
+      <c r="S100" s="2" t="inlineStr">
+        <is>
+          <t>4378543701.889999</t>
+        </is>
+      </c>
+      <c r="T100" s="2" t="inlineStr">
+        <is>
+          <t>1524</t>
+        </is>
+      </c>
+      <c r="U100" s="2" t="inlineStr">
+        <is>
+          <t>4146</t>
+        </is>
+      </c>
+      <c r="V100" s="2" t="inlineStr">
+        <is>
+          <t>16705</t>
+        </is>
+      </c>
+      <c r="W100" s="2" t="inlineStr">
+        <is>
+          <t>49211</t>
+        </is>
+      </c>
+      <c r="X100" s="2" t="inlineStr">
+        <is>
+          <t>1184116.5799999996</t>
+        </is>
+      </c>
+      <c r="Y100" s="2" t="inlineStr">
+        <is>
+          <t>115463757.5027143</t>
+        </is>
+      </c>
+      <c r="Z100" s="2" t="inlineStr">
+        <is>
+          <t>425758046.07271427</t>
+        </is>
+      </c>
+      <c r="AA100" s="2" t="inlineStr">
+        <is>
+          <t>1271664527.1435642</t>
+        </is>
+      </c>
+      <c r="AB100" s="2" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="AC100" s="2" t="inlineStr">
+        <is>
+          <t>54076</t>
+        </is>
+      </c>
+      <c r="AD100" s="2" t="inlineStr">
+        <is>
+          <t>230613</t>
+        </is>
+      </c>
+      <c r="AE100" s="2" t="inlineStr">
+        <is>
+          <t>651150</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-29
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE100"/>
+  <dimension ref="A1:AE101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16172,6 +16172,163 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>26580029676.86933</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>1756683316.571522</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>79322</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>1756643955.3622012</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>21259151250.829975</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>355908</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>6071</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>63739</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>323384</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>998290</t>
+        </is>
+      </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>2568.469333419368</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>102867.73266838679</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>334304.3783400228</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>956794.3460950651</t>
+        </is>
+      </c>
+      <c r="P101" s="2" t="inlineStr">
+        <is>
+          <t>76286978.93999983</t>
+        </is>
+      </c>
+      <c r="Q101" s="2" t="inlineStr">
+        <is>
+          <t>370973008.19000006</t>
+        </is>
+      </c>
+      <c r="R101" s="2" t="inlineStr">
+        <is>
+          <t>1581606333.2</t>
+        </is>
+      </c>
+      <c r="S101" s="2" t="inlineStr">
+        <is>
+          <t>4454422768.41</t>
+        </is>
+      </c>
+      <c r="T101" s="2" t="inlineStr">
+        <is>
+          <t>814</t>
+        </is>
+      </c>
+      <c r="U101" s="2" t="inlineStr">
+        <is>
+          <t>4226</t>
+        </is>
+      </c>
+      <c r="V101" s="2" t="inlineStr">
+        <is>
+          <t>18228</t>
+        </is>
+      </c>
+      <c r="W101" s="2" t="inlineStr">
+        <is>
+          <t>50164</t>
+        </is>
+      </c>
+      <c r="X101" s="2" t="inlineStr">
+        <is>
+          <t>709424.32</t>
+        </is>
+      </c>
+      <c r="Y101" s="2" t="inlineStr">
+        <is>
+          <t>111321143.32271416</t>
+        </is>
+      </c>
+      <c r="Z101" s="2" t="inlineStr">
+        <is>
+          <t>435519694.3027142</t>
+        </is>
+      </c>
+      <c r="AA101" s="2" t="inlineStr">
+        <is>
+          <t>1271166530.1835644</t>
+        </is>
+      </c>
+      <c r="AB101" s="2" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="AC101" s="2" t="inlineStr">
+        <is>
+          <t>55326</t>
+        </is>
+      </c>
+      <c r="AD101" s="2" t="inlineStr">
+        <is>
+          <t>231103</t>
+        </is>
+      </c>
+      <c r="AE101" s="2" t="inlineStr">
+        <is>
+          <t>653722</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-30
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE101"/>
+  <dimension ref="A1:AE102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16329,6 +16329,163 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>26634737940.430027</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>1772736979.8263218</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>79350</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>1771547922.8916128</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>21328402378.820007</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>356929</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>6803</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>63636</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>323776</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>998352</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>1588.028000062218</t>
+        </is>
+      </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>67933.40166815343</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>333363.9143400271</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>944792.566095075</t>
+        </is>
+      </c>
+      <c r="P102" s="2" t="inlineStr">
+        <is>
+          <t>79579568.16999997</t>
+        </is>
+      </c>
+      <c r="Q102" s="2" t="inlineStr">
+        <is>
+          <t>383169524.0999999</t>
+        </is>
+      </c>
+      <c r="R102" s="2" t="inlineStr">
+        <is>
+          <t>1656473048.79</t>
+        </is>
+      </c>
+      <c r="S102" s="2" t="inlineStr">
+        <is>
+          <t>4474841059.869999</t>
+        </is>
+      </c>
+      <c r="T102" s="2" t="inlineStr">
+        <is>
+          <t>920</t>
+        </is>
+      </c>
+      <c r="U102" s="2" t="inlineStr">
+        <is>
+          <t>4299</t>
+        </is>
+      </c>
+      <c r="V102" s="2" t="inlineStr">
+        <is>
+          <t>19039</t>
+        </is>
+      </c>
+      <c r="W102" s="2" t="inlineStr">
+        <is>
+          <t>50405</t>
+        </is>
+      </c>
+      <c r="X102" s="2" t="inlineStr">
+        <is>
+          <t>1526777.6099999999</t>
+        </is>
+      </c>
+      <c r="Y102" s="2" t="inlineStr">
+        <is>
+          <t>113676215.58271411</t>
+        </is>
+      </c>
+      <c r="Z102" s="2" t="inlineStr">
+        <is>
+          <t>438596252.7027142</t>
+        </is>
+      </c>
+      <c r="AA102" s="2" t="inlineStr">
+        <is>
+          <t>1275093632.5761278</t>
+        </is>
+      </c>
+      <c r="AB102" s="2" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="AC102" s="2" t="inlineStr">
+        <is>
+          <t>54102</t>
+        </is>
+      </c>
+      <c r="AD102" s="2" t="inlineStr">
+        <is>
+          <t>232055</t>
+        </is>
+      </c>
+      <c r="AE102" s="2" t="inlineStr">
+        <is>
+          <t>653796</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-07-31
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE102"/>
+  <dimension ref="A1:AE103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16486,6 +16486,163 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>26602346505.48905</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>1636259949.3529809</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>79390</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>1635788259.1337688</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>21365205723.850025</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>357531</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>6319</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>66879</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>325839</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>1013063</t>
+        </is>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>2417.472000079064</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>69278.17500148976</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>331886.46400672663</t>
+        </is>
+      </c>
+      <c r="O103" s="2" t="inlineStr">
+        <is>
+          <t>936411.0113548733</t>
+        </is>
+      </c>
+      <c r="P103" s="2" t="inlineStr">
+        <is>
+          <t>61277444.56000001</t>
+        </is>
+      </c>
+      <c r="Q103" s="2" t="inlineStr">
+        <is>
+          <t>396708620.1599998</t>
+        </is>
+      </c>
+      <c r="R103" s="2" t="inlineStr">
+        <is>
+          <t>1634499032.9199996</t>
+        </is>
+      </c>
+      <c r="S103" s="2" t="inlineStr">
+        <is>
+          <t>4508752849.2699995</t>
+        </is>
+      </c>
+      <c r="T103" s="2" t="inlineStr">
+        <is>
+          <t>703</t>
+        </is>
+      </c>
+      <c r="U103" s="2" t="inlineStr">
+        <is>
+          <t>4484</t>
+        </is>
+      </c>
+      <c r="V103" s="2" t="inlineStr">
+        <is>
+          <t>18740</t>
+        </is>
+      </c>
+      <c r="W103" s="2" t="inlineStr">
+        <is>
+          <t>50794</t>
+        </is>
+      </c>
+      <c r="X103" s="2" t="inlineStr">
+        <is>
+          <t>1100713.2799999998</t>
+        </is>
+      </c>
+      <c r="Y103" s="2" t="inlineStr">
+        <is>
+          <t>111786910.41771406</t>
+        </is>
+      </c>
+      <c r="Z103" s="2" t="inlineStr">
+        <is>
+          <t>436645239.14771426</t>
+        </is>
+      </c>
+      <c r="AA103" s="2" t="inlineStr">
+        <is>
+          <t>1275219120.1211276</t>
+        </is>
+      </c>
+      <c r="AB103" s="2" t="inlineStr">
+        <is>
+          <t>253</t>
+        </is>
+      </c>
+      <c r="AC103" s="2" t="inlineStr">
+        <is>
+          <t>53448</t>
+        </is>
+      </c>
+      <c r="AD103" s="2" t="inlineStr">
+        <is>
+          <t>232433</t>
+        </is>
+      </c>
+      <c r="AE103" s="2" t="inlineStr">
+        <is>
+          <t>651871</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-01
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE103"/>
+  <dimension ref="A1:AE104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16643,6 +16643,163 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>26647444286.090122</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>1621038706.1574051</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>79426</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>1620356991.3869731</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>21412724053.22</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>358197</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>4853</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>72643</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>320185</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t>1016963</t>
+        </is>
+      </c>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>1896.578666726664</t>
+        </is>
+      </c>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>67637.02000145617</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>330933.4366733553</t>
+        </is>
+      </c>
+      <c r="O104" s="2" t="inlineStr">
+        <is>
+          <t>936769.4157599701</t>
+        </is>
+      </c>
+      <c r="P104" s="2" t="inlineStr">
+        <is>
+          <t>59791977.73000002</t>
+        </is>
+      </c>
+      <c r="Q104" s="2" t="inlineStr">
+        <is>
+          <t>401719140.7899998</t>
+        </is>
+      </c>
+      <c r="R104" s="2" t="inlineStr">
+        <is>
+          <t>1636312887.8899996</t>
+        </is>
+      </c>
+      <c r="S104" s="2" t="inlineStr">
+        <is>
+          <t>4515831931.48</t>
+        </is>
+      </c>
+      <c r="T104" s="2" t="inlineStr">
+        <is>
+          <t>695</t>
+        </is>
+      </c>
+      <c r="U104" s="2" t="inlineStr">
+        <is>
+          <t>4563</t>
+        </is>
+      </c>
+      <c r="V104" s="2" t="inlineStr">
+        <is>
+          <t>18745</t>
+        </is>
+      </c>
+      <c r="W104" s="2" t="inlineStr">
+        <is>
+          <t>50918</t>
+        </is>
+      </c>
+      <c r="X104" s="2" t="inlineStr">
+        <is>
+          <t>945351.07</t>
+        </is>
+      </c>
+      <c r="Y104" s="2" t="inlineStr">
+        <is>
+          <t>110288486.7649999</t>
+        </is>
+      </c>
+      <c r="Z104" s="2" t="inlineStr">
+        <is>
+          <t>429504694.15771425</t>
+        </is>
+      </c>
+      <c r="AA104" s="2" t="inlineStr">
+        <is>
+          <t>1282441285.6011276</t>
+        </is>
+      </c>
+      <c r="AB104" s="2" t="inlineStr">
+        <is>
+          <t>265</t>
+        </is>
+      </c>
+      <c r="AC104" s="2" t="inlineStr">
+        <is>
+          <t>47812</t>
+        </is>
+      </c>
+      <c r="AD104" s="2" t="inlineStr">
+        <is>
+          <t>224993</t>
+        </is>
+      </c>
+      <c r="AE104" s="2" t="inlineStr">
+        <is>
+          <t>647593</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-02
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE104"/>
+  <dimension ref="A1:AE105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16800,6 +16800,163 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>26646709585.57293</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>1626107739.6788275</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>79455</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>1623792428.2791767</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>21407976347.979984</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>358211</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>1948</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>76684</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>317816</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>1019533</t>
+        </is>
+      </c>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>219.160000034152</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>66242.6656680724</t>
+        </is>
+      </c>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
+          <t>320592.51967309916</t>
+        </is>
+      </c>
+      <c r="O105" s="2" t="inlineStr">
+        <is>
+          <t>934623.7142019025</t>
+        </is>
+      </c>
+      <c r="P105" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q105" s="2" t="inlineStr">
+        <is>
+          <t>409478368.8699999</t>
+        </is>
+      </c>
+      <c r="R105" s="2" t="inlineStr">
+        <is>
+          <t>1601392823.1299999</t>
+        </is>
+      </c>
+      <c r="S105" s="2" t="inlineStr">
+        <is>
+          <t>4575633472.539999</t>
+        </is>
+      </c>
+      <c r="T105" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U105" s="2" t="inlineStr">
+        <is>
+          <t>4671</t>
+        </is>
+      </c>
+      <c r="V105" s="2" t="inlineStr">
+        <is>
+          <t>18403</t>
+        </is>
+      </c>
+      <c r="W105" s="2" t="inlineStr">
+        <is>
+          <t>51614</t>
+        </is>
+      </c>
+      <c r="X105" s="2" t="inlineStr">
+        <is>
+          <t>663806.03</t>
+        </is>
+      </c>
+      <c r="Y105" s="2" t="inlineStr">
+        <is>
+          <t>112286554.87499985</t>
+        </is>
+      </c>
+      <c r="Z105" s="2" t="inlineStr">
+        <is>
+          <t>418462041.0577141</t>
+        </is>
+      </c>
+      <c r="AA105" s="2" t="inlineStr">
+        <is>
+          <t>1286861876.0611277</t>
+        </is>
+      </c>
+      <c r="AB105" s="2" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="AC105" s="2" t="inlineStr">
+        <is>
+          <t>51508</t>
+        </is>
+      </c>
+      <c r="AD105" s="2" t="inlineStr">
+        <is>
+          <t>225810</t>
+        </is>
+      </c>
+      <c r="AE105" s="2" t="inlineStr">
+        <is>
+          <t>651098</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-03
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE105"/>
+  <dimension ref="A1:AE106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16957,6 +16957,163 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>26625389511.93637</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>1631179571.9252896</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>79483</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>1629178477.8457415</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>21391113580.819996</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>357977</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>2591</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>72870</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>318315</t>
+        </is>
+      </c>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>1000596</t>
+        </is>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>304.285333375527</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>65899.3800014137</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>315790.23200627894</t>
+        </is>
+      </c>
+      <c r="O106" s="2" t="inlineStr">
+        <is>
+          <t>921196.6530214102</t>
+        </is>
+      </c>
+      <c r="P106" s="2" t="inlineStr">
+        <is>
+          <t>55391.96000000001</t>
+        </is>
+      </c>
+      <c r="Q106" s="2" t="inlineStr">
+        <is>
+          <t>409589583.0599999</t>
+        </is>
+      </c>
+      <c r="R106" s="2" t="inlineStr">
+        <is>
+          <t>1549241478.9799998</t>
+        </is>
+      </c>
+      <c r="S106" s="2" t="inlineStr">
+        <is>
+          <t>4575602328.749999</t>
+        </is>
+      </c>
+      <c r="T106" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U106" s="2" t="inlineStr">
+        <is>
+          <t>4674</t>
+        </is>
+      </c>
+      <c r="V106" s="2" t="inlineStr">
+        <is>
+          <t>17783</t>
+        </is>
+      </c>
+      <c r="W106" s="2" t="inlineStr">
+        <is>
+          <t>51613</t>
+        </is>
+      </c>
+      <c r="X106" s="2" t="inlineStr">
+        <is>
+          <t>1036669.7200000006</t>
+        </is>
+      </c>
+      <c r="Y106" s="2" t="inlineStr">
+        <is>
+          <t>112244107.82499982</t>
+        </is>
+      </c>
+      <c r="Z106" s="2" t="inlineStr">
+        <is>
+          <t>416326668.9977141</t>
+        </is>
+      </c>
+      <c r="AA106" s="2" t="inlineStr">
+        <is>
+          <t>1272403294.7023802</t>
+        </is>
+      </c>
+      <c r="AB106" s="2" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="AC106" s="2" t="inlineStr">
+        <is>
+          <t>52495</t>
+        </is>
+      </c>
+      <c r="AD106" s="2" t="inlineStr">
+        <is>
+          <t>226070</t>
+        </is>
+      </c>
+      <c r="AE106" s="2" t="inlineStr">
+        <is>
+          <t>653213</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-04
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE106"/>
+  <dimension ref="A1:AE107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17114,6 +17114,163 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>26795362288.0904</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>1645242420.9698215</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>79523</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>1644176039.3121784</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>21516892101.869995</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>359612</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>8822</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>65910</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>324051</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>996571</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>2509.80800011492</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>62191.62133470763</t>
+        </is>
+      </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>323998.09333968227</t>
+        </is>
+      </c>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t>909371.5833546564</t>
+        </is>
+      </c>
+      <c r="P107" s="2" t="inlineStr">
+        <is>
+          <t>131384452.4599999</t>
+        </is>
+      </c>
+      <c r="Q107" s="2" t="inlineStr">
+        <is>
+          <t>410950483.14999986</t>
+        </is>
+      </c>
+      <c r="R107" s="2" t="inlineStr">
+        <is>
+          <t>1551111235.9399998</t>
+        </is>
+      </c>
+      <c r="S107" s="2" t="inlineStr">
+        <is>
+          <t>4470253353.2</t>
+        </is>
+      </c>
+      <c r="T107" s="2" t="inlineStr">
+        <is>
+          <t>1494</t>
+        </is>
+      </c>
+      <c r="U107" s="2" t="inlineStr">
+        <is>
+          <t>4674</t>
+        </is>
+      </c>
+      <c r="V107" s="2" t="inlineStr">
+        <is>
+          <t>17789</t>
+        </is>
+      </c>
+      <c r="W107" s="2" t="inlineStr">
+        <is>
+          <t>50413</t>
+        </is>
+      </c>
+      <c r="X107" s="2" t="inlineStr">
+        <is>
+          <t>1572836.7399999995</t>
+        </is>
+      </c>
+      <c r="Y107" s="2" t="inlineStr">
+        <is>
+          <t>115739168.18499988</t>
+        </is>
+      </c>
+      <c r="Z107" s="2" t="inlineStr">
+        <is>
+          <t>432263313.24771404</t>
+        </is>
+      </c>
+      <c r="AA107" s="2" t="inlineStr">
+        <is>
+          <t>1280014180.8923802</t>
+        </is>
+      </c>
+      <c r="AB107" s="2" t="inlineStr">
+        <is>
+          <t>269</t>
+        </is>
+      </c>
+      <c r="AC107" s="2" t="inlineStr">
+        <is>
+          <t>52859</t>
+        </is>
+      </c>
+      <c r="AD107" s="2" t="inlineStr">
+        <is>
+          <t>227693</t>
+        </is>
+      </c>
+      <c r="AE107" s="2" t="inlineStr">
+        <is>
+          <t>654842</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-05
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE107"/>
+  <dimension ref="A1:AE108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17271,6 +17271,163 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>26836877846.934532</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>1643948234.8547654</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>79554</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>1643552019.6344132</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>21699310519.73001</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>366087</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>5968</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>67879</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>332443</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>999111</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>2055.258333405172</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>57017.60833461245</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>331634.2086731794</t>
+        </is>
+      </c>
+      <c r="O108" s="2" t="inlineStr">
+        <is>
+          <t>901614.1493546988</t>
+        </is>
+      </c>
+      <c r="P108" s="2" t="inlineStr">
+        <is>
+          <t>68833258.76999997</t>
+        </is>
+      </c>
+      <c r="Q108" s="2" t="inlineStr">
+        <is>
+          <t>411426564.46999985</t>
+        </is>
+      </c>
+      <c r="R108" s="2" t="inlineStr">
+        <is>
+          <t>1683055095.1999998</t>
+        </is>
+      </c>
+      <c r="S108" s="2" t="inlineStr">
+        <is>
+          <t>4543933263.799999</t>
+        </is>
+      </c>
+      <c r="T108" s="2" t="inlineStr">
+        <is>
+          <t>806</t>
+        </is>
+      </c>
+      <c r="U108" s="2" t="inlineStr">
+        <is>
+          <t>4651</t>
+        </is>
+      </c>
+      <c r="V108" s="2" t="inlineStr">
+        <is>
+          <t>19288</t>
+        </is>
+      </c>
+      <c r="W108" s="2" t="inlineStr">
+        <is>
+          <t>51274</t>
+        </is>
+      </c>
+      <c r="X108" s="2" t="inlineStr">
+        <is>
+          <t>1303894.27</t>
+        </is>
+      </c>
+      <c r="Y108" s="2" t="inlineStr">
+        <is>
+          <t>111288262.37499991</t>
+        </is>
+      </c>
+      <c r="Z108" s="2" t="inlineStr">
+        <is>
+          <t>438584213.457714</t>
+        </is>
+      </c>
+      <c r="AA108" s="2" t="inlineStr">
+        <is>
+          <t>1277043542.6723802</t>
+        </is>
+      </c>
+      <c r="AB108" s="2" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="AC108" s="2" t="inlineStr">
+        <is>
+          <t>52143</t>
+        </is>
+      </c>
+      <c r="AD108" s="2" t="inlineStr">
+        <is>
+          <t>228263</t>
+        </is>
+      </c>
+      <c r="AE108" s="2" t="inlineStr">
+        <is>
+          <t>655079</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-06
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE108"/>
+  <dimension ref="A1:AE109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17428,6 +17428,163 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>26947761115.68814</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>1667891213.869032</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>79588</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>1667329314.392559</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>21761551161.639984</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>367049</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>5727</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>66107</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>331588</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>999779</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>2136.082666746888</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>59078.69566798385</t>
+        </is>
+      </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>333918.1740066224</t>
+        </is>
+      </c>
+      <c r="O109" s="2" t="inlineStr">
+        <is>
+          <t>897377.0560214148</t>
+        </is>
+      </c>
+      <c r="P109" s="2" t="inlineStr">
+        <is>
+          <t>67431270.84999992</t>
+        </is>
+      </c>
+      <c r="Q109" s="2" t="inlineStr">
+        <is>
+          <t>404366818.86999995</t>
+        </is>
+      </c>
+      <c r="R109" s="2" t="inlineStr">
+        <is>
+          <t>1750526828.2699997</t>
+        </is>
+      </c>
+      <c r="S109" s="2" t="inlineStr">
+        <is>
+          <t>4548927269.15</t>
+        </is>
+      </c>
+      <c r="T109" s="2" t="inlineStr">
+        <is>
+          <t>793</t>
+        </is>
+      </c>
+      <c r="U109" s="2" t="inlineStr">
+        <is>
+          <t>4645</t>
+        </is>
+      </c>
+      <c r="V109" s="2" t="inlineStr">
+        <is>
+          <t>20092</t>
+        </is>
+      </c>
+      <c r="W109" s="2" t="inlineStr">
+        <is>
+          <t>51374</t>
+        </is>
+      </c>
+      <c r="X109" s="2" t="inlineStr">
+        <is>
+          <t>2125028.1600000006</t>
+        </is>
+      </c>
+      <c r="Y109" s="2" t="inlineStr">
+        <is>
+          <t>107515837.00551961</t>
+        </is>
+      </c>
+      <c r="Z109" s="2" t="inlineStr">
+        <is>
+          <t>438254113.4782337</t>
+        </is>
+      </c>
+      <c r="AA109" s="2" t="inlineStr">
+        <is>
+          <t>1274235482.1128998</t>
+        </is>
+      </c>
+      <c r="AB109" s="2" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="AC109" s="2" t="inlineStr">
+        <is>
+          <t>52501</t>
+        </is>
+      </c>
+      <c r="AD109" s="2" t="inlineStr">
+        <is>
+          <t>228210</t>
+        </is>
+      </c>
+      <c r="AE109" s="2" t="inlineStr">
+        <is>
+          <t>656177</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-07
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE109"/>
+  <dimension ref="A1:AE110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17585,6 +17585,163 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>27006756903.75998</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>1668920686.1108856</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>79611</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>1667194372.3873196</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>21785485451.400005</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>367370</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>3922</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>64628</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>331122</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>1004417</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>2061.690666713976</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>59381.55166794438</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>334013.00267322746</t>
+        </is>
+      </c>
+      <c r="O110" s="2" t="inlineStr">
+        <is>
+          <t>898483.578688001</t>
+        </is>
+      </c>
+      <c r="P110" s="2" t="inlineStr">
+        <is>
+          <t>56053155.279999994</t>
+        </is>
+      </c>
+      <c r="Q110" s="2" t="inlineStr">
+        <is>
+          <t>392841793.43999994</t>
+        </is>
+      </c>
+      <c r="R110" s="2" t="inlineStr">
+        <is>
+          <t>1697181391.0799997</t>
+        </is>
+      </c>
+      <c r="S110" s="2" t="inlineStr">
+        <is>
+          <t>4560812942.15</t>
+        </is>
+      </c>
+      <c r="T110" s="2" t="inlineStr">
+        <is>
+          <t>643</t>
+        </is>
+      </c>
+      <c r="U110" s="2" t="inlineStr">
+        <is>
+          <t>4517</t>
+        </is>
+      </c>
+      <c r="V110" s="2" t="inlineStr">
+        <is>
+          <t>19508</t>
+        </is>
+      </c>
+      <c r="W110" s="2" t="inlineStr">
+        <is>
+          <t>51576</t>
+        </is>
+      </c>
+      <c r="X110" s="2" t="inlineStr">
+        <is>
+          <t>735377.9700000002</t>
+        </is>
+      </c>
+      <c r="Y110" s="2" t="inlineStr">
+        <is>
+          <t>98515254.78051953</t>
+        </is>
+      </c>
+      <c r="Z110" s="2" t="inlineStr">
+        <is>
+          <t>428651598.0182338</t>
+        </is>
+      </c>
+      <c r="AA110" s="2" t="inlineStr">
+        <is>
+          <t>1274079139.6529</t>
+        </is>
+      </c>
+      <c r="AB110" s="2" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="AC110" s="2" t="inlineStr">
+        <is>
+          <t>53295</t>
+        </is>
+      </c>
+      <c r="AD110" s="2" t="inlineStr">
+        <is>
+          <t>230422</t>
+        </is>
+      </c>
+      <c r="AE110" s="2" t="inlineStr">
+        <is>
+          <t>657812</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-08
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE110"/>
+  <dimension ref="A1:AE111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17742,6 +17742,163 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>27046069547.646046</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>1679973533.4178731</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>79635</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>1679938578.221693</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>21796461556.169983</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>367721</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>3513</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>71545</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>332009</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>1014384</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>1426.954666703545</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>60934.56833467845</t>
+        </is>
+      </c>
+      <c r="N111" s="2" t="inlineStr">
+        <is>
+          <t>333031.75233996107</t>
+        </is>
+      </c>
+      <c r="O111" s="2" t="inlineStr">
+        <is>
+          <t>905941.5300214133</t>
+        </is>
+      </c>
+      <c r="P111" s="2" t="inlineStr">
+        <is>
+          <t>53172771.48999998</t>
+        </is>
+      </c>
+      <c r="Q111" s="2" t="inlineStr">
+        <is>
+          <t>387691614.1499999</t>
+        </is>
+      </c>
+      <c r="R111" s="2" t="inlineStr">
+        <is>
+          <t>1685771767.7999997</t>
+        </is>
+      </c>
+      <c r="S111" s="2" t="inlineStr">
+        <is>
+          <t>4568452074.559999</t>
+        </is>
+      </c>
+      <c r="T111" s="2" t="inlineStr">
+        <is>
+          <t>608</t>
+        </is>
+      </c>
+      <c r="U111" s="2" t="inlineStr">
+        <is>
+          <t>4459</t>
+        </is>
+      </c>
+      <c r="V111" s="2" t="inlineStr">
+        <is>
+          <t>19401</t>
+        </is>
+      </c>
+      <c r="W111" s="2" t="inlineStr">
+        <is>
+          <t>51696</t>
+        </is>
+      </c>
+      <c r="X111" s="2" t="inlineStr">
+        <is>
+          <t>758739.2200000001</t>
+        </is>
+      </c>
+      <c r="Y111" s="2" t="inlineStr">
+        <is>
+          <t>100510392.27051951</t>
+        </is>
+      </c>
+      <c r="Z111" s="2" t="inlineStr">
+        <is>
+          <t>434345087.8682337</t>
+        </is>
+      </c>
+      <c r="AA111" s="2" t="inlineStr">
+        <is>
+          <t>1285004822.1128998</t>
+        </is>
+      </c>
+      <c r="AB111" s="2" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="AC111" s="2" t="inlineStr">
+        <is>
+          <t>57741</t>
+        </is>
+      </c>
+      <c r="AD111" s="2" t="inlineStr">
+        <is>
+          <t>230432</t>
+        </is>
+      </c>
+      <c r="AE111" s="2" t="inlineStr">
+        <is>
+          <t>659057</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-09
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE111"/>
+  <dimension ref="A1:AE112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17899,6 +17899,163 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>27038358252.208935</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>1680593209.2189202</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>79659</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>1680581758.2713542</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>21791862261.42001</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>367689</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>315</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>74297</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>326974</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>1012422</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>57.264666668132</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>60993.35200136382</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>325983.1070064334</t>
+        </is>
+      </c>
+      <c r="O112" s="2" t="inlineStr">
+        <is>
+          <t>907626.1206880622</t>
+        </is>
+      </c>
+      <c r="P112" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q112" s="2" t="inlineStr">
+        <is>
+          <t>381062844.5799998</t>
+        </is>
+      </c>
+      <c r="R112" s="2" t="inlineStr">
+        <is>
+          <t>1657745286.0399997</t>
+        </is>
+      </c>
+      <c r="S112" s="2" t="inlineStr">
+        <is>
+          <t>4621568220.379999</t>
+        </is>
+      </c>
+      <c r="T112" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U112" s="2" t="inlineStr">
+        <is>
+          <t>4371</t>
+        </is>
+      </c>
+      <c r="V112" s="2" t="inlineStr">
+        <is>
+          <t>19142</t>
+        </is>
+      </c>
+      <c r="W112" s="2" t="inlineStr">
+        <is>
+          <t>52303</t>
+        </is>
+      </c>
+      <c r="X112" s="2" t="inlineStr">
+        <is>
+          <t>889459.6100000001</t>
+        </is>
+      </c>
+      <c r="Y112" s="2" t="inlineStr">
+        <is>
+          <t>99630166.88051955</t>
+        </is>
+      </c>
+      <c r="Z112" s="2" t="inlineStr">
+        <is>
+          <t>431158451.73823375</t>
+        </is>
+      </c>
+      <c r="AA112" s="2" t="inlineStr">
+        <is>
+          <t>1287978205.5428998</t>
+        </is>
+      </c>
+      <c r="AB112" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="AC112" s="2" t="inlineStr">
+        <is>
+          <t>55613</t>
+        </is>
+      </c>
+      <c r="AD112" s="2" t="inlineStr">
+        <is>
+          <t>230492</t>
+        </is>
+      </c>
+      <c r="AE112" s="2" t="inlineStr">
+        <is>
+          <t>660710</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-10
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE112"/>
+  <dimension ref="A1:AE113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18056,6 +18056,163 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>27057156516.98719</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>1681897923.2227938</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>79685</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>1681834209.7805648</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>21786727961.939964</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>367649</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>380</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>68918</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>322675</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>1000855</t>
+        </is>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>214.850666669648</t>
+        </is>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>60538.07433467427</t>
+        </is>
+      </c>
+      <c r="N113" s="2" t="inlineStr">
+        <is>
+          <t>318884.3486729633</t>
+        </is>
+      </c>
+      <c r="O113" s="2" t="inlineStr">
+        <is>
+          <t>900614.4416878929</t>
+        </is>
+      </c>
+      <c r="P113" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q113" s="2" t="inlineStr">
+        <is>
+          <t>380951630.3899998</t>
+        </is>
+      </c>
+      <c r="R113" s="2" t="inlineStr">
+        <is>
+          <t>1575807124.6199996</t>
+        </is>
+      </c>
+      <c r="S113" s="2" t="inlineStr">
+        <is>
+          <t>4621486437.7699995</t>
+        </is>
+      </c>
+      <c r="T113" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U113" s="2" t="inlineStr">
+        <is>
+          <t>4368</t>
+        </is>
+      </c>
+      <c r="V113" s="2" t="inlineStr">
+        <is>
+          <t>18170</t>
+        </is>
+      </c>
+      <c r="W113" s="2" t="inlineStr">
+        <is>
+          <t>52301</t>
+        </is>
+      </c>
+      <c r="X113" s="2" t="inlineStr">
+        <is>
+          <t>622579.0199999999</t>
+        </is>
+      </c>
+      <c r="Y113" s="2" t="inlineStr">
+        <is>
+          <t>100154476.43051961</t>
+        </is>
+      </c>
+      <c r="Z113" s="2" t="inlineStr">
+        <is>
+          <t>426459819.8382338</t>
+        </is>
+      </c>
+      <c r="AA113" s="2" t="inlineStr">
+        <is>
+          <t>1286270391.4029</t>
+        </is>
+      </c>
+      <c r="AB113" s="2" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="AC113" s="2" t="inlineStr">
+        <is>
+          <t>54855</t>
+        </is>
+      </c>
+      <c r="AD113" s="2" t="inlineStr">
+        <is>
+          <t>229778</t>
+        </is>
+      </c>
+      <c r="AE113" s="2" t="inlineStr">
+        <is>
+          <t>662355</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-11
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE113"/>
+  <dimension ref="A1:AE114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18213,6 +18213,163 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>27178558767.048317</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>1695592766.2497263</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>79706</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>1694950466.8136272</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>21899310572.88004</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>369158</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>7048</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>60361</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>326017</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>994802</t>
+        </is>
+      </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>1853.539333444092</t>
+        </is>
+      </c>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>58284.63866793331</t>
+        </is>
+      </c>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>321835.03833957104</t>
+        </is>
+      </c>
+      <c r="O114" s="2" t="inlineStr">
+        <is>
+          <t>893648.1300209347</t>
+        </is>
+      </c>
+      <c r="P114" s="2" t="inlineStr">
+        <is>
+          <t>128589962.2399998</t>
+        </is>
+      </c>
+      <c r="Q114" s="2" t="inlineStr">
+        <is>
+          <t>380837648.3599998</t>
+        </is>
+      </c>
+      <c r="R114" s="2" t="inlineStr">
+        <is>
+          <t>1523311558.4199996</t>
+        </is>
+      </c>
+      <c r="S114" s="2" t="inlineStr">
+        <is>
+          <t>4511867218.529999</t>
+        </is>
+      </c>
+      <c r="T114" s="2" t="inlineStr">
+        <is>
+          <t>1469</t>
+        </is>
+      </c>
+      <c r="U114" s="2" t="inlineStr">
+        <is>
+          <t>4367</t>
+        </is>
+      </c>
+      <c r="V114" s="2" t="inlineStr">
+        <is>
+          <t>17542</t>
+        </is>
+      </c>
+      <c r="W114" s="2" t="inlineStr">
+        <is>
+          <t>51079</t>
+        </is>
+      </c>
+      <c r="X114" s="2" t="inlineStr">
+        <is>
+          <t>1364986.510000001</t>
+        </is>
+      </c>
+      <c r="Y114" s="2" t="inlineStr">
+        <is>
+          <t>99794622.84051974</t>
+        </is>
+      </c>
+      <c r="Z114" s="2" t="inlineStr">
+        <is>
+          <t>440853576.3982339</t>
+        </is>
+      </c>
+      <c r="AA114" s="2" t="inlineStr">
+        <is>
+          <t>1295726867.1429</t>
+        </is>
+      </c>
+      <c r="AB114" s="2" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
+      <c r="AC114" s="2" t="inlineStr">
+        <is>
+          <t>54731</t>
+        </is>
+      </c>
+      <c r="AD114" s="2" t="inlineStr">
+        <is>
+          <t>231002</t>
+        </is>
+      </c>
+      <c r="AE114" s="2" t="inlineStr">
+        <is>
+          <t>663805</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-12
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE114"/>
+  <dimension ref="A1:AE115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18370,6 +18370,163 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>27322148012.219685</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>1740991373.1657588</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>79733</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>1740979038.5016398</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>21959177457.519993</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>371511</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>5498</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>64936</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>336494</t>
+        </is>
+      </c>
+      <c r="K115" s="2" t="inlineStr">
+        <is>
+          <t>997261</t>
+        </is>
+      </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>2375.674666765576</t>
+        </is>
+      </c>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>61941.93133470413</t>
+        </is>
+      </c>
+      <c r="N115" s="2" t="inlineStr">
+        <is>
+          <t>332837.0116731714</t>
+        </is>
+      </c>
+      <c r="O115" s="2" t="inlineStr">
+        <is>
+          <t>893246.9040209336</t>
+        </is>
+      </c>
+      <c r="P115" s="2" t="inlineStr">
+        <is>
+          <t>78064569.75</t>
+        </is>
+      </c>
+      <c r="Q115" s="2" t="inlineStr">
+        <is>
+          <t>378197606.33999974</t>
+        </is>
+      </c>
+      <c r="R115" s="2" t="inlineStr">
+        <is>
+          <t>1652563607.2899995</t>
+        </is>
+      </c>
+      <c r="S115" s="2" t="inlineStr">
+        <is>
+          <t>4583895619.739999</t>
+        </is>
+      </c>
+      <c r="T115" s="2" t="inlineStr">
+        <is>
+          <t>905</t>
+        </is>
+      </c>
+      <c r="U115" s="2" t="inlineStr">
+        <is>
+          <t>4336</t>
+        </is>
+      </c>
+      <c r="V115" s="2" t="inlineStr">
+        <is>
+          <t>19010</t>
+        </is>
+      </c>
+      <c r="W115" s="2" t="inlineStr">
+        <is>
+          <t>51918</t>
+        </is>
+      </c>
+      <c r="X115" s="2" t="inlineStr">
+        <is>
+          <t>1512844.4000000004</t>
+        </is>
+      </c>
+      <c r="Y115" s="2" t="inlineStr">
+        <is>
+          <t>108160950.24051975</t>
+        </is>
+      </c>
+      <c r="Z115" s="2" t="inlineStr">
+        <is>
+          <t>456112773.1282339</t>
+        </is>
+      </c>
+      <c r="AA115" s="2" t="inlineStr">
+        <is>
+          <t>1305627424.1429</t>
+        </is>
+      </c>
+      <c r="AB115" s="2" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="AC115" s="2" t="inlineStr">
+        <is>
+          <t>54726</t>
+        </is>
+      </c>
+      <c r="AD115" s="2" t="inlineStr">
+        <is>
+          <t>231419</t>
+        </is>
+      </c>
+      <c r="AE115" s="2" t="inlineStr">
+        <is>
+          <t>664340</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-13
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE115"/>
+  <dimension ref="A1:AE116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18527,6 +18527,163 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>27400559057.99096</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>1745603653.2397223</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>79749</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>1745138606.5315092</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>22035822453.16003</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>372606</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>4829</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>67181</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>335466</t>
+        </is>
+      </c>
+      <c r="K116" s="2" t="inlineStr">
+        <is>
+          <t>997341</t>
+        </is>
+      </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>2050.10666672456</t>
+        </is>
+      </c>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>62220.74200145294</t>
+        </is>
+      </c>
+      <c r="N116" s="2" t="inlineStr">
+        <is>
+          <t>336423.16367332527</t>
+        </is>
+      </c>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>890795.4816875228</t>
+        </is>
+      </c>
+      <c r="P116" s="2" t="inlineStr">
+        <is>
+          <t>80630593.23999998</t>
+        </is>
+      </c>
+      <c r="Q116" s="2" t="inlineStr">
+        <is>
+          <t>388052498.11999977</t>
+        </is>
+      </c>
+      <c r="R116" s="2" t="inlineStr">
+        <is>
+          <t>1731550842.9099996</t>
+        </is>
+      </c>
+      <c r="S116" s="2" t="inlineStr">
+        <is>
+          <t>4596136733.0199995</t>
+        </is>
+      </c>
+      <c r="T116" s="2" t="inlineStr">
+        <is>
+          <t>881</t>
+        </is>
+      </c>
+      <c r="U116" s="2" t="inlineStr">
+        <is>
+          <t>4439</t>
+        </is>
+      </c>
+      <c r="V116" s="2" t="inlineStr">
+        <is>
+          <t>19921</t>
+        </is>
+      </c>
+      <c r="W116" s="2" t="inlineStr">
+        <is>
+          <t>52114</t>
+        </is>
+      </c>
+      <c r="X116" s="2" t="inlineStr">
+        <is>
+          <t>703398.3900000002</t>
+        </is>
+      </c>
+      <c r="Y116" s="2" t="inlineStr">
+        <is>
+          <t>109421638.58000013</t>
+        </is>
+      </c>
+      <c r="Z116" s="2" t="inlineStr">
+        <is>
+          <t>456698319.968234</t>
+        </is>
+      </c>
+      <c r="AA116" s="2" t="inlineStr">
+        <is>
+          <t>1304338659.2729</t>
+        </is>
+      </c>
+      <c r="AB116" s="2" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="AC116" s="2" t="inlineStr">
+        <is>
+          <t>54746</t>
+        </is>
+      </c>
+      <c r="AD116" s="2" t="inlineStr">
+        <is>
+          <t>231813</t>
+        </is>
+      </c>
+      <c r="AE116" s="2" t="inlineStr">
+        <is>
+          <t>665059</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-14
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE116"/>
+  <dimension ref="A1:AE117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18684,6 +18684,163 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>27455633588.419067</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>1766023030.944822</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>79780</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>1765104257.726262</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>22065684265.110004</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>372967</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>4251</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>66491</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>336575</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t>1002951</t>
+        </is>
+      </c>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>1722.863333376619</t>
+        </is>
+      </c>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>59553.45833479192</t>
+        </is>
+      </c>
+      <c r="N117" s="2" t="inlineStr">
+        <is>
+          <t>329560.01267321425</t>
+        </is>
+      </c>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>876768.6736872755</t>
+        </is>
+      </c>
+      <c r="P117" s="2" t="inlineStr">
+        <is>
+          <t>57994891.59000002</t>
+        </is>
+      </c>
+      <c r="Q117" s="2" t="inlineStr">
+        <is>
+          <t>400232832.2899998</t>
+        </is>
+      </c>
+      <c r="R117" s="2" t="inlineStr">
+        <is>
+          <t>1694162724.9999995</t>
+        </is>
+      </c>
+      <c r="S117" s="2" t="inlineStr">
+        <is>
+          <t>4630133773.169999</t>
+        </is>
+      </c>
+      <c r="T117" s="2" t="inlineStr">
+        <is>
+          <t>676</t>
+        </is>
+      </c>
+      <c r="U117" s="2" t="inlineStr">
+        <is>
+          <t>4526</t>
+        </is>
+      </c>
+      <c r="V117" s="2" t="inlineStr">
+        <is>
+          <t>19429</t>
+        </is>
+      </c>
+      <c r="W117" s="2" t="inlineStr">
+        <is>
+          <t>52468</t>
+        </is>
+      </c>
+      <c r="X117" s="2" t="inlineStr">
+        <is>
+          <t>1475822.3</t>
+        </is>
+      </c>
+      <c r="Y117" s="2" t="inlineStr">
+        <is>
+          <t>117487553.36000016</t>
+        </is>
+      </c>
+      <c r="Z117" s="2" t="inlineStr">
+        <is>
+          <t>465340339.478234</t>
+        </is>
+      </c>
+      <c r="AA117" s="2" t="inlineStr">
+        <is>
+          <t>1311540956.5829</t>
+        </is>
+      </c>
+      <c r="AB117" s="2" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="AC117" s="2" t="inlineStr">
+        <is>
+          <t>53799</t>
+        </is>
+      </c>
+      <c r="AD117" s="2" t="inlineStr">
+        <is>
+          <t>232719</t>
+        </is>
+      </c>
+      <c r="AE117" s="2" t="inlineStr">
+        <is>
+          <t>664102</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-15
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE117"/>
+  <dimension ref="A1:AE118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18841,6 +18841,163 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>27529939605.318844</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>1781549134.4894207</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>79800</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>1781477830.5199046</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>22050242588.189995</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>372772</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>4002</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>76115</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>340598</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>1014246</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>1294.190333375625</t>
+        </is>
+      </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>57732.960001403844</t>
+        </is>
+      </c>
+      <c r="N118" s="2" t="inlineStr">
+        <is>
+          <t>329901.05300654384</t>
+        </is>
+      </c>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>882347.4600206402</t>
+        </is>
+      </c>
+      <c r="P118" s="2" t="inlineStr">
+        <is>
+          <t>64354715.76</t>
+        </is>
+      </c>
+      <c r="Q118" s="2" t="inlineStr">
+        <is>
+          <t>402278575.3099998</t>
+        </is>
+      </c>
+      <c r="R118" s="2" t="inlineStr">
+        <is>
+          <t>1689860320.2199996</t>
+        </is>
+      </c>
+      <c r="S118" s="2" t="inlineStr">
+        <is>
+          <t>4641618349.029999</t>
+        </is>
+      </c>
+      <c r="T118" s="2" t="inlineStr">
+        <is>
+          <t>714</t>
+        </is>
+      </c>
+      <c r="U118" s="2" t="inlineStr">
+        <is>
+          <t>4558</t>
+        </is>
+      </c>
+      <c r="V118" s="2" t="inlineStr">
+        <is>
+          <t>19399</t>
+        </is>
+      </c>
+      <c r="W118" s="2" t="inlineStr">
+        <is>
+          <t>52628</t>
+        </is>
+      </c>
+      <c r="X118" s="2" t="inlineStr">
+        <is>
+          <t>1337931.7199999988</t>
+        </is>
+      </c>
+      <c r="Y118" s="2" t="inlineStr">
+        <is>
+          <t>118613845.56000018</t>
+        </is>
+      </c>
+      <c r="Z118" s="2" t="inlineStr">
+        <is>
+          <t>468377640.248234</t>
+        </is>
+      </c>
+      <c r="AA118" s="2" t="inlineStr">
+        <is>
+          <t>1323138933.2529</t>
+        </is>
+      </c>
+      <c r="AB118" s="2" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="AC118" s="2" t="inlineStr">
+        <is>
+          <t>54497</t>
+        </is>
+      </c>
+      <c r="AD118" s="2" t="inlineStr">
+        <is>
+          <t>231722</t>
+        </is>
+      </c>
+      <c r="AE118" s="2" t="inlineStr">
+        <is>
+          <t>665669</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-16
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE118"/>
+  <dimension ref="A1:AE119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18998,6 +18998,163 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>27521750821.6832</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>1782174171.3840303</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>79828</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>1782162047.0668542</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>22110104698.67</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>373600</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>430</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>80714</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>336332</t>
+        </is>
+      </c>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t>1012405</t>
+        </is>
+      </c>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>146.860000004088</t>
+        </is>
+      </c>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>57940.50400143998</t>
+        </is>
+      </c>
+      <c r="N119" s="2" t="inlineStr">
+        <is>
+          <t>321443.9650064241</t>
+        </is>
+      </c>
+      <c r="O119" s="2" t="inlineStr">
+        <is>
+          <t>883837.3980206035</t>
+        </is>
+      </c>
+      <c r="P119" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q119" s="2" t="inlineStr">
+        <is>
+          <t>413460519.5799998</t>
+        </is>
+      </c>
+      <c r="R119" s="2" t="inlineStr">
+        <is>
+          <t>1679144478.1699996</t>
+        </is>
+      </c>
+      <c r="S119" s="2" t="inlineStr">
+        <is>
+          <t>4705894437.829999</t>
+        </is>
+      </c>
+      <c r="T119" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U119" s="2" t="inlineStr">
+        <is>
+          <t>4664</t>
+        </is>
+      </c>
+      <c r="V119" s="2" t="inlineStr">
+        <is>
+          <t>19227</t>
+        </is>
+      </c>
+      <c r="W119" s="2" t="inlineStr">
+        <is>
+          <t>53340</t>
+        </is>
+      </c>
+      <c r="X119" s="2" t="inlineStr">
+        <is>
+          <t>649671.82</t>
+        </is>
+      </c>
+      <c r="Y119" s="2" t="inlineStr">
+        <is>
+          <t>120549164.62000015</t>
+        </is>
+      </c>
+      <c r="Z119" s="2" t="inlineStr">
+        <is>
+          <t>466462561.4982339</t>
+        </is>
+      </c>
+      <c r="AA119" s="2" t="inlineStr">
+        <is>
+          <t>1327770092.5929</t>
+        </is>
+      </c>
+      <c r="AB119" s="2" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
+      <c r="AC119" s="2" t="inlineStr">
+        <is>
+          <t>55951</t>
+        </is>
+      </c>
+      <c r="AD119" s="2" t="inlineStr">
+        <is>
+          <t>232741</t>
+        </is>
+      </c>
+      <c r="AE119" s="2" t="inlineStr">
+        <is>
+          <t>667742</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-17
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE119"/>
+  <dimension ref="A1:AE120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19155,6 +19155,163 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>27518192545.12339</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>1783620230.0468268</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>79856</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>1783158413.6074579</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>22105552784.789993</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>373567</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>347</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>78062</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t>332487</t>
+        </is>
+      </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>1000202</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>204.365000002583</t>
+        </is>
+      </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>58004.86200145182</t>
+        </is>
+      </c>
+      <c r="N120" s="2" t="inlineStr">
+        <is>
+          <t>310108.42600624525</t>
+        </is>
+      </c>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t>876173.2870204183</t>
+        </is>
+      </c>
+      <c r="P120" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q120" s="2" t="inlineStr">
+        <is>
+          <t>413460519.5799998</t>
+        </is>
+      </c>
+      <c r="R120" s="2" t="inlineStr">
+        <is>
+          <t>1627991332.0099995</t>
+        </is>
+      </c>
+      <c r="S120" s="2" t="inlineStr">
+        <is>
+          <t>4705730154.999999</t>
+        </is>
+      </c>
+      <c r="T120" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U120" s="2" t="inlineStr">
+        <is>
+          <t>4664</t>
+        </is>
+      </c>
+      <c r="V120" s="2" t="inlineStr">
+        <is>
+          <t>18633</t>
+        </is>
+      </c>
+      <c r="W120" s="2" t="inlineStr">
+        <is>
+          <t>53339</t>
+        </is>
+      </c>
+      <c r="X120" s="2" t="inlineStr">
+        <is>
+          <t>474440.49000000005</t>
+        </is>
+      </c>
+      <c r="Y120" s="2" t="inlineStr">
+        <is>
+          <t>119349965.82000011</t>
+        </is>
+      </c>
+      <c r="Z120" s="2" t="inlineStr">
+        <is>
+          <t>460071271.4982339</t>
+        </is>
+      </c>
+      <c r="AA120" s="2" t="inlineStr">
+        <is>
+          <t>1323498099.9129</t>
+        </is>
+      </c>
+      <c r="AB120" s="2" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="AC120" s="2" t="inlineStr">
+        <is>
+          <t>56082</t>
+        </is>
+      </c>
+      <c r="AD120" s="2" t="inlineStr">
+        <is>
+          <t>230983</t>
+        </is>
+      </c>
+      <c r="AE120" s="2" t="inlineStr">
+        <is>
+          <t>668444</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-18
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE120"/>
+  <dimension ref="A1:AE121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19312,6 +19312,163 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>27694194167.588726</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>1803128955.5888886</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>79887</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>1802970093.5398614</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>22084342844.81001</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>373285</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>6542</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>68161</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t>336421</t>
+        </is>
+      </c>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t>994202</t>
+        </is>
+      </c>
+      <c r="L121" s="2" t="inlineStr">
+        <is>
+          <t>2614.565333422896</t>
+        </is>
+      </c>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>60711.05233483927</t>
+        </is>
+      </c>
+      <c r="N121" s="2" t="inlineStr">
+        <is>
+          <t>315623.20733956294</t>
+        </is>
+      </c>
+      <c r="O121" s="2" t="inlineStr">
+        <is>
+          <t>871727.7890201509</t>
+        </is>
+      </c>
+      <c r="P121" s="2" t="inlineStr">
+        <is>
+          <t>132897038.6199999</t>
+        </is>
+      </c>
+      <c r="Q121" s="2" t="inlineStr">
+        <is>
+          <t>412925118.7499998</t>
+        </is>
+      </c>
+      <c r="R121" s="2" t="inlineStr">
+        <is>
+          <t>1565791161.1199994</t>
+        </is>
+      </c>
+      <c r="S121" s="2" t="inlineStr">
+        <is>
+          <t>4590132892.139999</t>
+        </is>
+      </c>
+      <c r="T121" s="2" t="inlineStr">
+        <is>
+          <t>1547</t>
+        </is>
+      </c>
+      <c r="U121" s="2" t="inlineStr">
+        <is>
+          <t>4665</t>
+        </is>
+      </c>
+      <c r="V121" s="2" t="inlineStr">
+        <is>
+          <t>17859</t>
+        </is>
+      </c>
+      <c r="W121" s="2" t="inlineStr">
+        <is>
+          <t>52039</t>
+        </is>
+      </c>
+      <c r="X121" s="2" t="inlineStr">
+        <is>
+          <t>1818975.679999999</t>
+        </is>
+      </c>
+      <c r="Y121" s="2" t="inlineStr">
+        <is>
+          <t>116293634.64</t>
+        </is>
+      </c>
+      <c r="Z121" s="2" t="inlineStr">
+        <is>
+          <t>469648365.1682339</t>
+        </is>
+      </c>
+      <c r="AA121" s="2" t="inlineStr">
+        <is>
+          <t>1328133826.8429</t>
+        </is>
+      </c>
+      <c r="AB121" s="2" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="AC121" s="2" t="inlineStr">
+        <is>
+          <t>57244</t>
+        </is>
+      </c>
+      <c r="AD121" s="2" t="inlineStr">
+        <is>
+          <t>232260</t>
+        </is>
+      </c>
+      <c r="AE121" s="2" t="inlineStr">
+        <is>
+          <t>672047</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-19
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE121"/>
+  <dimension ref="A1:AE122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19469,6 +19469,163 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>28018499648.104656</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>1888473887.3698142</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>79923</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>1883675593.2959821</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>22201654808.730003</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>377479</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>4293</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>70025</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t>345160</t>
+        </is>
+      </c>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t>996369</t>
+        </is>
+      </c>
+      <c r="L122" s="2" t="inlineStr">
+        <is>
+          <t>2151.885333386216</t>
+        </is>
+      </c>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>61832.92433479355</t>
+        </is>
+      </c>
+      <c r="N122" s="2" t="inlineStr">
+        <is>
+          <t>327568.1380064411</t>
+        </is>
+      </c>
+      <c r="O122" s="2" t="inlineStr">
+        <is>
+          <t>874539.7383534472</t>
+        </is>
+      </c>
+      <c r="P122" s="2" t="inlineStr">
+        <is>
+          <t>70882877.64000003</t>
+        </is>
+      </c>
+      <c r="Q122" s="2" t="inlineStr">
+        <is>
+          <t>419362395.6100001</t>
+        </is>
+      </c>
+      <c r="R122" s="2" t="inlineStr">
+        <is>
+          <t>1701575900.2199996</t>
+        </is>
+      </c>
+      <c r="S122" s="2" t="inlineStr">
+        <is>
+          <t>4665749202.379999</t>
+        </is>
+      </c>
+      <c r="T122" s="2" t="inlineStr">
+        <is>
+          <t>789</t>
+        </is>
+      </c>
+      <c r="U122" s="2" t="inlineStr">
+        <is>
+          <t>4754</t>
+        </is>
+      </c>
+      <c r="V122" s="2" t="inlineStr">
+        <is>
+          <t>19418</t>
+        </is>
+      </c>
+      <c r="W122" s="2" t="inlineStr">
+        <is>
+          <t>52938</t>
+        </is>
+      </c>
+      <c r="X122" s="2" t="inlineStr">
+        <is>
+          <t>967149.1500000001</t>
+        </is>
+      </c>
+      <c r="Y122" s="2" t="inlineStr">
+        <is>
+          <t>117409346.35000001</t>
+        </is>
+      </c>
+      <c r="Z122" s="2" t="inlineStr">
+        <is>
+          <t>487798852.4482339</t>
+        </is>
+      </c>
+      <c r="AA122" s="2" t="inlineStr">
+        <is>
+          <t>1334972081.2880354</t>
+        </is>
+      </c>
+      <c r="AB122" s="2" t="inlineStr">
+        <is>
+          <t>177</t>
+        </is>
+      </c>
+      <c r="AC122" s="2" t="inlineStr">
+        <is>
+          <t>58452</t>
+        </is>
+      </c>
+      <c r="AD122" s="2" t="inlineStr">
+        <is>
+          <t>235383</t>
+        </is>
+      </c>
+      <c r="AE122" s="2" t="inlineStr">
+        <is>
+          <t>672723</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-20
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE122"/>
+  <dimension ref="A1:AE123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19626,6 +19626,163 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>28118278277.648766</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>1894554924.4309418</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>79965</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>1893996944.5625968</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>22254147121.039974</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>378291</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>4547</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>71880</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t>341835</t>
+        </is>
+      </c>
+      <c r="K123" s="2" t="inlineStr">
+        <is>
+          <t>999764</t>
+        </is>
+      </c>
+      <c r="L123" s="2" t="inlineStr">
+        <is>
+          <t>2032.08000005892</t>
+        </is>
+      </c>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>62706.148334818965</t>
+        </is>
+      </c>
+      <c r="N123" s="2" t="inlineStr">
+        <is>
+          <t>331268.89533995715</t>
+        </is>
+      </c>
+      <c r="O123" s="2" t="inlineStr">
+        <is>
+          <t>873064.6686867358</t>
+        </is>
+      </c>
+      <c r="P123" s="2" t="inlineStr">
+        <is>
+          <t>71523253.71</t>
+        </is>
+      </c>
+      <c r="Q123" s="2" t="inlineStr">
+        <is>
+          <t>411153286.4900001</t>
+        </is>
+      </c>
+      <c r="R123" s="2" t="inlineStr">
+        <is>
+          <t>1772245522.0099998</t>
+        </is>
+      </c>
+      <c r="S123" s="2" t="inlineStr">
+        <is>
+          <t>4672044576.139999</t>
+        </is>
+      </c>
+      <c r="T123" s="2" t="inlineStr">
+        <is>
+          <t>849</t>
+        </is>
+      </c>
+      <c r="U123" s="2" t="inlineStr">
+        <is>
+          <t>4633</t>
+        </is>
+      </c>
+      <c r="V123" s="2" t="inlineStr">
+        <is>
+          <t>20202</t>
+        </is>
+      </c>
+      <c r="W123" s="2" t="inlineStr">
+        <is>
+          <t>53005</t>
+        </is>
+      </c>
+      <c r="X123" s="2" t="inlineStr">
+        <is>
+          <t>1456691.9999999998</t>
+        </is>
+      </c>
+      <c r="Y123" s="2" t="inlineStr">
+        <is>
+          <t>122428031.84999998</t>
+        </is>
+      </c>
+      <c r="Z123" s="2" t="inlineStr">
+        <is>
+          <t>488924092.09823394</t>
+        </is>
+      </c>
+      <c r="AA123" s="2" t="inlineStr">
+        <is>
+          <t>1338259276.5580354</t>
+        </is>
+      </c>
+      <c r="AB123" s="2" t="inlineStr">
+        <is>
+          <t>241</t>
+        </is>
+      </c>
+      <c r="AC123" s="2" t="inlineStr">
+        <is>
+          <t>57286</t>
+        </is>
+      </c>
+      <c r="AD123" s="2" t="inlineStr">
+        <is>
+          <t>233696</t>
+        </is>
+      </c>
+      <c r="AE123" s="2" t="inlineStr">
+        <is>
+          <t>672475</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-21
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE123"/>
+  <dimension ref="A1:AE124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19783,6 +19783,163 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>28151265695.19977</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>1879727707.7858276</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>79989</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>1879287565.5410066</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>22312875621.569973</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>380078</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>3963</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>69196</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>339797</t>
+        </is>
+      </c>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>1006134</t>
+        </is>
+      </c>
+      <c r="L124" s="2" t="inlineStr">
+        <is>
+          <t>2126.632000051424</t>
+        </is>
+      </c>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>65111.26133486211</t>
+        </is>
+      </c>
+      <c r="N124" s="2" t="inlineStr">
+        <is>
+          <t>308348.9966731103</t>
+        </is>
+      </c>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t>872916.5200200398</t>
+        </is>
+      </c>
+      <c r="P124" s="2" t="inlineStr">
+        <is>
+          <t>52353836.839999996</t>
+        </is>
+      </c>
+      <c r="Q124" s="2" t="inlineStr">
+        <is>
+          <t>402761135.66000015</t>
+        </is>
+      </c>
+      <c r="R124" s="2" t="inlineStr">
+        <is>
+          <t>1723157530.7099998</t>
+        </is>
+      </c>
+      <c r="S124" s="2" t="inlineStr">
+        <is>
+          <t>4695230535.909999</t>
+        </is>
+      </c>
+      <c r="T124" s="2" t="inlineStr">
+        <is>
+          <t>641</t>
+        </is>
+      </c>
+      <c r="U124" s="2" t="inlineStr">
+        <is>
+          <t>4607</t>
+        </is>
+      </c>
+      <c r="V124" s="2" t="inlineStr">
+        <is>
+          <t>19615</t>
+        </is>
+      </c>
+      <c r="W124" s="2" t="inlineStr">
+        <is>
+          <t>53313</t>
+        </is>
+      </c>
+      <c r="X124" s="2" t="inlineStr">
+        <is>
+          <t>1569380.8599999999</t>
+        </is>
+      </c>
+      <c r="Y124" s="2" t="inlineStr">
+        <is>
+          <t>124172348.4769718</t>
+        </is>
+      </c>
+      <c r="Z124" s="2" t="inlineStr">
+        <is>
+          <t>491175292.0352057</t>
+        </is>
+      </c>
+      <c r="AA124" s="2" t="inlineStr">
+        <is>
+          <t>1346924538.7850072</t>
+        </is>
+      </c>
+      <c r="AB124" s="2" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="AC124" s="2" t="inlineStr">
+        <is>
+          <t>59257</t>
+        </is>
+      </c>
+      <c r="AD124" s="2" t="inlineStr">
+        <is>
+          <t>236701</t>
+        </is>
+      </c>
+      <c r="AE124" s="2" t="inlineStr">
+        <is>
+          <t>674511</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-22
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE124"/>
+  <dimension ref="A1:AE125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19940,6 +19940,163 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>28206915343.422436</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>1942884675.3368275</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>80009</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>1930916338.0215364</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>22352249710.54996</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>379908</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>4164</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>74824</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>340182</t>
+        </is>
+      </c>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t>1015791</t>
+        </is>
+      </c>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t>1358.751333383052</t>
+        </is>
+      </c>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>66890.8210015628</t>
+        </is>
+      </c>
+      <c r="N125" s="2" t="inlineStr">
+        <is>
+          <t>275674.5156729457</t>
+        </is>
+      </c>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t>879902.9393534588</t>
+        </is>
+      </c>
+      <c r="P125" s="2" t="inlineStr">
+        <is>
+          <t>52730051.15000002</t>
+        </is>
+      </c>
+      <c r="Q125" s="2" t="inlineStr">
+        <is>
+          <t>398692368.4700001</t>
+        </is>
+      </c>
+      <c r="R125" s="2" t="inlineStr">
+        <is>
+          <t>1713166512.4299996</t>
+        </is>
+      </c>
+      <c r="S125" s="2" t="inlineStr">
+        <is>
+          <t>4699756543.94</t>
+        </is>
+      </c>
+      <c r="T125" s="2" t="inlineStr">
+        <is>
+          <t>624</t>
+        </is>
+      </c>
+      <c r="U125" s="2" t="inlineStr">
+        <is>
+          <t>4581</t>
+        </is>
+      </c>
+      <c r="V125" s="2" t="inlineStr">
+        <is>
+          <t>19526</t>
+        </is>
+      </c>
+      <c r="W125" s="2" t="inlineStr">
+        <is>
+          <t>53436</t>
+        </is>
+      </c>
+      <c r="X125" s="2" t="inlineStr">
+        <is>
+          <t>522407.0299999999</t>
+        </is>
+      </c>
+      <c r="Y125" s="2" t="inlineStr">
+        <is>
+          <t>121999965.81697188</t>
+        </is>
+      </c>
+      <c r="Z125" s="2" t="inlineStr">
+        <is>
+          <t>495426272.55520576</t>
+        </is>
+      </c>
+      <c r="AA125" s="2" t="inlineStr">
+        <is>
+          <t>1356232175.6450074</t>
+        </is>
+      </c>
+      <c r="AB125" s="2" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="AC125" s="2" t="inlineStr">
+        <is>
+          <t>58712</t>
+        </is>
+      </c>
+      <c r="AD125" s="2" t="inlineStr">
+        <is>
+          <t>236409</t>
+        </is>
+      </c>
+      <c r="AE125" s="2" t="inlineStr">
+        <is>
+          <t>675349</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-23
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE125"/>
+  <dimension ref="A1:AE126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20097,6 +20097,163 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>28243648414.844666</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>1926925578.5626767</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>80028</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>1926804246.1322076</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>22402862862.799957</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>380671</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>79470</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>337459</t>
+        </is>
+      </c>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>1020064</t>
+        </is>
+      </c>
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t>155.65333333808</t>
+        </is>
+      </c>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>66824.02633489326</t>
+        </is>
+      </c>
+      <c r="N126" s="2" t="inlineStr">
+        <is>
+          <t>269088.10233951424</t>
+        </is>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>881708.0693535149</t>
+        </is>
+      </c>
+      <c r="P126" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q126" s="2" t="inlineStr">
+        <is>
+          <t>387073763.86000013</t>
+        </is>
+      </c>
+      <c r="R126" s="2" t="inlineStr">
+        <is>
+          <t>1699410001.1099997</t>
+        </is>
+      </c>
+      <c r="S126" s="2" t="inlineStr">
+        <is>
+          <t>4752487655.089999</t>
+        </is>
+      </c>
+      <c r="T126" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U126" s="2" t="inlineStr">
+        <is>
+          <t>4492</t>
+        </is>
+      </c>
+      <c r="V126" s="2" t="inlineStr">
+        <is>
+          <t>19412</t>
+        </is>
+      </c>
+      <c r="W126" s="2" t="inlineStr">
+        <is>
+          <t>54060</t>
+        </is>
+      </c>
+      <c r="X126" s="2" t="inlineStr">
+        <is>
+          <t>513826.31</t>
+        </is>
+      </c>
+      <c r="Y126" s="2" t="inlineStr">
+        <is>
+          <t>120177123.57697195</t>
+        </is>
+      </c>
+      <c r="Z126" s="2" t="inlineStr">
+        <is>
+          <t>479126020.5452057</t>
+        </is>
+      </c>
+      <c r="AA126" s="2" t="inlineStr">
+        <is>
+          <t>1358650539.1750073</t>
+        </is>
+      </c>
+      <c r="AB126" s="2" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="AC126" s="2" t="inlineStr">
+        <is>
+          <t>57744</t>
+        </is>
+      </c>
+      <c r="AD126" s="2" t="inlineStr">
+        <is>
+          <t>236263</t>
+        </is>
+      </c>
+      <c r="AE126" s="2" t="inlineStr">
+        <is>
+          <t>676930</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-24
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE126"/>
+  <dimension ref="A1:AE127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20254,6 +20254,163 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>28244295328.289387</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>1931026821.3852935</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>80046</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>1929885746.5768776</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>22398602148.68</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>380670</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>477</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>76129</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>333843</t>
+        </is>
+      </c>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t>1015502</t>
+        </is>
+      </c>
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t>273.480000004688</t>
+        </is>
+      </c>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>67413.54933490089</t>
+        </is>
+      </c>
+      <c r="N127" s="2" t="inlineStr">
+        <is>
+          <t>259807.26800601307</t>
+        </is>
+      </c>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>883048.7013535082</t>
+        </is>
+      </c>
+      <c r="P127" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q127" s="2" t="inlineStr">
+        <is>
+          <t>387073763.86000013</t>
+        </is>
+      </c>
+      <c r="R127" s="2" t="inlineStr">
+        <is>
+          <t>1643117809.8699996</t>
+        </is>
+      </c>
+      <c r="S127" s="2" t="inlineStr">
+        <is>
+          <t>4752487655.089999</t>
+        </is>
+      </c>
+      <c r="T127" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U127" s="2" t="inlineStr">
+        <is>
+          <t>4492</t>
+        </is>
+      </c>
+      <c r="V127" s="2" t="inlineStr">
+        <is>
+          <t>18786</t>
+        </is>
+      </c>
+      <c r="W127" s="2" t="inlineStr">
+        <is>
+          <t>54060</t>
+        </is>
+      </c>
+      <c r="X127" s="2" t="inlineStr">
+        <is>
+          <t>211111.10999999993</t>
+        </is>
+      </c>
+      <c r="Y127" s="2" t="inlineStr">
+        <is>
+          <t>120537971.15697193</t>
+        </is>
+      </c>
+      <c r="Z127" s="2" t="inlineStr">
+        <is>
+          <t>469245522.7524915</t>
+        </is>
+      </c>
+      <c r="AA127" s="2" t="inlineStr">
+        <is>
+          <t>1361405034.671674</t>
+        </is>
+      </c>
+      <c r="AB127" s="2" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="AC127" s="2" t="inlineStr">
+        <is>
+          <t>57931</t>
+        </is>
+      </c>
+      <c r="AD127" s="2" t="inlineStr">
+        <is>
+          <t>234942</t>
+        </is>
+      </c>
+      <c r="AE127" s="2" t="inlineStr">
+        <is>
+          <t>679057</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-25
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE127"/>
+  <dimension ref="A1:AE128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20411,6 +20411,163 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>28379486989.81663</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>1935822124.3066995</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>80069</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>1927101046.9235353</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>22375225314.60999</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>380318</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>6438</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>68770</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>339215</t>
+        </is>
+      </c>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>1011440</t>
+        </is>
+      </c>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>2305.152000086712</t>
+        </is>
+      </c>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>68068.1760016364</t>
+        </is>
+      </c>
+      <c r="N128" s="2" t="inlineStr">
+        <is>
+          <t>265229.5853394045</t>
+        </is>
+      </c>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>881163.3066868411</t>
+        </is>
+      </c>
+      <c r="P128" s="2" t="inlineStr">
+        <is>
+          <t>134605082.58</t>
+        </is>
+      </c>
+      <c r="Q128" s="2" t="inlineStr">
+        <is>
+          <t>387599435.41000015</t>
+        </is>
+      </c>
+      <c r="R128" s="2" t="inlineStr">
+        <is>
+          <t>1592826617.5399995</t>
+        </is>
+      </c>
+      <c r="S128" s="2" t="inlineStr">
+        <is>
+          <t>4754228596.299999</t>
+        </is>
+      </c>
+      <c r="T128" s="2" t="inlineStr">
+        <is>
+          <t>1523</t>
+        </is>
+      </c>
+      <c r="U128" s="2" t="inlineStr">
+        <is>
+          <t>4494</t>
+        </is>
+      </c>
+      <c r="V128" s="2" t="inlineStr">
+        <is>
+          <t>18207</t>
+        </is>
+      </c>
+      <c r="W128" s="2" t="inlineStr">
+        <is>
+          <t>54068</t>
+        </is>
+      </c>
+      <c r="X128" s="2" t="inlineStr">
+        <is>
+          <t>1403362.0700000008</t>
+        </is>
+      </c>
+      <c r="Y128" s="2" t="inlineStr">
+        <is>
+          <t>123910648.58697183</t>
+        </is>
+      </c>
+      <c r="Z128" s="2" t="inlineStr">
+        <is>
+          <t>483082005.68249136</t>
+        </is>
+      </c>
+      <c r="AA128" s="2" t="inlineStr">
+        <is>
+          <t>1370277154.981674</t>
+        </is>
+      </c>
+      <c r="AB128" s="2" t="inlineStr">
+        <is>
+          <t>217</t>
+        </is>
+      </c>
+      <c r="AC128" s="2" t="inlineStr">
+        <is>
+          <t>57528</t>
+        </is>
+      </c>
+      <c r="AD128" s="2" t="inlineStr">
+        <is>
+          <t>237389</t>
+        </is>
+      </c>
+      <c r="AE128" s="2" t="inlineStr">
+        <is>
+          <t>681178</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-26
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE128"/>
+  <dimension ref="A1:AE129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20568,6 +20568,163 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>28451872684.307148</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>1943318002.1309338</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>80104</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>1943204546.4300888</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>22492253000.969994</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>381919</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>4570</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>70656</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>348210</t>
+        </is>
+      </c>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t>1012058</t>
+        </is>
+      </c>
+      <c r="L129" s="2" t="inlineStr">
+        <is>
+          <t>1875.395666716656</t>
+        </is>
+      </c>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>68676.65066833071</t>
+        </is>
+      </c>
+      <c r="N129" s="2" t="inlineStr">
+        <is>
+          <t>277539.9616729762</t>
+        </is>
+      </c>
+      <c r="O129" s="2" t="inlineStr">
+        <is>
+          <t>882676.2406868582</t>
+        </is>
+      </c>
+      <c r="P129" s="2" t="inlineStr">
+        <is>
+          <t>80270795.33999996</t>
+        </is>
+      </c>
+      <c r="Q129" s="2" t="inlineStr">
+        <is>
+          <t>387998495.48999995</t>
+        </is>
+      </c>
+      <c r="R129" s="2" t="inlineStr">
+        <is>
+          <t>1729010416.7199996</t>
+        </is>
+      </c>
+      <c r="S129" s="2" t="inlineStr">
+        <is>
+          <t>4795773452.409999</t>
+        </is>
+      </c>
+      <c r="T129" s="2" t="inlineStr">
+        <is>
+          <t>871</t>
+        </is>
+      </c>
+      <c r="U129" s="2" t="inlineStr">
+        <is>
+          <t>4466</t>
+        </is>
+      </c>
+      <c r="V129" s="2" t="inlineStr">
+        <is>
+          <t>19738</t>
+        </is>
+      </c>
+      <c r="W129" s="2" t="inlineStr">
+        <is>
+          <t>54538</t>
+        </is>
+      </c>
+      <c r="X129" s="2" t="inlineStr">
+        <is>
+          <t>454803.37000000017</t>
+        </is>
+      </c>
+      <c r="Y129" s="2" t="inlineStr">
+        <is>
+          <t>121151028.26697184</t>
+        </is>
+      </c>
+      <c r="Z129" s="2" t="inlineStr">
+        <is>
+          <t>494899368.2924914</t>
+        </is>
+      </c>
+      <c r="AA129" s="2" t="inlineStr">
+        <is>
+          <t>1378837194.8116739</t>
+        </is>
+      </c>
+      <c r="AB129" s="2" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="AC129" s="2" t="inlineStr">
+        <is>
+          <t>55998</t>
+        </is>
+      </c>
+      <c r="AD129" s="2" t="inlineStr">
+        <is>
+          <t>237058</t>
+        </is>
+      </c>
+      <c r="AE129" s="2" t="inlineStr">
+        <is>
+          <t>680809</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-27
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE129"/>
+  <dimension ref="A1:AE130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20725,6 +20725,163 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>28561379428.94687</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>1983241489.6290922</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>80146</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>1968781032.5041795</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>22624740443.760017</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>383747</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>10437</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>70866</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>346924</t>
+        </is>
+      </c>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>1012457</t>
+        </is>
+      </c>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>3918.893333494296</t>
+        </is>
+      </c>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>66334.85066821607</t>
+        </is>
+      </c>
+      <c r="N130" s="2" t="inlineStr">
+        <is>
+          <t>274553.973673005</t>
+        </is>
+      </c>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t>879413.4020200368</t>
+        </is>
+      </c>
+      <c r="P130" s="2" t="inlineStr">
+        <is>
+          <t>71630893.67999993</t>
+        </is>
+      </c>
+      <c r="Q130" s="2" t="inlineStr">
+        <is>
+          <t>399131512.11999995</t>
+        </is>
+      </c>
+      <c r="R130" s="2" t="inlineStr">
+        <is>
+          <t>1810532581.1399996</t>
+        </is>
+      </c>
+      <c r="S130" s="2" t="inlineStr">
+        <is>
+          <t>4791155496.459999</t>
+        </is>
+      </c>
+      <c r="T130" s="2" t="inlineStr">
+        <is>
+          <t>808</t>
+        </is>
+      </c>
+      <c r="U130" s="2" t="inlineStr">
+        <is>
+          <t>4557</t>
+        </is>
+      </c>
+      <c r="V130" s="2" t="inlineStr">
+        <is>
+          <t>20613</t>
+        </is>
+      </c>
+      <c r="W130" s="2" t="inlineStr">
+        <is>
+          <t>54489</t>
+        </is>
+      </c>
+      <c r="X130" s="2" t="inlineStr">
+        <is>
+          <t>10595040.879999982</t>
+        </is>
+      </c>
+      <c r="Y130" s="2" t="inlineStr">
+        <is>
+          <t>125350757.79697186</t>
+        </is>
+      </c>
+      <c r="Z130" s="2" t="inlineStr">
+        <is>
+          <t>498811092.39249146</t>
+        </is>
+      </c>
+      <c r="AA130" s="2" t="inlineStr">
+        <is>
+          <t>1382923406.401674</t>
+        </is>
+      </c>
+      <c r="AB130" s="2" t="inlineStr">
+        <is>
+          <t>8428</t>
+        </is>
+      </c>
+      <c r="AC130" s="2" t="inlineStr">
+        <is>
+          <t>57783</t>
+        </is>
+      </c>
+      <c r="AD130" s="2" t="inlineStr">
+        <is>
+          <t>237403</t>
+        </is>
+      </c>
+      <c r="AE130" s="2" t="inlineStr">
+        <is>
+          <t>680637</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-28
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE130"/>
+  <dimension ref="A1:AE131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20882,6 +20882,163 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>28578855190.841763</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>1952371508.1279473</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>80171</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>1951114578.410106</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>22662964318.81002</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>384335</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>10237</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>71678</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>348224</t>
+        </is>
+      </c>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t>1019015</t>
+        </is>
+      </c>
+      <c r="L131" s="2" t="inlineStr">
+        <is>
+          <t>3541.153000149128</t>
+        </is>
+      </c>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>66859.54666823079</t>
+        </is>
+      </c>
+      <c r="N131" s="2" t="inlineStr">
+        <is>
+          <t>272340.8106729543</t>
+        </is>
+      </c>
+      <c r="O131" s="2" t="inlineStr">
+        <is>
+          <t>878193.0800200227</t>
+        </is>
+      </c>
+      <c r="P131" s="2" t="inlineStr">
+        <is>
+          <t>58571770.70000006</t>
+        </is>
+      </c>
+      <c r="Q131" s="2" t="inlineStr">
+        <is>
+          <t>398520048.3399999</t>
+        </is>
+      </c>
+      <c r="R131" s="2" t="inlineStr">
+        <is>
+          <t>1750704570.8599997</t>
+        </is>
+      </c>
+      <c r="S131" s="2" t="inlineStr">
+        <is>
+          <t>4801312378.509999</t>
+        </is>
+      </c>
+      <c r="T131" s="2" t="inlineStr">
+        <is>
+          <t>677</t>
+        </is>
+      </c>
+      <c r="U131" s="2" t="inlineStr">
+        <is>
+          <t>4512</t>
+        </is>
+      </c>
+      <c r="V131" s="2" t="inlineStr">
+        <is>
+          <t>19901</t>
+        </is>
+      </c>
+      <c r="W131" s="2" t="inlineStr">
+        <is>
+          <t>54658</t>
+        </is>
+      </c>
+      <c r="X131" s="2" t="inlineStr">
+        <is>
+          <t>10552573.728032336</t>
+        </is>
+      </c>
+      <c r="Y131" s="2" t="inlineStr">
+        <is>
+          <t>124959019.55999994</t>
+        </is>
+      </c>
+      <c r="Z131" s="2" t="inlineStr">
+        <is>
+          <t>504813168.27249146</t>
+        </is>
+      </c>
+      <c r="AA131" s="2" t="inlineStr">
+        <is>
+          <t>1388498895.661674</t>
+        </is>
+      </c>
+      <c r="AB131" s="2" t="inlineStr">
+        <is>
+          <t>8777</t>
+        </is>
+      </c>
+      <c r="AC131" s="2" t="inlineStr">
+        <is>
+          <t>57568</t>
+        </is>
+      </c>
+      <c r="AD131" s="2" t="inlineStr">
+        <is>
+          <t>238943</t>
+        </is>
+      </c>
+      <c r="AE131" s="2" t="inlineStr">
+        <is>
+          <t>683470</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-29
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE131"/>
+  <dimension ref="A1:AE132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21039,6 +21039,163 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>28659459404.583614</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>1950131690.5858347</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>80186</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>1950115716.7545228</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>22713358216.930016</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>385092</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>7634</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>76517</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>347097</t>
+        </is>
+      </c>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>1028038</t>
+        </is>
+      </c>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t>1678.048000143432</t>
+        </is>
+      </c>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>66366.55733488647</t>
+        </is>
+      </c>
+      <c r="N132" s="2" t="inlineStr">
+        <is>
+          <t>274107.67133967875</t>
+        </is>
+      </c>
+      <c r="O132" s="2" t="inlineStr">
+        <is>
+          <t>884506.0333534423</t>
+        </is>
+      </c>
+      <c r="P132" s="2" t="inlineStr">
+        <is>
+          <t>64285546.23000001</t>
+        </is>
+      </c>
+      <c r="Q132" s="2" t="inlineStr">
+        <is>
+          <t>403016405.20000005</t>
+        </is>
+      </c>
+      <c r="R132" s="2" t="inlineStr">
+        <is>
+          <t>1733013393.5299997</t>
+        </is>
+      </c>
+      <c r="S132" s="2" t="inlineStr">
+        <is>
+          <t>4807011496.969999</t>
+        </is>
+      </c>
+      <c r="T132" s="2" t="inlineStr">
+        <is>
+          <t>729</t>
+        </is>
+      </c>
+      <c r="U132" s="2" t="inlineStr">
+        <is>
+          <t>4537</t>
+        </is>
+      </c>
+      <c r="V132" s="2" t="inlineStr">
+        <is>
+          <t>19764</t>
+        </is>
+      </c>
+      <c r="W132" s="2" t="inlineStr">
+        <is>
+          <t>54752</t>
+        </is>
+      </c>
+      <c r="X132" s="2" t="inlineStr">
+        <is>
+          <t>6053511.249999988</t>
+        </is>
+      </c>
+      <c r="Y132" s="2" t="inlineStr">
+        <is>
+          <t>126663808.14803214</t>
+        </is>
+      </c>
+      <c r="Z132" s="2" t="inlineStr">
+        <is>
+          <t>508413865.12052375</t>
+        </is>
+      </c>
+      <c r="AA132" s="2" t="inlineStr">
+        <is>
+          <t>1400615866.5897062</t>
+        </is>
+      </c>
+      <c r="AB132" s="2" t="inlineStr">
+        <is>
+          <t>6674</t>
+        </is>
+      </c>
+      <c r="AC132" s="2" t="inlineStr">
+        <is>
+          <t>59264</t>
+        </is>
+      </c>
+      <c r="AD132" s="2" t="inlineStr">
+        <is>
+          <t>241571</t>
+        </is>
+      </c>
+      <c r="AE132" s="2" t="inlineStr">
+        <is>
+          <t>686773</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-30
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE132"/>
+  <dimension ref="A1:AE133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21196,6 +21196,163 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>28631143852.269848</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>1947512751.4246702</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>80200</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>1947474517.9940183</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>22708919218.38997</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>385073</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>3373</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>80747</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>341947</t>
+        </is>
+      </c>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>1029166</t>
+        </is>
+      </c>
+      <c r="L133" s="2" t="inlineStr">
+        <is>
+          <t>261.487333382933</t>
+        </is>
+      </c>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>65965.82800153932</t>
+        </is>
+      </c>
+      <c r="N133" s="2" t="inlineStr">
+        <is>
+          <t>265775.7553395638</t>
+        </is>
+      </c>
+      <c r="O133" s="2" t="inlineStr">
+        <is>
+          <t>885578.1926868123</t>
+        </is>
+      </c>
+      <c r="P133" s="2" t="inlineStr">
+        <is>
+          <t>162801.95</t>
+        </is>
+      </c>
+      <c r="Q133" s="2" t="inlineStr">
+        <is>
+          <t>414565840.28</t>
+        </is>
+      </c>
+      <c r="R133" s="2" t="inlineStr">
+        <is>
+          <t>1717267221.2299998</t>
+        </is>
+      </c>
+      <c r="S133" s="2" t="inlineStr">
+        <is>
+          <t>4871285798.009999</t>
+        </is>
+      </c>
+      <c r="T133" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U133" s="2" t="inlineStr">
+        <is>
+          <t>4641</t>
+        </is>
+      </c>
+      <c r="V133" s="2" t="inlineStr">
+        <is>
+          <t>19569</t>
+        </is>
+      </c>
+      <c r="W133" s="2" t="inlineStr">
+        <is>
+          <t>55480</t>
+        </is>
+      </c>
+      <c r="X133" s="2" t="inlineStr">
+        <is>
+          <t>570548.1499999999</t>
+        </is>
+      </c>
+      <c r="Y133" s="2" t="inlineStr">
+        <is>
+          <t>125875384.27803208</t>
+        </is>
+      </c>
+      <c r="Z133" s="2" t="inlineStr">
+        <is>
+          <t>493214494.4055237</t>
+        </is>
+      </c>
+      <c r="AA133" s="2" t="inlineStr">
+        <is>
+          <t>1406844114.9997063</t>
+        </is>
+      </c>
+      <c r="AB133" s="2" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="AC133" s="2" t="inlineStr">
+        <is>
+          <t>58304</t>
+        </is>
+      </c>
+      <c r="AD133" s="2" t="inlineStr">
+        <is>
+          <t>241119</t>
+        </is>
+      </c>
+      <c r="AE133" s="2" t="inlineStr">
+        <is>
+          <t>692795</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-08-31
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE133"/>
+  <dimension ref="A1:AE134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21353,6 +21353,163 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>28632336243.50329</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>1952067835.4410255</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>80217</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>1951853457.9628384</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>22704226982.83004</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>384995</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>4184</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>75938</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>338469</t>
+        </is>
+      </c>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>1016466</t>
+        </is>
+      </c>
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t>331.639000060634</t>
+        </is>
+      </c>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>65238.41433485468</t>
+        </is>
+      </c>
+      <c r="N134" s="2" t="inlineStr">
+        <is>
+          <t>257408.66233941156</t>
+        </is>
+      </c>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t>879121.5936867553</t>
+        </is>
+      </c>
+      <c r="P134" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q134" s="2" t="inlineStr">
+        <is>
+          <t>414735678.23</t>
+        </is>
+      </c>
+      <c r="R134" s="2" t="inlineStr">
+        <is>
+          <t>1656134347.3099997</t>
+        </is>
+      </c>
+      <c r="S134" s="2" t="inlineStr">
+        <is>
+          <t>4871429233.779999</t>
+        </is>
+      </c>
+      <c r="T134" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U134" s="2" t="inlineStr">
+        <is>
+          <t>4644</t>
+        </is>
+      </c>
+      <c r="V134" s="2" t="inlineStr">
+        <is>
+          <t>18867</t>
+        </is>
+      </c>
+      <c r="W134" s="2" t="inlineStr">
+        <is>
+          <t>55481</t>
+        </is>
+      </c>
+      <c r="X134" s="2" t="inlineStr">
+        <is>
+          <t>1844172.086517824</t>
+        </is>
+      </c>
+      <c r="Y134" s="2" t="inlineStr">
+        <is>
+          <t>125583100.56303209</t>
+        </is>
+      </c>
+      <c r="Z134" s="2" t="inlineStr">
+        <is>
+          <t>484540136.5505237</t>
+        </is>
+      </c>
+      <c r="AA134" s="2" t="inlineStr">
+        <is>
+          <t>1392122350.4547062</t>
+        </is>
+      </c>
+      <c r="AB134" s="2" t="inlineStr">
+        <is>
+          <t>1765</t>
+        </is>
+      </c>
+      <c r="AC134" s="2" t="inlineStr">
+        <is>
+          <t>57619</t>
+        </is>
+      </c>
+      <c r="AD134" s="2" t="inlineStr">
+        <is>
+          <t>244749</t>
+        </is>
+      </c>
+      <c r="AE134" s="2" t="inlineStr">
+        <is>
+          <t>691164</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-01
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE134"/>
+  <dimension ref="A1:AE135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21510,6 +21510,163 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 502</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="L135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="N135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="O135" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="P135" s="2" t="inlineStr">
+        <is>
+          <t>123624318.03999977</t>
+        </is>
+      </c>
+      <c r="Q135" s="2" t="inlineStr">
+        <is>
+          <t>415508303.77</t>
+        </is>
+      </c>
+      <c r="R135" s="2" t="inlineStr">
+        <is>
+          <t>1598856552.4399998</t>
+        </is>
+      </c>
+      <c r="S135" s="2" t="inlineStr">
+        <is>
+          <t>4740073917.289999</t>
+        </is>
+      </c>
+      <c r="T135" s="2" t="inlineStr">
+        <is>
+          <t>1459</t>
+        </is>
+      </c>
+      <c r="U135" s="2" t="inlineStr">
+        <is>
+          <t>4648</t>
+        </is>
+      </c>
+      <c r="V135" s="2" t="inlineStr">
+        <is>
+          <t>18184</t>
+        </is>
+      </c>
+      <c r="W135" s="2" t="inlineStr">
+        <is>
+          <t>54093</t>
+        </is>
+      </c>
+      <c r="X135" s="2" t="inlineStr">
+        <is>
+          <t>1167679.5799999994</t>
+        </is>
+      </c>
+      <c r="Y135" s="2" t="inlineStr">
+        <is>
+          <t>120837795.37955008</t>
+        </is>
+      </c>
+      <c r="Z135" s="2" t="inlineStr">
+        <is>
+          <t>491633246.1870416</t>
+        </is>
+      </c>
+      <c r="AA135" s="2" t="inlineStr">
+        <is>
+          <t>1387523752.781224</t>
+        </is>
+      </c>
+      <c r="AB135" s="2" t="inlineStr">
+        <is>
+          <t>335</t>
+        </is>
+      </c>
+      <c r="AC135" s="2" t="inlineStr">
+        <is>
+          <t>52152</t>
+        </is>
+      </c>
+      <c r="AD135" s="2" t="inlineStr">
+        <is>
+          <t>238033</t>
+        </is>
+      </c>
+      <c r="AE135" s="2" t="inlineStr">
+        <is>
+          <t>686333</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-02
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE135"/>
+  <dimension ref="A1:AE136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21667,6 +21667,163 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>28856241055.147907</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>1958008277.8660278</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>80257</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>1957807150.2174628</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>22635385686.67</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>377493</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>8848</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>68774</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>349788</t>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>1015242</t>
+        </is>
+      </c>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>2689.272000162056</t>
+        </is>
+      </c>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>64087.0063347852</t>
+        </is>
+      </c>
+      <c r="N136" s="2" t="inlineStr">
+        <is>
+          <t>275727.5880063477</t>
+        </is>
+      </c>
+      <c r="O136" s="2" t="inlineStr">
+        <is>
+          <t>878723.2886866329</t>
+        </is>
+      </c>
+      <c r="P136" s="2" t="inlineStr">
+        <is>
+          <t>76925836.67999996</t>
+        </is>
+      </c>
+      <c r="Q136" s="2" t="inlineStr">
+        <is>
+          <t>403447606.88</t>
+        </is>
+      </c>
+      <c r="R136" s="2" t="inlineStr">
+        <is>
+          <t>1722868440.5399997</t>
+        </is>
+      </c>
+      <c r="S136" s="2" t="inlineStr">
+        <is>
+          <t>4811098754.0199995</t>
+        </is>
+      </c>
+      <c r="T136" s="2" t="inlineStr">
+        <is>
+          <t>852</t>
+        </is>
+      </c>
+      <c r="U136" s="2" t="inlineStr">
+        <is>
+          <t>4584</t>
+        </is>
+      </c>
+      <c r="V136" s="2" t="inlineStr">
+        <is>
+          <t>19648</t>
+        </is>
+      </c>
+      <c r="W136" s="2" t="inlineStr">
+        <is>
+          <t>54957</t>
+        </is>
+      </c>
+      <c r="X136" s="2" t="inlineStr">
+        <is>
+          <t>1394434.55</t>
+        </is>
+      </c>
+      <c r="Y136" s="2" t="inlineStr">
+        <is>
+          <t>132717707.49955024</t>
+        </is>
+      </c>
+      <c r="Z136" s="2" t="inlineStr">
+        <is>
+          <t>515372967.9670418</t>
+        </is>
+      </c>
+      <c r="AA136" s="2" t="inlineStr">
+        <is>
+          <t>1404368310.9112241</t>
+        </is>
+      </c>
+      <c r="AB136" s="2" t="inlineStr">
+        <is>
+          <t>303</t>
+        </is>
+      </c>
+      <c r="AC136" s="2" t="inlineStr">
+        <is>
+          <t>56088</t>
+        </is>
+      </c>
+      <c r="AD136" s="2" t="inlineStr">
+        <is>
+          <t>240651</t>
+        </is>
+      </c>
+      <c r="AE136" s="2" t="inlineStr">
+        <is>
+          <t>689894</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-03
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE136"/>
+  <dimension ref="A1:AE137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21824,6 +21824,163 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>28958738252.43062</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>1975358792.5852442</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>80275</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>1974482673.958245</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>22713044432.38</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>378649</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>8986</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>68851</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>349196</t>
+        </is>
+      </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>1015945</t>
+        </is>
+      </c>
+      <c r="L137" s="2" t="inlineStr">
+        <is>
+          <t>2848.37600012704</t>
+        </is>
+      </c>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>64634.6420014752</t>
+        </is>
+      </c>
+      <c r="N137" s="2" t="inlineStr">
+        <is>
+          <t>276996.9943397726</t>
+        </is>
+      </c>
+      <c r="O137" s="2" t="inlineStr">
+        <is>
+          <t>878690.6993532957</t>
+        </is>
+      </c>
+      <c r="P137" s="2" t="inlineStr">
+        <is>
+          <t>84116742.72999999</t>
+        </is>
+      </c>
+      <c r="Q137" s="2" t="inlineStr">
+        <is>
+          <t>399259701.03999996</t>
+        </is>
+      </c>
+      <c r="R137" s="2" t="inlineStr">
+        <is>
+          <t>1798841799.0299997</t>
+        </is>
+      </c>
+      <c r="S137" s="2" t="inlineStr">
+        <is>
+          <t>4821076074.86</t>
+        </is>
+      </c>
+      <c r="T137" s="2" t="inlineStr">
+        <is>
+          <t>945</t>
+        </is>
+      </c>
+      <c r="U137" s="2" t="inlineStr">
+        <is>
+          <t>4564</t>
+        </is>
+      </c>
+      <c r="V137" s="2" t="inlineStr">
+        <is>
+          <t>20503</t>
+        </is>
+      </c>
+      <c r="W137" s="2" t="inlineStr">
+        <is>
+          <t>55064</t>
+        </is>
+      </c>
+      <c r="X137" s="2" t="inlineStr">
+        <is>
+          <t>1625740.79</t>
+        </is>
+      </c>
+      <c r="Y137" s="2" t="inlineStr">
+        <is>
+          <t>127612165.87955022</t>
+        </is>
+      </c>
+      <c r="Z137" s="2" t="inlineStr">
+        <is>
+          <t>510684090.0870418</t>
+        </is>
+      </c>
+      <c r="AA137" s="2" t="inlineStr">
+        <is>
+          <t>1399983529.147381</t>
+        </is>
+      </c>
+      <c r="AB137" s="2" t="inlineStr">
+        <is>
+          <t>285</t>
+        </is>
+      </c>
+      <c r="AC137" s="2" t="inlineStr">
+        <is>
+          <t>56979</t>
+        </is>
+      </c>
+      <c r="AD137" s="2" t="inlineStr">
+        <is>
+          <t>241523</t>
+        </is>
+      </c>
+      <c r="AE137" s="2" t="inlineStr">
+        <is>
+          <t>691720</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-04
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE137"/>
+  <dimension ref="A1:AE138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21981,6 +21981,163 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>29014285520.18626</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>1983481858.841594</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>80300</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>1983116193.349902</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>22769228369.98999</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>379356</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>7538</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>70187</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>351177</t>
+        </is>
+      </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>1022760</t>
+        </is>
+      </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>2199.535333440641</t>
+        </is>
+      </c>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>63256.61400144208</t>
+        </is>
+      </c>
+      <c r="N138" s="2" t="inlineStr">
+        <is>
+          <t>278579.8163397839</t>
+        </is>
+      </c>
+      <c r="O138" s="2" t="inlineStr">
+        <is>
+          <t>878498.1693532772</t>
+        </is>
+      </c>
+      <c r="P138" s="2" t="inlineStr">
+        <is>
+          <t>51150691.53999998</t>
+        </is>
+      </c>
+      <c r="Q138" s="2" t="inlineStr">
+        <is>
+          <t>415490853.76000005</t>
+        </is>
+      </c>
+      <c r="R138" s="2" t="inlineStr">
+        <is>
+          <t>1754768860.1499999</t>
+        </is>
+      </c>
+      <c r="S138" s="2" t="inlineStr">
+        <is>
+          <t>4854618463.53</t>
+        </is>
+      </c>
+      <c r="T138" s="2" t="inlineStr">
+        <is>
+          <t>617</t>
+        </is>
+      </c>
+      <c r="U138" s="2" t="inlineStr">
+        <is>
+          <t>4704</t>
+        </is>
+      </c>
+      <c r="V138" s="2" t="inlineStr">
+        <is>
+          <t>19954</t>
+        </is>
+      </c>
+      <c r="W138" s="2" t="inlineStr">
+        <is>
+          <t>55399</t>
+        </is>
+      </c>
+      <c r="X138" s="2" t="inlineStr">
+        <is>
+          <t>1776702.0199999993</t>
+        </is>
+      </c>
+      <c r="Y138" s="2" t="inlineStr">
+        <is>
+          <t>119831424.02030782</t>
+        </is>
+      </c>
+      <c r="Z138" s="2" t="inlineStr">
+        <is>
+          <t>513356329.91779935</t>
+        </is>
+      </c>
+      <c r="AA138" s="2" t="inlineStr">
+        <is>
+          <t>1396814422.0481384</t>
+        </is>
+      </c>
+      <c r="AB138" s="2" t="inlineStr">
+        <is>
+          <t>305</t>
+        </is>
+      </c>
+      <c r="AC138" s="2" t="inlineStr">
+        <is>
+          <t>56787</t>
+        </is>
+      </c>
+      <c r="AD138" s="2" t="inlineStr">
+        <is>
+          <t>243587</t>
+        </is>
+      </c>
+      <c r="AE138" s="2" t="inlineStr">
+        <is>
+          <t>693101</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-05
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE138"/>
+  <dimension ref="A1:AE139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22138,6 +22138,163 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>29118151226.486637</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>1985404588.1349747</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>80323</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>1985388189.7348597</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>22833824104.34999</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>375627</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>7211</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>74794</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>352113</t>
+        </is>
+      </c>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>1031404</t>
+        </is>
+      </c>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>2227.533333433864</t>
+        </is>
+      </c>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>65097.09400144544</t>
+        </is>
+      </c>
+      <c r="N139" s="2" t="inlineStr">
+        <is>
+          <t>280126.0696731403</t>
+        </is>
+      </c>
+      <c r="O139" s="2" t="inlineStr">
+        <is>
+          <t>887145.7410200345</t>
+        </is>
+      </c>
+      <c r="P139" s="2" t="inlineStr">
+        <is>
+          <t>60860932.63000004</t>
+        </is>
+      </c>
+      <c r="Q139" s="2" t="inlineStr">
+        <is>
+          <t>408392645.6100001</t>
+        </is>
+      </c>
+      <c r="R139" s="2" t="inlineStr">
+        <is>
+          <t>1737039220.27</t>
+        </is>
+      </c>
+      <c r="S139" s="2" t="inlineStr">
+        <is>
+          <t>4851717894.849999</t>
+        </is>
+      </c>
+      <c r="T139" s="2" t="inlineStr">
+        <is>
+          <t>695</t>
+        </is>
+      </c>
+      <c r="U139" s="2" t="inlineStr">
+        <is>
+          <t>4651</t>
+        </is>
+      </c>
+      <c r="V139" s="2" t="inlineStr">
+        <is>
+          <t>19770</t>
+        </is>
+      </c>
+      <c r="W139" s="2" t="inlineStr">
+        <is>
+          <t>55446</t>
+        </is>
+      </c>
+      <c r="X139" s="2" t="inlineStr">
+        <is>
+          <t>853485.6800000004</t>
+        </is>
+      </c>
+      <c r="Y139" s="2" t="inlineStr">
+        <is>
+          <t>115830173.34227556</t>
+        </is>
+      </c>
+      <c r="Z139" s="2" t="inlineStr">
+        <is>
+          <t>516728201.45727974</t>
+        </is>
+      </c>
+      <c r="AA139" s="2" t="inlineStr">
+        <is>
+          <t>1403847056.9881384</t>
+        </is>
+      </c>
+      <c r="AB139" s="2" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="AC139" s="2" t="inlineStr">
+        <is>
+          <t>55698</t>
+        </is>
+      </c>
+      <c r="AD139" s="2" t="inlineStr">
+        <is>
+          <t>244768</t>
+        </is>
+      </c>
+      <c r="AE139" s="2" t="inlineStr">
+        <is>
+          <t>694844</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>